<commit_message>
exporte les indicateurs de C4 dans le fichier excel
</commit_message>
<xml_diff>
--- a/impact/vsme/xlsx/VSME.xlsx
+++ b/impact/vsme/xlsx/VSME.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmonteiro-de-mac-adc\Desktop\ancien bureau\Fichier\CSRD\Tableau ESRS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6C9B35E-26DD-41A5-AB02-16B6713B0860}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19C032B9-A9CA-4337-A9EE-CC37BC8FCA4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="15375" windowHeight="7785" tabRatio="500" firstSheet="6" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" firstSheet="1" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="&gt;&gt;&gt; " sheetId="3" r:id="rId1"/>
@@ -22,15 +22,16 @@
     <sheet name="B5" sheetId="17" r:id="rId7"/>
     <sheet name="B6" sheetId="9" r:id="rId8"/>
     <sheet name="B7" sheetId="10" r:id="rId9"/>
-    <sheet name="B8" sheetId="15" r:id="rId10"/>
-    <sheet name="B9" sheetId="11" r:id="rId11"/>
-    <sheet name="B10" sheetId="16" r:id="rId12"/>
-    <sheet name="C5" sheetId="23" r:id="rId13"/>
-    <sheet name="C6" sheetId="21" r:id="rId14"/>
-    <sheet name="C7" sheetId="24" r:id="rId15"/>
-    <sheet name="B11" sheetId="14" r:id="rId16"/>
-    <sheet name="C8" sheetId="22" r:id="rId17"/>
-    <sheet name="C9" sheetId="20" r:id="rId18"/>
+    <sheet name="C4" sheetId="25" r:id="rId10"/>
+    <sheet name="B8" sheetId="15" r:id="rId11"/>
+    <sheet name="B9" sheetId="11" r:id="rId12"/>
+    <sheet name="B10" sheetId="16" r:id="rId13"/>
+    <sheet name="C5" sheetId="23" r:id="rId14"/>
+    <sheet name="C6" sheetId="21" r:id="rId15"/>
+    <sheet name="C7" sheetId="24" r:id="rId16"/>
+    <sheet name="B11" sheetId="14" r:id="rId17"/>
+    <sheet name="C8" sheetId="22" r:id="rId18"/>
+    <sheet name="C9" sheetId="20" r:id="rId19"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -51,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="193">
   <si>
     <t/>
   </si>
@@ -597,6 +598,39 @@
   </si>
   <si>
     <t>C7 - Incidents graves en matière de droits de l’homme</t>
+  </si>
+  <si>
+    <t>Aléas et risques climatiques recensés</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Méthode d'évaluation </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Horizon temporel </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Actions d’adaptation entreprises </t>
+  </si>
+  <si>
+    <t>Impacts financiers potentiels des risques climatiques</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ce risque a-t-il des impacts financiers potentiels ? </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Description des impacts financiers potentiels</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Niveau de risque </t>
+  </si>
+  <si>
+    <t>C4 - Risques climatiques</t>
+  </si>
+  <si>
+    <t>N° du risque</t>
   </si>
 </sst>
 </file>
@@ -1779,6 +1813,114 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AD57197-9ADC-43C0-B70E-801EE1BD86F4}">
+  <sheetPr>
+    <tabColor rgb="FFB8FEC9"/>
+  </sheetPr>
+  <dimension ref="A1:P3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7109375" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="3" width="15.7109375" style="1"/>
+    <col min="4" max="5" width="15.7109375" style="2"/>
+    <col min="6" max="6" width="15.7109375" style="14"/>
+    <col min="7" max="8" width="15.7109375" style="2"/>
+    <col min="9" max="9" width="15.7109375" style="12"/>
+    <col min="10" max="16384" width="15.7109375" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" s="20" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="72" t="s">
+        <v>191</v>
+      </c>
+      <c r="B1" s="72"/>
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
+      <c r="E1" s="72"/>
+      <c r="F1" s="72"/>
+      <c r="G1" s="72"/>
+      <c r="H1" s="72"/>
+      <c r="I1" s="72"/>
+      <c r="J1" s="72"/>
+      <c r="K1" s="72"/>
+      <c r="L1" s="72"/>
+      <c r="M1" s="72"/>
+      <c r="N1" s="72"/>
+      <c r="O1" s="72"/>
+      <c r="P1" s="72"/>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A2" s="48" t="s">
+        <v>182</v>
+      </c>
+      <c r="B2" s="49"/>
+      <c r="C2" s="49"/>
+      <c r="D2" s="49"/>
+      <c r="E2" s="50"/>
+      <c r="F2" s="48" t="s">
+        <v>187</v>
+      </c>
+      <c r="G2" s="49"/>
+      <c r="H2" s="49"/>
+      <c r="I2" s="50"/>
+    </row>
+    <row r="3" spans="1:16" ht="38.25" x14ac:dyDescent="0.35">
+      <c r="A3" s="15" t="s">
+        <v>192</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>183</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>184</v>
+      </c>
+      <c r="D3" s="15" t="s">
+        <v>185</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>186</v>
+      </c>
+      <c r="F3" s="17" t="s">
+        <v>188</v>
+      </c>
+      <c r="G3" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="H3" s="15" t="s">
+        <v>190</v>
+      </c>
+      <c r="I3" s="16" t="s">
+        <v>185</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="F2:I2"/>
+  </mergeCells>
+  <dataValidations count="5">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A4:B227" xr:uid="{60BE6B91-29AF-41C7-B3A4-C4179A88EB71}">
+      <formula1>"mètres carrés (m²),hectares (ha)"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4:E1048576" xr:uid="{AD7C7AAC-4515-4F38-AACF-A38E6B99C9CF}">
+      <formula1>"OUI,NON"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4:F1048576" xr:uid="{29B113A3-BA67-47E6-8B8A-E2219ADE32EA}">
+      <formula1>"Oui,Non"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I5:I1048576 I4 D4:D1048576" xr:uid="{409DDD9F-A932-41BF-BED3-9D409CF955FD}">
+      <formula1>"Court terme, Moyen terme, Long terme"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H4:H1048576" xr:uid="{08B2E6BA-9233-4696-B15F-4D1D036C4550}">
+      <formula1>"Elevé,Moyen,Faible"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAD01D35-7DA1-4A19-9314-8C6D84659D0B}">
   <sheetPr>
     <tabColor rgb="FFFEE7FC"/>
@@ -1877,7 +2019,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D36321D-28CF-4197-97E4-15B03B8FE828}">
   <sheetPr>
     <tabColor rgb="FFFEE7FC"/>
@@ -1943,7 +2085,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8767C8CD-15EF-412F-8BDE-09F42DF51D25}">
   <sheetPr>
     <tabColor rgb="FFFEE7FC"/>
@@ -2066,7 +2208,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93F62B1A-C319-4701-AD63-7BD53F525CF6}">
   <sheetPr>
     <tabColor rgb="FFFEE7FC"/>
@@ -2147,7 +2289,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C465E33-2082-481B-93DA-B52297D05DCF}">
   <sheetPr>
     <tabColor rgb="FFFEE7FC"/>
@@ -2241,7 +2383,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81D0B7EC-F23C-48FB-98BB-3AFB974D2AA9}">
   <sheetPr>
     <tabColor rgb="FFFEE7FC"/>
@@ -2335,7 +2477,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E35E0E35-59BE-44D0-9FD8-FA3A89A617DC}">
   <sheetPr>
     <tabColor rgb="FFE8EDFF"/>
@@ -2391,7 +2533,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBA71AC8-3159-49A5-B6FC-4FA1DF3F7E26}">
   <sheetPr>
     <tabColor rgb="FFE8EDFF"/>
@@ -2476,7 +2618,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDD13986-9BC7-428C-BEF7-5E284E22308C}">
   <sheetPr>
     <tabColor rgb="FFE8EDFF"/>

</xml_diff>

<commit_message>
exporte les indicateurs de C3
</commit_message>
<xml_diff>
--- a/impact/vsme/xlsx/VSME.xlsx
+++ b/impact/vsme/xlsx/VSME.xlsx
@@ -8,30 +8,32 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmonteiro-de-mac-adc\Desktop\ancien bureau\Fichier\CSRD\Tableau ESRS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F85F3BE4-E26B-4DE8-B69D-7530A0D7FF19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2578CB28-8C22-4A67-A7F3-50ADB1D46C11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" firstSheet="1" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="25440" windowHeight="15270" tabRatio="500" firstSheet="2" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="&gt;&gt;&gt; " sheetId="3" r:id="rId1"/>
     <sheet name="B1" sheetId="7" r:id="rId2"/>
     <sheet name="B2" sheetId="2" r:id="rId3"/>
     <sheet name="C1" sheetId="19" r:id="rId4"/>
-    <sheet name="B3" sheetId="18" r:id="rId5"/>
-    <sheet name="B4" sheetId="8" r:id="rId6"/>
-    <sheet name="B5" sheetId="17" r:id="rId7"/>
-    <sheet name="B6" sheetId="9" r:id="rId8"/>
-    <sheet name="B7" sheetId="10" r:id="rId9"/>
-    <sheet name="C4" sheetId="25" r:id="rId10"/>
-    <sheet name="B8" sheetId="15" r:id="rId11"/>
-    <sheet name="B9" sheetId="11" r:id="rId12"/>
-    <sheet name="B10" sheetId="16" r:id="rId13"/>
-    <sheet name="C5" sheetId="23" r:id="rId14"/>
-    <sheet name="C6" sheetId="21" r:id="rId15"/>
-    <sheet name="C7" sheetId="24" r:id="rId16"/>
-    <sheet name="B11" sheetId="14" r:id="rId17"/>
-    <sheet name="C8" sheetId="22" r:id="rId18"/>
-    <sheet name="C9" sheetId="20" r:id="rId19"/>
+    <sheet name="C2" sheetId="27" r:id="rId5"/>
+    <sheet name="B3" sheetId="18" r:id="rId6"/>
+    <sheet name="B4" sheetId="8" r:id="rId7"/>
+    <sheet name="B5" sheetId="17" r:id="rId8"/>
+    <sheet name="B6" sheetId="9" r:id="rId9"/>
+    <sheet name="B7" sheetId="10" r:id="rId10"/>
+    <sheet name="C3" sheetId="28" r:id="rId11"/>
+    <sheet name="C4" sheetId="25" r:id="rId12"/>
+    <sheet name="B8" sheetId="15" r:id="rId13"/>
+    <sheet name="B9" sheetId="11" r:id="rId14"/>
+    <sheet name="B10" sheetId="16" r:id="rId15"/>
+    <sheet name="C5" sheetId="23" r:id="rId16"/>
+    <sheet name="C6" sheetId="21" r:id="rId17"/>
+    <sheet name="C7" sheetId="24" r:id="rId18"/>
+    <sheet name="B11" sheetId="14" r:id="rId19"/>
+    <sheet name="C8" sheetId="22" r:id="rId20"/>
+    <sheet name="C9" sheetId="20" r:id="rId21"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -52,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="232">
   <si>
     <t/>
   </si>
@@ -426,9 +428,6 @@
     <t>Consommation d'électricité</t>
   </si>
   <si>
-    <t>Estimation des émissions brutes de gaz à effet de serre (GES)</t>
-  </si>
-  <si>
     <t>Scope 1</t>
   </si>
   <si>
@@ -631,6 +630,126 @@
   </si>
   <si>
     <t>N° du risque</t>
+  </si>
+  <si>
+    <t>Estimation des émissions brutes de gaz à effet de serre (GES) des scopes 1 et 2</t>
+  </si>
+  <si>
+    <t>Estimation des émissions brutes de gaz à effet de serre (GES) du scope 3</t>
+  </si>
+  <si>
+    <t>Biens et services achetés</t>
+  </si>
+  <si>
+    <t>Biens d'investissement</t>
+  </si>
+  <si>
+    <t>Activités relevant des secteurs des combustibles et de l'énergie</t>
+  </si>
+  <si>
+    <t>Transport et distribution en amont</t>
+  </si>
+  <si>
+    <t>Déchets produits lors de l'exploitation</t>
+  </si>
+  <si>
+    <t>Voyages d'affaires</t>
+  </si>
+  <si>
+    <t>Déplacements domicile-travail des salariés</t>
+  </si>
+  <si>
+    <t>Actifs loués en amont</t>
+  </si>
+  <si>
+    <t>Acheminement en aval</t>
+  </si>
+  <si>
+    <t>Transformation des produits vendus</t>
+  </si>
+  <si>
+    <t>Utilisation des produits vendus</t>
+  </si>
+  <si>
+    <t>Traitement en fin de vie des produits vendus</t>
+  </si>
+  <si>
+    <t>Actifs loués en aval</t>
+  </si>
+  <si>
+    <t>Franchises</t>
+  </si>
+  <si>
+    <t>Investissements</t>
+  </si>
+  <si>
+    <t>Émissions totales des GES du scope 3</t>
+  </si>
+  <si>
+    <t>Émissions totales des GES des scopes 1, 2 (basé sur la localisation) et 3</t>
+  </si>
+  <si>
+    <t>Cibles de réduction des émissions de GES des scopes 1 et 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Année de référence </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Année cible </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valeur de l'année de référence </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valeur de l'année cible </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réduction en pourcentage par rapport à l'année de référence </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Principales actions prévues </t>
+  </si>
+  <si>
+    <t>Plan de transition climatique</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> L'entreprise dispose-t-elle d'un plan de transition climatique ? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Description du plan de transition climatique </t>
+  </si>
+  <si>
+    <t>Contribution du plan de transition climatique à la réduction des émissions de GES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Année prévue d'adoption d'un plan de transition climatique </t>
+  </si>
+  <si>
+    <t>C3 - Cibles de réduction des émissions de GES et transition climatique</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 	Description des pratiques, politiques ou initiatives futures </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Description des cibles définies </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Niveau hiérarchique le plus élevé responsable de la mise en œuvre des politiques </t>
+  </si>
+  <si>
+    <t>Description des pratiques et politiques de durabilité</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2 - Description des pratiques, des politiques et des initiatives futures pour une transition vers une économie plus durable </t>
+  </si>
+  <si>
+    <t>Total scope 3</t>
+  </si>
+  <si>
+    <t>Total scopes 1, 2 et 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total </t>
   </si>
 </sst>
 </file>
@@ -730,7 +849,7 @@
       <name val="Marianne"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -791,6 +910,18 @@
         <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor rgb="FFFEE7FC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB8FEC9"/>
+        <bgColor rgb="FFE8EDFF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="27">
     <border>
@@ -1118,7 +1249,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="79">
+  <cellXfs count="96">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
@@ -1197,6 +1328,15 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1206,6 +1346,15 @@
     <xf numFmtId="0" fontId="11" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1221,24 +1370,6 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1289,6 +1420,57 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1813,6 +1995,410 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{773AF20E-74BF-463C-9F61-BFE009D6FACB}">
+  <sheetPr>
+    <tabColor rgb="FFB8FEC9"/>
+  </sheetPr>
+  <dimension ref="A1:O3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7109375" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="15.7109375" style="11"/>
+    <col min="2" max="2" width="15.7109375" style="1"/>
+    <col min="3" max="7" width="15.7109375" style="2"/>
+    <col min="8" max="8" width="15.7109375" style="14"/>
+    <col min="9" max="9" width="15.7109375" style="2"/>
+    <col min="10" max="10" width="15.7109375" style="12"/>
+    <col min="11" max="16384" width="15.7109375" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" s="20" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="72" t="s">
+        <v>51</v>
+      </c>
+      <c r="B1" s="72"/>
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
+      <c r="E1" s="72"/>
+      <c r="F1" s="72"/>
+      <c r="G1" s="72"/>
+      <c r="H1" s="72"/>
+      <c r="I1" s="72"/>
+      <c r="J1" s="72"/>
+      <c r="K1" s="72"/>
+      <c r="L1" s="72"/>
+      <c r="M1" s="72"/>
+      <c r="N1" s="72"/>
+      <c r="O1" s="72"/>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A2" s="58" t="s">
+        <v>91</v>
+      </c>
+      <c r="B2" s="51" t="s">
+        <v>53</v>
+      </c>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="53"/>
+      <c r="H2" s="51" t="s">
+        <v>60</v>
+      </c>
+      <c r="I2" s="52"/>
+      <c r="J2" s="53"/>
+    </row>
+    <row r="3" spans="1:15" ht="51" x14ac:dyDescent="0.35">
+      <c r="A3" s="59"/>
+      <c r="B3" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="D3" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="F3" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="G3" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="H3" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="I3" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="J3" s="16" t="s">
+        <v>61</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="A1:O1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{749A6938-FD3C-42AA-A2AB-FBC63AEF511E}">
+  <sheetPr>
+    <tabColor rgb="FFB8FEC9"/>
+  </sheetPr>
+  <dimension ref="A1:P21"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7109375" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="2" width="15.7109375" style="12"/>
+    <col min="3" max="6" width="15.7109375" style="82"/>
+    <col min="7" max="7" width="15.7109375" style="87"/>
+    <col min="8" max="11" width="15.7109375" style="82"/>
+    <col min="12" max="12" width="15.7109375" style="87"/>
+    <col min="13" max="15" width="15.7109375" style="93"/>
+    <col min="16" max="16" width="15.7109375" style="94"/>
+    <col min="17" max="16384" width="15.7109375" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" s="20" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="72" t="s">
+        <v>223</v>
+      </c>
+      <c r="B1" s="72"/>
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
+      <c r="E1" s="72"/>
+      <c r="F1" s="72"/>
+      <c r="G1" s="72"/>
+      <c r="H1" s="72"/>
+      <c r="I1" s="72"/>
+      <c r="J1" s="72"/>
+      <c r="K1" s="72"/>
+      <c r="L1" s="72"/>
+      <c r="M1" s="72"/>
+      <c r="N1" s="72"/>
+      <c r="O1" s="72"/>
+      <c r="P1" s="88"/>
+    </row>
+    <row r="2" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="58" t="s">
+        <v>212</v>
+      </c>
+      <c r="B2" s="58" t="s">
+        <v>213</v>
+      </c>
+      <c r="C2" s="83" t="s">
+        <v>211</v>
+      </c>
+      <c r="D2" s="84"/>
+      <c r="E2" s="84"/>
+      <c r="F2" s="84"/>
+      <c r="G2" s="85"/>
+      <c r="H2" s="51" t="s">
+        <v>193</v>
+      </c>
+      <c r="I2" s="52"/>
+      <c r="J2" s="52"/>
+      <c r="K2" s="52"/>
+      <c r="L2" s="53"/>
+      <c r="M2" s="83" t="s">
+        <v>218</v>
+      </c>
+      <c r="N2" s="84"/>
+      <c r="O2" s="84"/>
+      <c r="P2" s="85"/>
+    </row>
+    <row r="3" spans="1:16" ht="63.75" x14ac:dyDescent="0.35">
+      <c r="A3" s="59"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="86"/>
+      <c r="D3" s="18" t="s">
+        <v>214</v>
+      </c>
+      <c r="E3" s="18" t="s">
+        <v>215</v>
+      </c>
+      <c r="F3" s="18" t="s">
+        <v>216</v>
+      </c>
+      <c r="G3" s="16" t="s">
+        <v>217</v>
+      </c>
+      <c r="H3" s="18"/>
+      <c r="I3" s="18" t="s">
+        <v>214</v>
+      </c>
+      <c r="J3" s="18" t="s">
+        <v>215</v>
+      </c>
+      <c r="K3" s="15" t="s">
+        <v>216</v>
+      </c>
+      <c r="L3" s="16" t="s">
+        <v>217</v>
+      </c>
+      <c r="M3" s="18" t="s">
+        <v>219</v>
+      </c>
+      <c r="N3" s="18" t="s">
+        <v>220</v>
+      </c>
+      <c r="O3" s="18" t="s">
+        <v>221</v>
+      </c>
+      <c r="P3" s="16" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="C4" s="18" t="s">
+        <v>124</v>
+      </c>
+      <c r="D4" s="86"/>
+      <c r="E4" s="86"/>
+      <c r="F4" s="86"/>
+      <c r="G4" s="16"/>
+      <c r="H4" s="80" t="s">
+        <v>194</v>
+      </c>
+      <c r="I4" s="89"/>
+      <c r="J4" s="86"/>
+      <c r="K4" s="86"/>
+      <c r="L4" s="90"/>
+      <c r="M4" s="91"/>
+      <c r="N4" s="91"/>
+      <c r="O4" s="91"/>
+      <c r="P4" s="92"/>
+    </row>
+    <row r="5" spans="1:16" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="C5" s="18" t="s">
+        <v>125</v>
+      </c>
+      <c r="D5" s="86"/>
+      <c r="E5" s="86"/>
+      <c r="F5" s="86"/>
+      <c r="G5" s="16"/>
+      <c r="H5" s="80" t="s">
+        <v>195</v>
+      </c>
+      <c r="I5" s="89"/>
+      <c r="J5" s="86"/>
+      <c r="K5" s="86"/>
+      <c r="L5" s="90"/>
+    </row>
+    <row r="6" spans="1:16" ht="51" x14ac:dyDescent="0.35">
+      <c r="C6" s="18" t="s">
+        <v>231</v>
+      </c>
+      <c r="D6" s="86"/>
+      <c r="E6" s="86"/>
+      <c r="F6" s="86"/>
+      <c r="G6" s="16"/>
+      <c r="H6" s="80" t="s">
+        <v>196</v>
+      </c>
+      <c r="I6" s="86"/>
+      <c r="J6" s="86"/>
+      <c r="K6" s="86"/>
+      <c r="L6" s="90"/>
+    </row>
+    <row r="7" spans="1:16" ht="38.25" x14ac:dyDescent="0.35">
+      <c r="C7" s="18"/>
+      <c r="D7" s="86"/>
+      <c r="E7" s="86"/>
+      <c r="F7" s="86"/>
+      <c r="G7" s="16"/>
+      <c r="H7" s="80" t="s">
+        <v>197</v>
+      </c>
+      <c r="I7" s="86"/>
+      <c r="J7" s="86"/>
+      <c r="K7" s="86"/>
+      <c r="L7" s="90"/>
+    </row>
+    <row r="8" spans="1:16" ht="38.25" x14ac:dyDescent="0.35">
+      <c r="H8" s="80" t="s">
+        <v>198</v>
+      </c>
+      <c r="I8" s="86"/>
+      <c r="J8" s="86"/>
+      <c r="K8" s="86"/>
+      <c r="L8" s="95"/>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="H9" s="80" t="s">
+        <v>199</v>
+      </c>
+      <c r="I9" s="86"/>
+      <c r="J9" s="86"/>
+      <c r="K9" s="86"/>
+      <c r="L9" s="95"/>
+    </row>
+    <row r="10" spans="1:16" ht="38.25" x14ac:dyDescent="0.35">
+      <c r="H10" s="80" t="s">
+        <v>200</v>
+      </c>
+      <c r="I10" s="86"/>
+      <c r="J10" s="86"/>
+      <c r="K10" s="86"/>
+      <c r="L10" s="95"/>
+    </row>
+    <row r="11" spans="1:16" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="H11" s="80" t="s">
+        <v>201</v>
+      </c>
+      <c r="I11" s="86"/>
+      <c r="J11" s="86"/>
+      <c r="K11" s="86"/>
+      <c r="L11" s="95"/>
+    </row>
+    <row r="12" spans="1:16" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="H12" s="80" t="s">
+        <v>202</v>
+      </c>
+      <c r="I12" s="86"/>
+      <c r="J12" s="86"/>
+      <c r="K12" s="86"/>
+      <c r="L12" s="95"/>
+    </row>
+    <row r="13" spans="1:16" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="H13" s="80" t="s">
+        <v>203</v>
+      </c>
+      <c r="I13" s="86"/>
+      <c r="J13" s="86"/>
+      <c r="K13" s="86"/>
+      <c r="L13" s="95"/>
+    </row>
+    <row r="14" spans="1:16" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="H14" s="80" t="s">
+        <v>204</v>
+      </c>
+      <c r="I14" s="86"/>
+      <c r="J14" s="86"/>
+      <c r="K14" s="86"/>
+      <c r="L14" s="95"/>
+    </row>
+    <row r="15" spans="1:16" ht="38.25" x14ac:dyDescent="0.35">
+      <c r="H15" s="80" t="s">
+        <v>205</v>
+      </c>
+      <c r="I15" s="86"/>
+      <c r="J15" s="86"/>
+      <c r="K15" s="86"/>
+      <c r="L15" s="95"/>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="H16" s="80" t="s">
+        <v>206</v>
+      </c>
+      <c r="I16" s="86"/>
+      <c r="J16" s="86"/>
+      <c r="K16" s="86"/>
+      <c r="L16" s="95"/>
+    </row>
+    <row r="17" spans="8:12" x14ac:dyDescent="0.35">
+      <c r="H17" s="80" t="s">
+        <v>207</v>
+      </c>
+      <c r="I17" s="86"/>
+      <c r="J17" s="86"/>
+      <c r="K17" s="86"/>
+      <c r="L17" s="95"/>
+    </row>
+    <row r="18" spans="8:12" x14ac:dyDescent="0.35">
+      <c r="H18" s="80" t="s">
+        <v>208</v>
+      </c>
+      <c r="I18" s="86"/>
+      <c r="J18" s="86"/>
+      <c r="K18" s="86"/>
+      <c r="L18" s="95"/>
+    </row>
+    <row r="19" spans="8:12" x14ac:dyDescent="0.35">
+      <c r="H19" s="80" t="s">
+        <v>229</v>
+      </c>
+      <c r="I19" s="89"/>
+      <c r="J19" s="89"/>
+      <c r="K19" s="89"/>
+      <c r="L19" s="90"/>
+    </row>
+    <row r="20" spans="8:12" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="H20" s="80" t="s">
+        <v>230</v>
+      </c>
+      <c r="I20" s="89"/>
+      <c r="J20" s="89"/>
+      <c r="K20" s="89"/>
+      <c r="L20" s="90"/>
+    </row>
+    <row r="21" spans="8:12" x14ac:dyDescent="0.35">
+      <c r="H21" s="81"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:G2"/>
+    <mergeCell ref="H2:L2"/>
+    <mergeCell ref="M2:P2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AD57197-9ADC-43C0-B70E-801EE1BD86F4}">
   <sheetPr>
     <tabColor rgb="FFB8FEC9"/>
@@ -1830,7 +2416,7 @@
   <sheetData>
     <row r="1" spans="1:16" s="20" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="72" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B1" s="72"/>
       <c r="C1" s="72"/>
@@ -1849,47 +2435,47 @@
       <c r="P1" s="72"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A2" s="48" t="s">
-        <v>182</v>
-      </c>
-      <c r="B2" s="49"/>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="50"/>
-      <c r="F2" s="48" t="s">
-        <v>187</v>
-      </c>
-      <c r="G2" s="49"/>
-      <c r="H2" s="49"/>
-      <c r="I2" s="50"/>
+      <c r="A2" s="51" t="s">
+        <v>181</v>
+      </c>
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="53"/>
+      <c r="F2" s="51" t="s">
+        <v>186</v>
+      </c>
+      <c r="G2" s="52"/>
+      <c r="H2" s="52"/>
+      <c r="I2" s="53"/>
     </row>
     <row r="3" spans="1:16" ht="38.25" x14ac:dyDescent="0.35">
       <c r="A3" s="15" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B3" s="15" t="s">
+        <v>182</v>
+      </c>
+      <c r="C3" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="D3" s="15" t="s">
         <v>184</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="E3" s="15" t="s">
         <v>185</v>
       </c>
-      <c r="E3" s="15" t="s">
-        <v>186</v>
-      </c>
       <c r="F3" s="17" t="s">
+        <v>187</v>
+      </c>
+      <c r="G3" s="15" t="s">
         <v>188</v>
       </c>
-      <c r="G3" s="15" t="s">
+      <c r="H3" s="15" t="s">
         <v>189</v>
       </c>
-      <c r="H3" s="15" t="s">
-        <v>190</v>
-      </c>
       <c r="I3" s="16" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
   </sheetData>
@@ -1914,7 +2500,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAD01D35-7DA1-4A19-9314-8C6D84659D0B}">
   <sheetPr>
     <tabColor rgb="FFFEE7FC"/>
@@ -1952,21 +2538,21 @@
       <c r="O1" s="73"/>
     </row>
     <row r="2" spans="1:15" ht="39" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="48" t="s">
+      <c r="A2" s="51" t="s">
         <v>80</v>
       </c>
-      <c r="B2" s="50"/>
-      <c r="C2" s="48" t="s">
+      <c r="B2" s="53"/>
+      <c r="C2" s="51" t="s">
         <v>83</v>
       </c>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="50"/>
-      <c r="G2" s="48" t="s">
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="53"/>
+      <c r="G2" s="51" t="s">
         <v>86</v>
       </c>
-      <c r="H2" s="50"/>
-      <c r="I2" s="52" t="s">
+      <c r="H2" s="53"/>
+      <c r="I2" s="58" t="s">
         <v>88</v>
       </c>
     </row>
@@ -1995,7 +2581,7 @@
       <c r="H3" s="15" t="s">
         <v>87</v>
       </c>
-      <c r="I3" s="53"/>
+      <c r="I3" s="59"/>
     </row>
     <row r="12" spans="1:15" ht="72.75" x14ac:dyDescent="1.25">
       <c r="E12" s="22"/>
@@ -2013,7 +2599,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D36321D-28CF-4197-97E4-15B03B8FE828}">
   <sheetPr>
     <tabColor rgb="FFFEE7FC"/>
@@ -2048,11 +2634,11 @@
       <c r="O1" s="73"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A2" s="48" t="s">
+      <c r="A2" s="51" t="s">
         <v>64</v>
       </c>
-      <c r="B2" s="50"/>
-      <c r="C2" s="52" t="s">
+      <c r="B2" s="53"/>
+      <c r="C2" s="58" t="s">
         <v>67</v>
       </c>
     </row>
@@ -2063,7 +2649,7 @@
       <c r="B3" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="C3" s="53"/>
+      <c r="C3" s="59"/>
     </row>
     <row r="12" spans="1:15" ht="72.75" x14ac:dyDescent="1.25">
       <c r="E12" s="22"/>
@@ -2079,7 +2665,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8767C8CD-15EF-412F-8BDE-09F42DF51D25}">
   <sheetPr>
     <tabColor rgb="FFFEE7FC"/>
@@ -2118,26 +2704,26 @@
       <c r="O1" s="73"/>
     </row>
     <row r="2" spans="1:15" ht="54.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="58" t="s">
         <v>93</v>
       </c>
-      <c r="B2" s="48" t="s">
+      <c r="B2" s="51" t="s">
         <v>94</v>
       </c>
-      <c r="C2" s="49"/>
-      <c r="D2" s="50"/>
-      <c r="E2" s="48" t="s">
+      <c r="C2" s="52"/>
+      <c r="D2" s="53"/>
+      <c r="E2" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="F2" s="50"/>
-      <c r="G2" s="48" t="s">
+      <c r="F2" s="53"/>
+      <c r="G2" s="51" t="s">
         <v>105</v>
       </c>
-      <c r="H2" s="49"/>
-      <c r="I2" s="50"/>
+      <c r="H2" s="52"/>
+      <c r="I2" s="53"/>
     </row>
     <row r="3" spans="1:15" ht="97.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="53"/>
+      <c r="A3" s="59"/>
       <c r="B3" s="15" t="s">
         <v>95</v>
       </c>
@@ -2202,7 +2788,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93F62B1A-C319-4701-AD63-7BD53F525CF6}">
   <sheetPr>
     <tabColor rgb="FFFEE7FC"/>
@@ -2219,7 +2805,7 @@
   <sheetData>
     <row r="1" spans="1:15" s="21" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="73" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B1" s="73"/>
       <c r="C1" s="73"/>
@@ -2237,31 +2823,31 @@
       <c r="O1" s="73"/>
     </row>
     <row r="2" spans="1:15" ht="53.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="48" t="s">
-        <v>168</v>
-      </c>
-      <c r="B2" s="49"/>
-      <c r="C2" s="50"/>
-      <c r="D2" s="48" t="s">
-        <v>171</v>
-      </c>
-      <c r="E2" s="50"/>
+      <c r="A2" s="51" t="s">
+        <v>167</v>
+      </c>
+      <c r="B2" s="52"/>
+      <c r="C2" s="53"/>
+      <c r="D2" s="51" t="s">
+        <v>170</v>
+      </c>
+      <c r="E2" s="53"/>
     </row>
     <row r="3" spans="1:15" ht="114.75" x14ac:dyDescent="0.35">
       <c r="A3" s="15" t="s">
+        <v>165</v>
+      </c>
+      <c r="B3" s="15" t="s">
         <v>166</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="C3" s="16" t="s">
         <v>167</v>
       </c>
-      <c r="C3" s="16" t="s">
+      <c r="D3" s="15" t="s">
         <v>168</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="E3" s="16" t="s">
         <v>169</v>
-      </c>
-      <c r="E3" s="16" t="s">
-        <v>170</v>
       </c>
     </row>
   </sheetData>
@@ -2283,7 +2869,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C465E33-2082-481B-93DA-B52297D05DCF}">
   <sheetPr>
     <tabColor rgb="FFFEE7FC"/>
@@ -2300,7 +2886,7 @@
   <sheetData>
     <row r="1" spans="1:19" s="21" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="73" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B1" s="73"/>
       <c r="C1" s="73"/>
@@ -2322,38 +2908,38 @@
       <c r="S1" s="73"/>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A2" s="48" t="s">
-        <v>147</v>
-      </c>
-      <c r="B2" s="49"/>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="50"/>
-      <c r="G2" s="52" t="s">
-        <v>154</v>
+      <c r="A2" s="51" t="s">
+        <v>146</v>
+      </c>
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="53"/>
+      <c r="G2" s="58" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="3" spans="1:19" ht="89.25" x14ac:dyDescent="0.35">
       <c r="A3" s="15" t="s">
+        <v>147</v>
+      </c>
+      <c r="B3" s="15" t="s">
         <v>148</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="C3" s="15" t="s">
         <v>149</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="D3" s="15" t="s">
         <v>150</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="E3" s="15" t="s">
         <v>151</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="F3" s="16" t="s">
         <v>152</v>
       </c>
-      <c r="F3" s="16" t="s">
-        <v>153</v>
-      </c>
-      <c r="G3" s="53"/>
+      <c r="G3" s="59"/>
     </row>
     <row r="12" spans="1:19" ht="72.75" x14ac:dyDescent="1.25">
       <c r="I12" s="22"/>
@@ -2377,7 +2963,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81D0B7EC-F23C-48FB-98BB-3AFB974D2AA9}">
   <sheetPr>
     <tabColor rgb="FFFEE7FC"/>
@@ -2394,7 +2980,7 @@
   <sheetData>
     <row r="1" spans="1:19" s="21" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="73" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B1" s="73"/>
       <c r="C1" s="73"/>
@@ -2416,38 +3002,38 @@
       <c r="S1" s="73"/>
     </row>
     <row r="2" spans="1:19" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="48" t="s">
-        <v>173</v>
-      </c>
-      <c r="B2" s="49"/>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="50"/>
-      <c r="G2" s="52" t="s">
-        <v>180</v>
+      <c r="A2" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="53"/>
+      <c r="G2" s="58" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="3" spans="1:19" ht="127.5" x14ac:dyDescent="0.35">
       <c r="A3" s="15" t="s">
+        <v>173</v>
+      </c>
+      <c r="B3" s="15" t="s">
         <v>174</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="C3" s="15" t="s">
         <v>175</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="D3" s="15" t="s">
         <v>176</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="E3" s="15" t="s">
+        <v>178</v>
+      </c>
+      <c r="F3" s="16" t="s">
         <v>177</v>
       </c>
-      <c r="E3" s="15" t="s">
-        <v>179</v>
-      </c>
-      <c r="F3" s="16" t="s">
-        <v>178</v>
-      </c>
-      <c r="G3" s="53"/>
+      <c r="G3" s="59"/>
     </row>
     <row r="12" spans="1:19" ht="72.75" x14ac:dyDescent="1.25">
       <c r="I12" s="22"/>
@@ -2471,7 +3057,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E35E0E35-59BE-44D0-9FD8-FA3A89A617DC}">
   <sheetPr>
     <tabColor rgb="FFE8EDFF"/>
@@ -2521,140 +3107,6 @@
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="A1:O1"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBA71AC8-3159-49A5-B6FC-4FA1DF3F7E26}">
-  <sheetPr>
-    <tabColor rgb="FFE8EDFF"/>
-  </sheetPr>
-  <dimension ref="A1:L3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7109375" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="15.7109375" style="1"/>
-    <col min="2" max="6" width="15.7109375" style="2"/>
-    <col min="7" max="7" width="15.7109375" style="12"/>
-    <col min="8" max="8" width="18.140625" style="12" customWidth="1"/>
-    <col min="9" max="16384" width="15.7109375" style="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:12" s="23" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="78" t="s">
-        <v>164</v>
-      </c>
-      <c r="B1" s="78"/>
-      <c r="C1" s="78"/>
-      <c r="D1" s="78"/>
-      <c r="E1" s="78"/>
-      <c r="F1" s="78"/>
-      <c r="G1" s="78"/>
-      <c r="H1" s="78"/>
-      <c r="I1" s="78"/>
-      <c r="J1" s="78"/>
-      <c r="K1" s="78"/>
-      <c r="L1" s="78"/>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A2" s="48" t="s">
-        <v>163</v>
-      </c>
-      <c r="B2" s="49"/>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="49"/>
-      <c r="G2" s="50"/>
-      <c r="H2" s="51" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" ht="63.75" x14ac:dyDescent="0.35">
-      <c r="A3" s="15" t="s">
-        <v>156</v>
-      </c>
-      <c r="B3" s="15" t="s">
-        <v>157</v>
-      </c>
-      <c r="C3" s="15" t="s">
-        <v>158</v>
-      </c>
-      <c r="D3" s="15" t="s">
-        <v>159</v>
-      </c>
-      <c r="E3" s="15" t="s">
-        <v>160</v>
-      </c>
-      <c r="F3" s="15" t="s">
-        <v>165</v>
-      </c>
-      <c r="G3" s="16" t="s">
-        <v>161</v>
-      </c>
-      <c r="H3" s="50"/>
-    </row>
-  </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="H2:H3"/>
-  </mergeCells>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H4:H6" xr:uid="{B7229605-3AFC-4A61-911C-7A7A7D3FA5D1}">
-      <formula1>"Oui,Non"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDD13986-9BC7-428C-BEF7-5E284E22308C}">
-  <sheetPr>
-    <tabColor rgb="FFE8EDFF"/>
-  </sheetPr>
-  <dimension ref="A1:N3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="22.28515625" style="11" customWidth="1"/>
-    <col min="2" max="4" width="11.42578125" style="2" customWidth="1"/>
-    <col min="5" max="16384" width="11.42578125" style="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:14" s="23" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="78" t="s">
-        <v>145</v>
-      </c>
-      <c r="B1" s="78"/>
-      <c r="C1" s="78"/>
-      <c r="D1" s="78"/>
-      <c r="E1" s="78"/>
-      <c r="F1" s="78"/>
-      <c r="G1" s="78"/>
-      <c r="H1" s="78"/>
-      <c r="I1" s="78"/>
-      <c r="J1" s="78"/>
-      <c r="K1" s="78"/>
-      <c r="L1" s="78"/>
-      <c r="M1" s="78"/>
-      <c r="N1" s="78"/>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A2" s="74" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" ht="55.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="75"/>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:N1"/>
-    <mergeCell ref="A2:A3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -2688,86 +3140,86 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" s="10" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="56" t="s">
+      <c r="A1" s="48" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
-      <c r="K1" s="56"/>
-      <c r="L1" s="56"/>
-      <c r="M1" s="56"/>
-      <c r="N1" s="56"/>
-      <c r="O1" s="56"/>
-      <c r="P1" s="56"/>
-      <c r="Q1" s="56"/>
-      <c r="R1" s="56"/>
-      <c r="S1" s="56"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
+      <c r="K1" s="48"/>
+      <c r="L1" s="48"/>
+      <c r="M1" s="48"/>
+      <c r="N1" s="48"/>
+      <c r="O1" s="48"/>
+      <c r="P1" s="48"/>
+      <c r="Q1" s="48"/>
+      <c r="R1" s="48"/>
+      <c r="S1" s="48"/>
     </row>
     <row r="2" spans="1:28" s="19" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="51" t="s">
+      <c r="A2" s="57" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="52" t="s">
+      <c r="B2" s="58" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="52" t="s">
+      <c r="C2" s="58" t="s">
         <v>19</v>
       </c>
-      <c r="D2" s="48" t="s">
+      <c r="D2" s="51" t="s">
         <v>20</v>
       </c>
-      <c r="E2" s="49"/>
-      <c r="F2" s="49"/>
-      <c r="G2" s="49"/>
-      <c r="H2" s="50"/>
-      <c r="I2" s="57" t="s">
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52"/>
+      <c r="H2" s="53"/>
+      <c r="I2" s="49" t="s">
         <v>31</v>
       </c>
-      <c r="J2" s="58"/>
-      <c r="K2" s="54" t="s">
+      <c r="J2" s="50"/>
+      <c r="K2" s="60" t="s">
         <v>90</v>
       </c>
-      <c r="L2" s="52" t="s">
+      <c r="L2" s="58" t="s">
         <v>21</v>
       </c>
-      <c r="M2" s="54" t="s">
+      <c r="M2" s="60" t="s">
         <v>89</v>
       </c>
-      <c r="N2" s="57" t="s">
+      <c r="N2" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="O2" s="58"/>
-      <c r="P2" s="54" t="s">
+      <c r="O2" s="50"/>
+      <c r="P2" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="Q2" s="59" t="s">
+      <c r="Q2" s="54" t="s">
         <v>24</v>
       </c>
-      <c r="R2" s="60"/>
-      <c r="S2" s="60"/>
-      <c r="T2" s="60"/>
-      <c r="U2" s="60"/>
-      <c r="V2" s="60"/>
-      <c r="W2" s="61"/>
-      <c r="X2" s="48" t="s">
+      <c r="R2" s="55"/>
+      <c r="S2" s="55"/>
+      <c r="T2" s="55"/>
+      <c r="U2" s="55"/>
+      <c r="V2" s="55"/>
+      <c r="W2" s="56"/>
+      <c r="X2" s="51" t="s">
         <v>25</v>
       </c>
-      <c r="Y2" s="49"/>
-      <c r="Z2" s="49"/>
-      <c r="AA2" s="49"/>
-      <c r="AB2" s="50"/>
+      <c r="Y2" s="52"/>
+      <c r="Z2" s="52"/>
+      <c r="AA2" s="52"/>
+      <c r="AB2" s="53"/>
     </row>
     <row r="3" spans="1:28" ht="38.25" x14ac:dyDescent="0.35">
-      <c r="A3" s="50"/>
-      <c r="B3" s="53"/>
-      <c r="C3" s="53"/>
+      <c r="A3" s="53"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="59"/>
       <c r="D3" s="15" t="s">
         <v>26</v>
       </c>
@@ -2789,16 +3241,16 @@
       <c r="J3" s="46" t="s">
         <v>73</v>
       </c>
-      <c r="K3" s="55"/>
-      <c r="L3" s="53"/>
-      <c r="M3" s="55"/>
+      <c r="K3" s="61"/>
+      <c r="L3" s="59"/>
+      <c r="M3" s="61"/>
       <c r="N3" s="45" t="s">
         <v>74</v>
       </c>
       <c r="O3" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="P3" s="55"/>
+      <c r="P3" s="61"/>
       <c r="Q3" s="17" t="s">
         <v>72</v>
       </c>
@@ -2838,11 +3290,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="A1:S1"/>
-    <mergeCell ref="N2:O2"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="Q2:W2"/>
     <mergeCell ref="X2:AB2"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="B2:B3"/>
@@ -2851,9 +3298,148 @@
     <mergeCell ref="M2:M3"/>
     <mergeCell ref="P2:P3"/>
     <mergeCell ref="K2:K3"/>
+    <mergeCell ref="A1:S1"/>
+    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="Q2:W2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBA71AC8-3159-49A5-B6FC-4FA1DF3F7E26}">
+  <sheetPr>
+    <tabColor rgb="FFE8EDFF"/>
+  </sheetPr>
+  <dimension ref="A1:L3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7109375" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="15.7109375" style="1"/>
+    <col min="2" max="6" width="15.7109375" style="2"/>
+    <col min="7" max="7" width="15.7109375" style="12"/>
+    <col min="8" max="8" width="18.140625" style="12" customWidth="1"/>
+    <col min="9" max="16384" width="15.7109375" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" s="23" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="78" t="s">
+        <v>163</v>
+      </c>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
+      <c r="F1" s="78"/>
+      <c r="G1" s="78"/>
+      <c r="H1" s="78"/>
+      <c r="I1" s="78"/>
+      <c r="J1" s="78"/>
+      <c r="K1" s="78"/>
+      <c r="L1" s="78"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A2" s="51" t="s">
+        <v>162</v>
+      </c>
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="53"/>
+      <c r="H2" s="57" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="63.75" x14ac:dyDescent="0.35">
+      <c r="A3" s="15" t="s">
+        <v>155</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>156</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>157</v>
+      </c>
+      <c r="D3" s="15" t="s">
+        <v>158</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>159</v>
+      </c>
+      <c r="F3" s="15" t="s">
+        <v>164</v>
+      </c>
+      <c r="G3" s="16" t="s">
+        <v>160</v>
+      </c>
+      <c r="H3" s="53"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="H2:H3"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H4:H6" xr:uid="{B7229605-3AFC-4A61-911C-7A7A7D3FA5D1}">
+      <formula1>"Oui,Non"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDD13986-9BC7-428C-BEF7-5E284E22308C}">
+  <sheetPr>
+    <tabColor rgb="FFE8EDFF"/>
+  </sheetPr>
+  <dimension ref="A1:N3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="22.28515625" style="11" customWidth="1"/>
+    <col min="2" max="4" width="11.42578125" style="2" customWidth="1"/>
+    <col min="5" max="16384" width="11.42578125" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" s="23" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="78" t="s">
+        <v>144</v>
+      </c>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
+      <c r="F1" s="78"/>
+      <c r="G1" s="78"/>
+      <c r="H1" s="78"/>
+      <c r="I1" s="78"/>
+      <c r="J1" s="78"/>
+      <c r="K1" s="78"/>
+      <c r="L1" s="78"/>
+      <c r="M1" s="78"/>
+      <c r="N1" s="78"/>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A2" s="74" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" ht="55.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="75"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A2:A3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
@@ -2876,29 +3462,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" s="10" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="56" t="s">
+      <c r="A1" s="48" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
-      <c r="K1" s="56"/>
-      <c r="L1" s="56"/>
-      <c r="M1" s="56"/>
-      <c r="N1" s="56"/>
-      <c r="O1" s="56"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
+      <c r="K1" s="48"/>
+      <c r="L1" s="48"/>
+      <c r="M1" s="48"/>
+      <c r="N1" s="48"/>
+      <c r="O1" s="48"/>
     </row>
     <row r="2" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="62" t="s">
         <v>75</v>
       </c>
-      <c r="B2" s="52" t="s">
+      <c r="B2" s="58" t="s">
         <v>76</v>
       </c>
       <c r="C2" s="64" t="s">
@@ -2913,12 +3499,12 @@
     </row>
     <row r="3" spans="1:15" ht="41.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="63"/>
-      <c r="B3" s="53"/>
-      <c r="C3" s="49"/>
-      <c r="D3" s="48"/>
-      <c r="E3" s="49"/>
-      <c r="F3" s="49"/>
-      <c r="G3" s="50"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="52"/>
+      <c r="D3" s="51"/>
+      <c r="E3" s="52"/>
+      <c r="F3" s="52"/>
+      <c r="G3" s="53"/>
     </row>
     <row r="4" spans="1:15" ht="48" thickBot="1" x14ac:dyDescent="0.4">
       <c r="E4" s="25" t="s">
@@ -3044,41 +3630,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" s="10" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="56" t="s">
-        <v>144</v>
-      </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
-      <c r="K1" s="56"/>
-      <c r="L1" s="56"/>
-      <c r="M1" s="56"/>
+      <c r="A1" s="48" t="s">
+        <v>143</v>
+      </c>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
+      <c r="K1" s="48"/>
+      <c r="L1" s="48"/>
+      <c r="M1" s="48"/>
     </row>
     <row r="2" spans="1:13" s="19" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="51" t="s">
+      <c r="A2" s="57" t="s">
+        <v>139</v>
+      </c>
+      <c r="B2" s="58" t="s">
         <v>140</v>
       </c>
-      <c r="B2" s="52" t="s">
+      <c r="C2" s="58" t="s">
         <v>141</v>
       </c>
-      <c r="C2" s="52" t="s">
+      <c r="D2" s="58" t="s">
         <v>142</v>
       </c>
-      <c r="D2" s="52" t="s">
-        <v>143</v>
-      </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A3" s="50"/>
-      <c r="B3" s="53"/>
-      <c r="C3" s="53"/>
-      <c r="D3" s="53"/>
+      <c r="A3" s="53"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -3094,11 +3680,158 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3A89080-2C89-4599-81BF-8F339FE8E625}">
+  <sheetPr>
+    <tabColor rgb="FFFFEDC3"/>
+  </sheetPr>
+  <dimension ref="A1:M14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7109375" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="38.28515625" style="14" customWidth="1"/>
+    <col min="2" max="2" width="23.7109375" style="2" customWidth="1"/>
+    <col min="3" max="3" width="21.85546875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="20.42578125" style="12" customWidth="1"/>
+    <col min="5" max="16384" width="15.7109375" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" s="10" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="48" t="s">
+        <v>228</v>
+      </c>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
+      <c r="K1" s="48"/>
+      <c r="L1" s="48"/>
+      <c r="M1" s="48"/>
+    </row>
+    <row r="2" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="65" t="s">
+        <v>227</v>
+      </c>
+      <c r="B2" s="66"/>
+      <c r="C2" s="66"/>
+      <c r="D2" s="67"/>
+    </row>
+    <row r="3" spans="1:13" ht="41.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="51"/>
+      <c r="B3" s="52"/>
+      <c r="C3" s="52"/>
+      <c r="D3" s="53"/>
+    </row>
+    <row r="4" spans="1:13" ht="79.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B4" s="25" t="s">
+        <v>224</v>
+      </c>
+      <c r="C4" s="26" t="s">
+        <v>225</v>
+      </c>
+      <c r="D4" s="27" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A5" s="28" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="29"/>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A6" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="29"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A7" s="31" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="9"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="29"/>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A8" s="31" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="9"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="29"/>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A9" s="31" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="9"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="29"/>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A10" s="32" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="9"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="29"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A11" s="32" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="9"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="29"/>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A12" s="32" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="9"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="29"/>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A13" s="32" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="9"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="29"/>
+    </row>
+    <row r="14" spans="1:13" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="33" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="34"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:D3"/>
+    <mergeCell ref="A1:M1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C0E4342-D345-4F6D-8348-EF5BA58D69DD}">
   <sheetPr>
     <tabColor rgb="FFB8FEC9"/>
   </sheetPr>
-  <dimension ref="A1:U4"/>
+  <dimension ref="A1:AL4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="15.7109375" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="15.7109375" style="1"/>
@@ -3113,10 +3846,13 @@
     <col min="18" max="19" width="15.7109375" style="1"/>
     <col min="20" max="20" width="15.7109375" style="11"/>
     <col min="21" max="21" width="15.7109375" style="12"/>
-    <col min="22" max="16384" width="15.7109375" style="2"/>
+    <col min="22" max="36" width="15.7109375" style="1"/>
+    <col min="37" max="37" width="15.7109375" style="24"/>
+    <col min="38" max="38" width="15.7109375" style="12"/>
+    <col min="39" max="16384" width="15.7109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" s="20" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:38" s="20" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="72" t="s">
         <v>119</v>
       </c>
@@ -3136,15 +3872,32 @@
       <c r="S1" s="44"/>
       <c r="T1" s="44"/>
       <c r="U1" s="44"/>
-    </row>
-    <row r="2" spans="1:21" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="49" t="s">
+      <c r="V1" s="44"/>
+      <c r="W1" s="44"/>
+      <c r="X1" s="44"/>
+      <c r="Y1" s="44"/>
+      <c r="Z1" s="44"/>
+      <c r="AA1" s="44"/>
+      <c r="AB1" s="44"/>
+      <c r="AC1" s="44"/>
+      <c r="AD1" s="44"/>
+      <c r="AE1" s="44"/>
+      <c r="AF1" s="44"/>
+      <c r="AG1" s="44"/>
+      <c r="AH1" s="44"/>
+      <c r="AI1" s="44"/>
+      <c r="AJ1" s="44"/>
+      <c r="AK1" s="44"/>
+      <c r="AL1" s="44"/>
+    </row>
+    <row r="2" spans="1:38" ht="35.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="52" t="s">
         <v>123</v>
       </c>
-      <c r="B2" s="49"/>
-      <c r="C2" s="50"/>
+      <c r="B2" s="52"/>
+      <c r="C2" s="53"/>
       <c r="D2" s="69" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E2" s="70"/>
       <c r="F2" s="70"/>
@@ -3159,14 +3912,33 @@
       <c r="O2" s="70"/>
       <c r="P2" s="70"/>
       <c r="Q2" s="71"/>
-      <c r="R2" s="49" t="s">
-        <v>124</v>
-      </c>
-      <c r="S2" s="49"/>
-      <c r="T2" s="49"/>
-      <c r="U2" s="50"/>
-    </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="R2" s="52" t="s">
+        <v>192</v>
+      </c>
+      <c r="S2" s="52"/>
+      <c r="T2" s="52"/>
+      <c r="U2" s="53"/>
+      <c r="V2" s="52" t="s">
+        <v>193</v>
+      </c>
+      <c r="W2" s="52"/>
+      <c r="X2" s="52"/>
+      <c r="Y2" s="52"/>
+      <c r="Z2" s="52"/>
+      <c r="AA2" s="52"/>
+      <c r="AB2" s="52"/>
+      <c r="AC2" s="52"/>
+      <c r="AD2" s="52"/>
+      <c r="AE2" s="52"/>
+      <c r="AF2" s="52"/>
+      <c r="AG2" s="52"/>
+      <c r="AH2" s="52"/>
+      <c r="AI2" s="52"/>
+      <c r="AJ2" s="52"/>
+      <c r="AK2" s="52"/>
+      <c r="AL2" s="53"/>
+    </row>
+    <row r="3" spans="1:38" ht="51" x14ac:dyDescent="0.35">
       <c r="A3" s="15" t="s">
         <v>120</v>
       </c>
@@ -3177,7 +3949,7 @@
         <v>122</v>
       </c>
       <c r="D3" s="68" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E3" s="68"/>
       <c r="F3" s="68"/>
@@ -3187,61 +3959,112 @@
       <c r="J3" s="68"/>
       <c r="K3" s="68"/>
       <c r="L3" s="68" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="M3" s="68"/>
       <c r="N3" s="68"/>
       <c r="O3" s="68" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="P3" s="68"/>
       <c r="Q3" s="68"/>
       <c r="R3" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="S3" s="15" t="s">
         <v>125</v>
-      </c>
-      <c r="S3" s="15" t="s">
-        <v>126</v>
       </c>
       <c r="T3" s="16" t="s">
         <v>122</v>
       </c>
       <c r="U3" s="16" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="4" spans="1:21" ht="25.5" x14ac:dyDescent="0.35">
+        <v>126</v>
+      </c>
+      <c r="V3" s="15" t="s">
+        <v>194</v>
+      </c>
+      <c r="W3" s="15" t="s">
+        <v>195</v>
+      </c>
+      <c r="X3" s="15" t="s">
+        <v>196</v>
+      </c>
+      <c r="Y3" s="15" t="s">
+        <v>197</v>
+      </c>
+      <c r="Z3" s="15" t="s">
+        <v>198</v>
+      </c>
+      <c r="AA3" s="15" t="s">
+        <v>199</v>
+      </c>
+      <c r="AB3" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="AC3" s="15" t="s">
+        <v>201</v>
+      </c>
+      <c r="AD3" s="15" t="s">
+        <v>202</v>
+      </c>
+      <c r="AE3" s="15" t="s">
+        <v>203</v>
+      </c>
+      <c r="AF3" s="15" t="s">
+        <v>204</v>
+      </c>
+      <c r="AG3" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="AH3" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="AI3" s="15" t="s">
+        <v>207</v>
+      </c>
+      <c r="AJ3" s="15" t="s">
+        <v>208</v>
+      </c>
+      <c r="AK3" s="79" t="s">
+        <v>209</v>
+      </c>
+      <c r="AL3" s="16" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="4" spans="1:38" ht="25.5" x14ac:dyDescent="0.35">
       <c r="D4" s="16" t="s">
+        <v>130</v>
+      </c>
+      <c r="E4" s="16" t="s">
         <v>131</v>
       </c>
-      <c r="E4" s="16" t="s">
+      <c r="F4" s="16" t="s">
         <v>132</v>
       </c>
-      <c r="F4" s="16" t="s">
+      <c r="G4" s="16" t="s">
+        <v>137</v>
+      </c>
+      <c r="H4" s="16" t="s">
+        <v>138</v>
+      </c>
+      <c r="I4" s="16" t="s">
         <v>133</v>
-      </c>
-      <c r="G4" s="16" t="s">
-        <v>138</v>
-      </c>
-      <c r="H4" s="16" t="s">
-        <v>139</v>
-      </c>
-      <c r="I4" s="16" t="s">
-        <v>134</v>
       </c>
       <c r="J4" s="16" t="s">
         <v>42</v>
       </c>
       <c r="K4" s="16" t="s">
+        <v>134</v>
+      </c>
+      <c r="L4" s="16" t="s">
+        <v>130</v>
+      </c>
+      <c r="M4" s="16" t="s">
+        <v>132</v>
+      </c>
+      <c r="N4" s="16" t="s">
         <v>135</v>
-      </c>
-      <c r="L4" s="16" t="s">
-        <v>131</v>
-      </c>
-      <c r="M4" s="16" t="s">
-        <v>133</v>
-      </c>
-      <c r="N4" s="16" t="s">
-        <v>136</v>
       </c>
       <c r="O4" s="16" t="s">
         <v>120</v>
@@ -3254,7 +4077,8 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
+    <mergeCell ref="V2:AL2"/>
     <mergeCell ref="O3:Q3"/>
     <mergeCell ref="D2:Q2"/>
     <mergeCell ref="A1:M1"/>
@@ -3268,7 +4092,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5692AB71-D55C-4890-A4C4-4497C431AAF2}">
   <sheetPr>
     <tabColor rgb="FFB8FEC9"/>
@@ -3306,21 +4130,21 @@
       <c r="O1" s="72"/>
     </row>
     <row r="2" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="48" t="s">
+      <c r="A2" s="51" t="s">
         <v>44</v>
       </c>
-      <c r="B2" s="49"/>
-      <c r="C2" s="50"/>
-      <c r="D2" s="48" t="s">
+      <c r="B2" s="52"/>
+      <c r="C2" s="53"/>
+      <c r="D2" s="51" t="s">
         <v>45</v>
       </c>
-      <c r="E2" s="49"/>
-      <c r="F2" s="50"/>
-      <c r="G2" s="48" t="s">
+      <c r="E2" s="52"/>
+      <c r="F2" s="53"/>
+      <c r="G2" s="51" t="s">
         <v>46</v>
       </c>
-      <c r="H2" s="49"/>
-      <c r="I2" s="50"/>
+      <c r="H2" s="52"/>
+      <c r="I2" s="53"/>
     </row>
     <row r="3" spans="1:15" ht="25.5" x14ac:dyDescent="0.35">
       <c r="A3" s="15" t="s">
@@ -3363,7 +4187,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB1C31A0-C7DA-43B1-B6AB-AA5BBBECAE63}">
   <sheetPr>
     <tabColor rgb="FFB8FEC9"/>
@@ -3401,20 +4225,20 @@
       <c r="Q1" s="72"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A2" s="48" t="s">
+      <c r="A2" s="51" t="s">
         <v>109</v>
       </c>
-      <c r="B2" s="49"/>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="50"/>
-      <c r="F2" s="48" t="s">
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="53"/>
+      <c r="F2" s="51" t="s">
         <v>110</v>
       </c>
-      <c r="G2" s="49"/>
-      <c r="H2" s="49"/>
-      <c r="I2" s="49"/>
-      <c r="J2" s="50"/>
+      <c r="G2" s="52"/>
+      <c r="H2" s="52"/>
+      <c r="I2" s="52"/>
+      <c r="J2" s="53"/>
     </row>
     <row r="3" spans="1:17" ht="38.25" x14ac:dyDescent="0.35">
       <c r="A3" s="15" t="s">
@@ -3467,7 +4291,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD8FBBB6-BAD2-4D62-996E-E16FA2533A1A}">
   <sheetPr>
     <tabColor rgb="FFB8FEC9"/>
@@ -3501,11 +4325,11 @@
       <c r="O1" s="72"/>
     </row>
     <row r="2" spans="1:15" ht="36" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="48" t="s">
+      <c r="A2" s="51" t="s">
         <v>47</v>
       </c>
-      <c r="B2" s="50"/>
-      <c r="C2" s="52" t="s">
+      <c r="B2" s="53"/>
+      <c r="C2" s="58" t="s">
         <v>50</v>
       </c>
     </row>
@@ -3516,7 +4340,7 @@
       <c r="B3" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="C3" s="53"/>
+      <c r="C3" s="59"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -3527,100 +4351,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{773AF20E-74BF-463C-9F61-BFE009D6FACB}">
-  <sheetPr>
-    <tabColor rgb="FFB8FEC9"/>
-  </sheetPr>
-  <dimension ref="A1:O3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7109375" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="15.7109375" style="11"/>
-    <col min="2" max="2" width="15.7109375" style="1"/>
-    <col min="3" max="7" width="15.7109375" style="2"/>
-    <col min="8" max="8" width="15.7109375" style="14"/>
-    <col min="9" max="9" width="15.7109375" style="2"/>
-    <col min="10" max="10" width="15.7109375" style="12"/>
-    <col min="11" max="16384" width="15.7109375" style="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:15" s="20" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="72" t="s">
-        <v>51</v>
-      </c>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="D1" s="72"/>
-      <c r="E1" s="72"/>
-      <c r="F1" s="72"/>
-      <c r="G1" s="72"/>
-      <c r="H1" s="72"/>
-      <c r="I1" s="72"/>
-      <c r="J1" s="72"/>
-      <c r="K1" s="72"/>
-      <c r="L1" s="72"/>
-      <c r="M1" s="72"/>
-      <c r="N1" s="72"/>
-      <c r="O1" s="72"/>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A2" s="52" t="s">
-        <v>91</v>
-      </c>
-      <c r="B2" s="48" t="s">
-        <v>53</v>
-      </c>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="49"/>
-      <c r="G2" s="50"/>
-      <c r="H2" s="48" t="s">
-        <v>60</v>
-      </c>
-      <c r="I2" s="49"/>
-      <c r="J2" s="50"/>
-    </row>
-    <row r="3" spans="1:15" ht="51" x14ac:dyDescent="0.35">
-      <c r="A3" s="53"/>
-      <c r="B3" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="C3" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="D3" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="E3" s="15" t="s">
-        <v>57</v>
-      </c>
-      <c r="F3" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="G3" s="15" t="s">
-        <v>59</v>
-      </c>
-      <c r="H3" s="17" t="s">
-        <v>63</v>
-      </c>
-      <c r="I3" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="J3" s="16" t="s">
-        <v>61</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="A1:O1"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
exporte l'exigence de publication C2 dans le template excel
</commit_message>
<xml_diff>
--- a/impact/vsme/xlsx/VSME.xlsx
+++ b/impact/vsme/xlsx/VSME.xlsx
@@ -8,30 +8,32 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmonteiro-de-mac-adc\Desktop\ancien bureau\Fichier\CSRD\Tableau ESRS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F85F3BE4-E26B-4DE8-B69D-7530A0D7FF19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2578CB28-8C22-4A67-A7F3-50ADB1D46C11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" firstSheet="1" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="25440" windowHeight="15270" tabRatio="500" firstSheet="2" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="&gt;&gt;&gt; " sheetId="3" r:id="rId1"/>
     <sheet name="B1" sheetId="7" r:id="rId2"/>
     <sheet name="B2" sheetId="2" r:id="rId3"/>
     <sheet name="C1" sheetId="19" r:id="rId4"/>
-    <sheet name="B3" sheetId="18" r:id="rId5"/>
-    <sheet name="B4" sheetId="8" r:id="rId6"/>
-    <sheet name="B5" sheetId="17" r:id="rId7"/>
-    <sheet name="B6" sheetId="9" r:id="rId8"/>
-    <sheet name="B7" sheetId="10" r:id="rId9"/>
-    <sheet name="C4" sheetId="25" r:id="rId10"/>
-    <sheet name="B8" sheetId="15" r:id="rId11"/>
-    <sheet name="B9" sheetId="11" r:id="rId12"/>
-    <sheet name="B10" sheetId="16" r:id="rId13"/>
-    <sheet name="C5" sheetId="23" r:id="rId14"/>
-    <sheet name="C6" sheetId="21" r:id="rId15"/>
-    <sheet name="C7" sheetId="24" r:id="rId16"/>
-    <sheet name="B11" sheetId="14" r:id="rId17"/>
-    <sheet name="C8" sheetId="22" r:id="rId18"/>
-    <sheet name="C9" sheetId="20" r:id="rId19"/>
+    <sheet name="C2" sheetId="27" r:id="rId5"/>
+    <sheet name="B3" sheetId="18" r:id="rId6"/>
+    <sheet name="B4" sheetId="8" r:id="rId7"/>
+    <sheet name="B5" sheetId="17" r:id="rId8"/>
+    <sheet name="B6" sheetId="9" r:id="rId9"/>
+    <sheet name="B7" sheetId="10" r:id="rId10"/>
+    <sheet name="C3" sheetId="28" r:id="rId11"/>
+    <sheet name="C4" sheetId="25" r:id="rId12"/>
+    <sheet name="B8" sheetId="15" r:id="rId13"/>
+    <sheet name="B9" sheetId="11" r:id="rId14"/>
+    <sheet name="B10" sheetId="16" r:id="rId15"/>
+    <sheet name="C5" sheetId="23" r:id="rId16"/>
+    <sheet name="C6" sheetId="21" r:id="rId17"/>
+    <sheet name="C7" sheetId="24" r:id="rId18"/>
+    <sheet name="B11" sheetId="14" r:id="rId19"/>
+    <sheet name="C8" sheetId="22" r:id="rId20"/>
+    <sheet name="C9" sheetId="20" r:id="rId21"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -52,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="232">
   <si>
     <t/>
   </si>
@@ -426,9 +428,6 @@
     <t>Consommation d'électricité</t>
   </si>
   <si>
-    <t>Estimation des émissions brutes de gaz à effet de serre (GES)</t>
-  </si>
-  <si>
     <t>Scope 1</t>
   </si>
   <si>
@@ -631,6 +630,126 @@
   </si>
   <si>
     <t>N° du risque</t>
+  </si>
+  <si>
+    <t>Estimation des émissions brutes de gaz à effet de serre (GES) des scopes 1 et 2</t>
+  </si>
+  <si>
+    <t>Estimation des émissions brutes de gaz à effet de serre (GES) du scope 3</t>
+  </si>
+  <si>
+    <t>Biens et services achetés</t>
+  </si>
+  <si>
+    <t>Biens d'investissement</t>
+  </si>
+  <si>
+    <t>Activités relevant des secteurs des combustibles et de l'énergie</t>
+  </si>
+  <si>
+    <t>Transport et distribution en amont</t>
+  </si>
+  <si>
+    <t>Déchets produits lors de l'exploitation</t>
+  </si>
+  <si>
+    <t>Voyages d'affaires</t>
+  </si>
+  <si>
+    <t>Déplacements domicile-travail des salariés</t>
+  </si>
+  <si>
+    <t>Actifs loués en amont</t>
+  </si>
+  <si>
+    <t>Acheminement en aval</t>
+  </si>
+  <si>
+    <t>Transformation des produits vendus</t>
+  </si>
+  <si>
+    <t>Utilisation des produits vendus</t>
+  </si>
+  <si>
+    <t>Traitement en fin de vie des produits vendus</t>
+  </si>
+  <si>
+    <t>Actifs loués en aval</t>
+  </si>
+  <si>
+    <t>Franchises</t>
+  </si>
+  <si>
+    <t>Investissements</t>
+  </si>
+  <si>
+    <t>Émissions totales des GES du scope 3</t>
+  </si>
+  <si>
+    <t>Émissions totales des GES des scopes 1, 2 (basé sur la localisation) et 3</t>
+  </si>
+  <si>
+    <t>Cibles de réduction des émissions de GES des scopes 1 et 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Année de référence </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Année cible </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valeur de l'année de référence </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valeur de l'année cible </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réduction en pourcentage par rapport à l'année de référence </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Principales actions prévues </t>
+  </si>
+  <si>
+    <t>Plan de transition climatique</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> L'entreprise dispose-t-elle d'un plan de transition climatique ? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Description du plan de transition climatique </t>
+  </si>
+  <si>
+    <t>Contribution du plan de transition climatique à la réduction des émissions de GES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Année prévue d'adoption d'un plan de transition climatique </t>
+  </si>
+  <si>
+    <t>C3 - Cibles de réduction des émissions de GES et transition climatique</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 	Description des pratiques, politiques ou initiatives futures </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Description des cibles définies </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Niveau hiérarchique le plus élevé responsable de la mise en œuvre des politiques </t>
+  </si>
+  <si>
+    <t>Description des pratiques et politiques de durabilité</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2 - Description des pratiques, des politiques et des initiatives futures pour une transition vers une économie plus durable </t>
+  </si>
+  <si>
+    <t>Total scope 3</t>
+  </si>
+  <si>
+    <t>Total scopes 1, 2 et 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total </t>
   </si>
 </sst>
 </file>
@@ -730,7 +849,7 @@
       <name val="Marianne"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -791,6 +910,18 @@
         <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor rgb="FFFEE7FC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB8FEC9"/>
+        <bgColor rgb="FFE8EDFF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="27">
     <border>
@@ -1118,7 +1249,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="79">
+  <cellXfs count="96">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
@@ -1197,6 +1328,15 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1206,6 +1346,15 @@
     <xf numFmtId="0" fontId="11" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1221,24 +1370,6 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1289,6 +1420,57 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1813,6 +1995,410 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{773AF20E-74BF-463C-9F61-BFE009D6FACB}">
+  <sheetPr>
+    <tabColor rgb="FFB8FEC9"/>
+  </sheetPr>
+  <dimension ref="A1:O3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7109375" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="15.7109375" style="11"/>
+    <col min="2" max="2" width="15.7109375" style="1"/>
+    <col min="3" max="7" width="15.7109375" style="2"/>
+    <col min="8" max="8" width="15.7109375" style="14"/>
+    <col min="9" max="9" width="15.7109375" style="2"/>
+    <col min="10" max="10" width="15.7109375" style="12"/>
+    <col min="11" max="16384" width="15.7109375" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" s="20" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="72" t="s">
+        <v>51</v>
+      </c>
+      <c r="B1" s="72"/>
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
+      <c r="E1" s="72"/>
+      <c r="F1" s="72"/>
+      <c r="G1" s="72"/>
+      <c r="H1" s="72"/>
+      <c r="I1" s="72"/>
+      <c r="J1" s="72"/>
+      <c r="K1" s="72"/>
+      <c r="L1" s="72"/>
+      <c r="M1" s="72"/>
+      <c r="N1" s="72"/>
+      <c r="O1" s="72"/>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A2" s="58" t="s">
+        <v>91</v>
+      </c>
+      <c r="B2" s="51" t="s">
+        <v>53</v>
+      </c>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="53"/>
+      <c r="H2" s="51" t="s">
+        <v>60</v>
+      </c>
+      <c r="I2" s="52"/>
+      <c r="J2" s="53"/>
+    </row>
+    <row r="3" spans="1:15" ht="51" x14ac:dyDescent="0.35">
+      <c r="A3" s="59"/>
+      <c r="B3" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="D3" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="F3" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="G3" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="H3" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="I3" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="J3" s="16" t="s">
+        <v>61</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="A1:O1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{749A6938-FD3C-42AA-A2AB-FBC63AEF511E}">
+  <sheetPr>
+    <tabColor rgb="FFB8FEC9"/>
+  </sheetPr>
+  <dimension ref="A1:P21"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7109375" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="2" width="15.7109375" style="12"/>
+    <col min="3" max="6" width="15.7109375" style="82"/>
+    <col min="7" max="7" width="15.7109375" style="87"/>
+    <col min="8" max="11" width="15.7109375" style="82"/>
+    <col min="12" max="12" width="15.7109375" style="87"/>
+    <col min="13" max="15" width="15.7109375" style="93"/>
+    <col min="16" max="16" width="15.7109375" style="94"/>
+    <col min="17" max="16384" width="15.7109375" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" s="20" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="72" t="s">
+        <v>223</v>
+      </c>
+      <c r="B1" s="72"/>
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
+      <c r="E1" s="72"/>
+      <c r="F1" s="72"/>
+      <c r="G1" s="72"/>
+      <c r="H1" s="72"/>
+      <c r="I1" s="72"/>
+      <c r="J1" s="72"/>
+      <c r="K1" s="72"/>
+      <c r="L1" s="72"/>
+      <c r="M1" s="72"/>
+      <c r="N1" s="72"/>
+      <c r="O1" s="72"/>
+      <c r="P1" s="88"/>
+    </row>
+    <row r="2" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="58" t="s">
+        <v>212</v>
+      </c>
+      <c r="B2" s="58" t="s">
+        <v>213</v>
+      </c>
+      <c r="C2" s="83" t="s">
+        <v>211</v>
+      </c>
+      <c r="D2" s="84"/>
+      <c r="E2" s="84"/>
+      <c r="F2" s="84"/>
+      <c r="G2" s="85"/>
+      <c r="H2" s="51" t="s">
+        <v>193</v>
+      </c>
+      <c r="I2" s="52"/>
+      <c r="J2" s="52"/>
+      <c r="K2" s="52"/>
+      <c r="L2" s="53"/>
+      <c r="M2" s="83" t="s">
+        <v>218</v>
+      </c>
+      <c r="N2" s="84"/>
+      <c r="O2" s="84"/>
+      <c r="P2" s="85"/>
+    </row>
+    <row r="3" spans="1:16" ht="63.75" x14ac:dyDescent="0.35">
+      <c r="A3" s="59"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="86"/>
+      <c r="D3" s="18" t="s">
+        <v>214</v>
+      </c>
+      <c r="E3" s="18" t="s">
+        <v>215</v>
+      </c>
+      <c r="F3" s="18" t="s">
+        <v>216</v>
+      </c>
+      <c r="G3" s="16" t="s">
+        <v>217</v>
+      </c>
+      <c r="H3" s="18"/>
+      <c r="I3" s="18" t="s">
+        <v>214</v>
+      </c>
+      <c r="J3" s="18" t="s">
+        <v>215</v>
+      </c>
+      <c r="K3" s="15" t="s">
+        <v>216</v>
+      </c>
+      <c r="L3" s="16" t="s">
+        <v>217</v>
+      </c>
+      <c r="M3" s="18" t="s">
+        <v>219</v>
+      </c>
+      <c r="N3" s="18" t="s">
+        <v>220</v>
+      </c>
+      <c r="O3" s="18" t="s">
+        <v>221</v>
+      </c>
+      <c r="P3" s="16" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="C4" s="18" t="s">
+        <v>124</v>
+      </c>
+      <c r="D4" s="86"/>
+      <c r="E4" s="86"/>
+      <c r="F4" s="86"/>
+      <c r="G4" s="16"/>
+      <c r="H4" s="80" t="s">
+        <v>194</v>
+      </c>
+      <c r="I4" s="89"/>
+      <c r="J4" s="86"/>
+      <c r="K4" s="86"/>
+      <c r="L4" s="90"/>
+      <c r="M4" s="91"/>
+      <c r="N4" s="91"/>
+      <c r="O4" s="91"/>
+      <c r="P4" s="92"/>
+    </row>
+    <row r="5" spans="1:16" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="C5" s="18" t="s">
+        <v>125</v>
+      </c>
+      <c r="D5" s="86"/>
+      <c r="E5" s="86"/>
+      <c r="F5" s="86"/>
+      <c r="G5" s="16"/>
+      <c r="H5" s="80" t="s">
+        <v>195</v>
+      </c>
+      <c r="I5" s="89"/>
+      <c r="J5" s="86"/>
+      <c r="K5" s="86"/>
+      <c r="L5" s="90"/>
+    </row>
+    <row r="6" spans="1:16" ht="51" x14ac:dyDescent="0.35">
+      <c r="C6" s="18" t="s">
+        <v>231</v>
+      </c>
+      <c r="D6" s="86"/>
+      <c r="E6" s="86"/>
+      <c r="F6" s="86"/>
+      <c r="G6" s="16"/>
+      <c r="H6" s="80" t="s">
+        <v>196</v>
+      </c>
+      <c r="I6" s="86"/>
+      <c r="J6" s="86"/>
+      <c r="K6" s="86"/>
+      <c r="L6" s="90"/>
+    </row>
+    <row r="7" spans="1:16" ht="38.25" x14ac:dyDescent="0.35">
+      <c r="C7" s="18"/>
+      <c r="D7" s="86"/>
+      <c r="E7" s="86"/>
+      <c r="F7" s="86"/>
+      <c r="G7" s="16"/>
+      <c r="H7" s="80" t="s">
+        <v>197</v>
+      </c>
+      <c r="I7" s="86"/>
+      <c r="J7" s="86"/>
+      <c r="K7" s="86"/>
+      <c r="L7" s="90"/>
+    </row>
+    <row r="8" spans="1:16" ht="38.25" x14ac:dyDescent="0.35">
+      <c r="H8" s="80" t="s">
+        <v>198</v>
+      </c>
+      <c r="I8" s="86"/>
+      <c r="J8" s="86"/>
+      <c r="K8" s="86"/>
+      <c r="L8" s="95"/>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="H9" s="80" t="s">
+        <v>199</v>
+      </c>
+      <c r="I9" s="86"/>
+      <c r="J9" s="86"/>
+      <c r="K9" s="86"/>
+      <c r="L9" s="95"/>
+    </row>
+    <row r="10" spans="1:16" ht="38.25" x14ac:dyDescent="0.35">
+      <c r="H10" s="80" t="s">
+        <v>200</v>
+      </c>
+      <c r="I10" s="86"/>
+      <c r="J10" s="86"/>
+      <c r="K10" s="86"/>
+      <c r="L10" s="95"/>
+    </row>
+    <row r="11" spans="1:16" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="H11" s="80" t="s">
+        <v>201</v>
+      </c>
+      <c r="I11" s="86"/>
+      <c r="J11" s="86"/>
+      <c r="K11" s="86"/>
+      <c r="L11" s="95"/>
+    </row>
+    <row r="12" spans="1:16" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="H12" s="80" t="s">
+        <v>202</v>
+      </c>
+      <c r="I12" s="86"/>
+      <c r="J12" s="86"/>
+      <c r="K12" s="86"/>
+      <c r="L12" s="95"/>
+    </row>
+    <row r="13" spans="1:16" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="H13" s="80" t="s">
+        <v>203</v>
+      </c>
+      <c r="I13" s="86"/>
+      <c r="J13" s="86"/>
+      <c r="K13" s="86"/>
+      <c r="L13" s="95"/>
+    </row>
+    <row r="14" spans="1:16" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="H14" s="80" t="s">
+        <v>204</v>
+      </c>
+      <c r="I14" s="86"/>
+      <c r="J14" s="86"/>
+      <c r="K14" s="86"/>
+      <c r="L14" s="95"/>
+    </row>
+    <row r="15" spans="1:16" ht="38.25" x14ac:dyDescent="0.35">
+      <c r="H15" s="80" t="s">
+        <v>205</v>
+      </c>
+      <c r="I15" s="86"/>
+      <c r="J15" s="86"/>
+      <c r="K15" s="86"/>
+      <c r="L15" s="95"/>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="H16" s="80" t="s">
+        <v>206</v>
+      </c>
+      <c r="I16" s="86"/>
+      <c r="J16" s="86"/>
+      <c r="K16" s="86"/>
+      <c r="L16" s="95"/>
+    </row>
+    <row r="17" spans="8:12" x14ac:dyDescent="0.35">
+      <c r="H17" s="80" t="s">
+        <v>207</v>
+      </c>
+      <c r="I17" s="86"/>
+      <c r="J17" s="86"/>
+      <c r="K17" s="86"/>
+      <c r="L17" s="95"/>
+    </row>
+    <row r="18" spans="8:12" x14ac:dyDescent="0.35">
+      <c r="H18" s="80" t="s">
+        <v>208</v>
+      </c>
+      <c r="I18" s="86"/>
+      <c r="J18" s="86"/>
+      <c r="K18" s="86"/>
+      <c r="L18" s="95"/>
+    </row>
+    <row r="19" spans="8:12" x14ac:dyDescent="0.35">
+      <c r="H19" s="80" t="s">
+        <v>229</v>
+      </c>
+      <c r="I19" s="89"/>
+      <c r="J19" s="89"/>
+      <c r="K19" s="89"/>
+      <c r="L19" s="90"/>
+    </row>
+    <row r="20" spans="8:12" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="H20" s="80" t="s">
+        <v>230</v>
+      </c>
+      <c r="I20" s="89"/>
+      <c r="J20" s="89"/>
+      <c r="K20" s="89"/>
+      <c r="L20" s="90"/>
+    </row>
+    <row r="21" spans="8:12" x14ac:dyDescent="0.35">
+      <c r="H21" s="81"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:G2"/>
+    <mergeCell ref="H2:L2"/>
+    <mergeCell ref="M2:P2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AD57197-9ADC-43C0-B70E-801EE1BD86F4}">
   <sheetPr>
     <tabColor rgb="FFB8FEC9"/>
@@ -1830,7 +2416,7 @@
   <sheetData>
     <row r="1" spans="1:16" s="20" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="72" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B1" s="72"/>
       <c r="C1" s="72"/>
@@ -1849,47 +2435,47 @@
       <c r="P1" s="72"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A2" s="48" t="s">
-        <v>182</v>
-      </c>
-      <c r="B2" s="49"/>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="50"/>
-      <c r="F2" s="48" t="s">
-        <v>187</v>
-      </c>
-      <c r="G2" s="49"/>
-      <c r="H2" s="49"/>
-      <c r="I2" s="50"/>
+      <c r="A2" s="51" t="s">
+        <v>181</v>
+      </c>
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="53"/>
+      <c r="F2" s="51" t="s">
+        <v>186</v>
+      </c>
+      <c r="G2" s="52"/>
+      <c r="H2" s="52"/>
+      <c r="I2" s="53"/>
     </row>
     <row r="3" spans="1:16" ht="38.25" x14ac:dyDescent="0.35">
       <c r="A3" s="15" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B3" s="15" t="s">
+        <v>182</v>
+      </c>
+      <c r="C3" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="D3" s="15" t="s">
         <v>184</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="E3" s="15" t="s">
         <v>185</v>
       </c>
-      <c r="E3" s="15" t="s">
-        <v>186</v>
-      </c>
       <c r="F3" s="17" t="s">
+        <v>187</v>
+      </c>
+      <c r="G3" s="15" t="s">
         <v>188</v>
       </c>
-      <c r="G3" s="15" t="s">
+      <c r="H3" s="15" t="s">
         <v>189</v>
       </c>
-      <c r="H3" s="15" t="s">
-        <v>190</v>
-      </c>
       <c r="I3" s="16" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
   </sheetData>
@@ -1914,7 +2500,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAD01D35-7DA1-4A19-9314-8C6D84659D0B}">
   <sheetPr>
     <tabColor rgb="FFFEE7FC"/>
@@ -1952,21 +2538,21 @@
       <c r="O1" s="73"/>
     </row>
     <row r="2" spans="1:15" ht="39" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="48" t="s">
+      <c r="A2" s="51" t="s">
         <v>80</v>
       </c>
-      <c r="B2" s="50"/>
-      <c r="C2" s="48" t="s">
+      <c r="B2" s="53"/>
+      <c r="C2" s="51" t="s">
         <v>83</v>
       </c>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="50"/>
-      <c r="G2" s="48" t="s">
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="53"/>
+      <c r="G2" s="51" t="s">
         <v>86</v>
       </c>
-      <c r="H2" s="50"/>
-      <c r="I2" s="52" t="s">
+      <c r="H2" s="53"/>
+      <c r="I2" s="58" t="s">
         <v>88</v>
       </c>
     </row>
@@ -1995,7 +2581,7 @@
       <c r="H3" s="15" t="s">
         <v>87</v>
       </c>
-      <c r="I3" s="53"/>
+      <c r="I3" s="59"/>
     </row>
     <row r="12" spans="1:15" ht="72.75" x14ac:dyDescent="1.25">
       <c r="E12" s="22"/>
@@ -2013,7 +2599,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D36321D-28CF-4197-97E4-15B03B8FE828}">
   <sheetPr>
     <tabColor rgb="FFFEE7FC"/>
@@ -2048,11 +2634,11 @@
       <c r="O1" s="73"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A2" s="48" t="s">
+      <c r="A2" s="51" t="s">
         <v>64</v>
       </c>
-      <c r="B2" s="50"/>
-      <c r="C2" s="52" t="s">
+      <c r="B2" s="53"/>
+      <c r="C2" s="58" t="s">
         <v>67</v>
       </c>
     </row>
@@ -2063,7 +2649,7 @@
       <c r="B3" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="C3" s="53"/>
+      <c r="C3" s="59"/>
     </row>
     <row r="12" spans="1:15" ht="72.75" x14ac:dyDescent="1.25">
       <c r="E12" s="22"/>
@@ -2079,7 +2665,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8767C8CD-15EF-412F-8BDE-09F42DF51D25}">
   <sheetPr>
     <tabColor rgb="FFFEE7FC"/>
@@ -2118,26 +2704,26 @@
       <c r="O1" s="73"/>
     </row>
     <row r="2" spans="1:15" ht="54.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="58" t="s">
         <v>93</v>
       </c>
-      <c r="B2" s="48" t="s">
+      <c r="B2" s="51" t="s">
         <v>94</v>
       </c>
-      <c r="C2" s="49"/>
-      <c r="D2" s="50"/>
-      <c r="E2" s="48" t="s">
+      <c r="C2" s="52"/>
+      <c r="D2" s="53"/>
+      <c r="E2" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="F2" s="50"/>
-      <c r="G2" s="48" t="s">
+      <c r="F2" s="53"/>
+      <c r="G2" s="51" t="s">
         <v>105</v>
       </c>
-      <c r="H2" s="49"/>
-      <c r="I2" s="50"/>
+      <c r="H2" s="52"/>
+      <c r="I2" s="53"/>
     </row>
     <row r="3" spans="1:15" ht="97.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="53"/>
+      <c r="A3" s="59"/>
       <c r="B3" s="15" t="s">
         <v>95</v>
       </c>
@@ -2202,7 +2788,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93F62B1A-C319-4701-AD63-7BD53F525CF6}">
   <sheetPr>
     <tabColor rgb="FFFEE7FC"/>
@@ -2219,7 +2805,7 @@
   <sheetData>
     <row r="1" spans="1:15" s="21" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="73" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B1" s="73"/>
       <c r="C1" s="73"/>
@@ -2237,31 +2823,31 @@
       <c r="O1" s="73"/>
     </row>
     <row r="2" spans="1:15" ht="53.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="48" t="s">
-        <v>168</v>
-      </c>
-      <c r="B2" s="49"/>
-      <c r="C2" s="50"/>
-      <c r="D2" s="48" t="s">
-        <v>171</v>
-      </c>
-      <c r="E2" s="50"/>
+      <c r="A2" s="51" t="s">
+        <v>167</v>
+      </c>
+      <c r="B2" s="52"/>
+      <c r="C2" s="53"/>
+      <c r="D2" s="51" t="s">
+        <v>170</v>
+      </c>
+      <c r="E2" s="53"/>
     </row>
     <row r="3" spans="1:15" ht="114.75" x14ac:dyDescent="0.35">
       <c r="A3" s="15" t="s">
+        <v>165</v>
+      </c>
+      <c r="B3" s="15" t="s">
         <v>166</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="C3" s="16" t="s">
         <v>167</v>
       </c>
-      <c r="C3" s="16" t="s">
+      <c r="D3" s="15" t="s">
         <v>168</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="E3" s="16" t="s">
         <v>169</v>
-      </c>
-      <c r="E3" s="16" t="s">
-        <v>170</v>
       </c>
     </row>
   </sheetData>
@@ -2283,7 +2869,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C465E33-2082-481B-93DA-B52297D05DCF}">
   <sheetPr>
     <tabColor rgb="FFFEE7FC"/>
@@ -2300,7 +2886,7 @@
   <sheetData>
     <row r="1" spans="1:19" s="21" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="73" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B1" s="73"/>
       <c r="C1" s="73"/>
@@ -2322,38 +2908,38 @@
       <c r="S1" s="73"/>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A2" s="48" t="s">
-        <v>147</v>
-      </c>
-      <c r="B2" s="49"/>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="50"/>
-      <c r="G2" s="52" t="s">
-        <v>154</v>
+      <c r="A2" s="51" t="s">
+        <v>146</v>
+      </c>
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="53"/>
+      <c r="G2" s="58" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="3" spans="1:19" ht="89.25" x14ac:dyDescent="0.35">
       <c r="A3" s="15" t="s">
+        <v>147</v>
+      </c>
+      <c r="B3" s="15" t="s">
         <v>148</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="C3" s="15" t="s">
         <v>149</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="D3" s="15" t="s">
         <v>150</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="E3" s="15" t="s">
         <v>151</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="F3" s="16" t="s">
         <v>152</v>
       </c>
-      <c r="F3" s="16" t="s">
-        <v>153</v>
-      </c>
-      <c r="G3" s="53"/>
+      <c r="G3" s="59"/>
     </row>
     <row r="12" spans="1:19" ht="72.75" x14ac:dyDescent="1.25">
       <c r="I12" s="22"/>
@@ -2377,7 +2963,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81D0B7EC-F23C-48FB-98BB-3AFB974D2AA9}">
   <sheetPr>
     <tabColor rgb="FFFEE7FC"/>
@@ -2394,7 +2980,7 @@
   <sheetData>
     <row r="1" spans="1:19" s="21" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="73" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B1" s="73"/>
       <c r="C1" s="73"/>
@@ -2416,38 +3002,38 @@
       <c r="S1" s="73"/>
     </row>
     <row r="2" spans="1:19" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="48" t="s">
-        <v>173</v>
-      </c>
-      <c r="B2" s="49"/>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="50"/>
-      <c r="G2" s="52" t="s">
-        <v>180</v>
+      <c r="A2" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="53"/>
+      <c r="G2" s="58" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="3" spans="1:19" ht="127.5" x14ac:dyDescent="0.35">
       <c r="A3" s="15" t="s">
+        <v>173</v>
+      </c>
+      <c r="B3" s="15" t="s">
         <v>174</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="C3" s="15" t="s">
         <v>175</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="D3" s="15" t="s">
         <v>176</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="E3" s="15" t="s">
+        <v>178</v>
+      </c>
+      <c r="F3" s="16" t="s">
         <v>177</v>
       </c>
-      <c r="E3" s="15" t="s">
-        <v>179</v>
-      </c>
-      <c r="F3" s="16" t="s">
-        <v>178</v>
-      </c>
-      <c r="G3" s="53"/>
+      <c r="G3" s="59"/>
     </row>
     <row r="12" spans="1:19" ht="72.75" x14ac:dyDescent="1.25">
       <c r="I12" s="22"/>
@@ -2471,7 +3057,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E35E0E35-59BE-44D0-9FD8-FA3A89A617DC}">
   <sheetPr>
     <tabColor rgb="FFE8EDFF"/>
@@ -2521,140 +3107,6 @@
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="A1:O1"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBA71AC8-3159-49A5-B6FC-4FA1DF3F7E26}">
-  <sheetPr>
-    <tabColor rgb="FFE8EDFF"/>
-  </sheetPr>
-  <dimension ref="A1:L3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7109375" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="15.7109375" style="1"/>
-    <col min="2" max="6" width="15.7109375" style="2"/>
-    <col min="7" max="7" width="15.7109375" style="12"/>
-    <col min="8" max="8" width="18.140625" style="12" customWidth="1"/>
-    <col min="9" max="16384" width="15.7109375" style="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:12" s="23" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="78" t="s">
-        <v>164</v>
-      </c>
-      <c r="B1" s="78"/>
-      <c r="C1" s="78"/>
-      <c r="D1" s="78"/>
-      <c r="E1" s="78"/>
-      <c r="F1" s="78"/>
-      <c r="G1" s="78"/>
-      <c r="H1" s="78"/>
-      <c r="I1" s="78"/>
-      <c r="J1" s="78"/>
-      <c r="K1" s="78"/>
-      <c r="L1" s="78"/>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A2" s="48" t="s">
-        <v>163</v>
-      </c>
-      <c r="B2" s="49"/>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="49"/>
-      <c r="G2" s="50"/>
-      <c r="H2" s="51" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" ht="63.75" x14ac:dyDescent="0.35">
-      <c r="A3" s="15" t="s">
-        <v>156</v>
-      </c>
-      <c r="B3" s="15" t="s">
-        <v>157</v>
-      </c>
-      <c r="C3" s="15" t="s">
-        <v>158</v>
-      </c>
-      <c r="D3" s="15" t="s">
-        <v>159</v>
-      </c>
-      <c r="E3" s="15" t="s">
-        <v>160</v>
-      </c>
-      <c r="F3" s="15" t="s">
-        <v>165</v>
-      </c>
-      <c r="G3" s="16" t="s">
-        <v>161</v>
-      </c>
-      <c r="H3" s="50"/>
-    </row>
-  </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="H2:H3"/>
-  </mergeCells>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H4:H6" xr:uid="{B7229605-3AFC-4A61-911C-7A7A7D3FA5D1}">
-      <formula1>"Oui,Non"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDD13986-9BC7-428C-BEF7-5E284E22308C}">
-  <sheetPr>
-    <tabColor rgb="FFE8EDFF"/>
-  </sheetPr>
-  <dimension ref="A1:N3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="22.28515625" style="11" customWidth="1"/>
-    <col min="2" max="4" width="11.42578125" style="2" customWidth="1"/>
-    <col min="5" max="16384" width="11.42578125" style="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:14" s="23" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="78" t="s">
-        <v>145</v>
-      </c>
-      <c r="B1" s="78"/>
-      <c r="C1" s="78"/>
-      <c r="D1" s="78"/>
-      <c r="E1" s="78"/>
-      <c r="F1" s="78"/>
-      <c r="G1" s="78"/>
-      <c r="H1" s="78"/>
-      <c r="I1" s="78"/>
-      <c r="J1" s="78"/>
-      <c r="K1" s="78"/>
-      <c r="L1" s="78"/>
-      <c r="M1" s="78"/>
-      <c r="N1" s="78"/>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A2" s="74" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" ht="55.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="75"/>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:N1"/>
-    <mergeCell ref="A2:A3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -2688,86 +3140,86 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" s="10" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="56" t="s">
+      <c r="A1" s="48" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
-      <c r="K1" s="56"/>
-      <c r="L1" s="56"/>
-      <c r="M1" s="56"/>
-      <c r="N1" s="56"/>
-      <c r="O1" s="56"/>
-      <c r="P1" s="56"/>
-      <c r="Q1" s="56"/>
-      <c r="R1" s="56"/>
-      <c r="S1" s="56"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
+      <c r="K1" s="48"/>
+      <c r="L1" s="48"/>
+      <c r="M1" s="48"/>
+      <c r="N1" s="48"/>
+      <c r="O1" s="48"/>
+      <c r="P1" s="48"/>
+      <c r="Q1" s="48"/>
+      <c r="R1" s="48"/>
+      <c r="S1" s="48"/>
     </row>
     <row r="2" spans="1:28" s="19" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="51" t="s">
+      <c r="A2" s="57" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="52" t="s">
+      <c r="B2" s="58" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="52" t="s">
+      <c r="C2" s="58" t="s">
         <v>19</v>
       </c>
-      <c r="D2" s="48" t="s">
+      <c r="D2" s="51" t="s">
         <v>20</v>
       </c>
-      <c r="E2" s="49"/>
-      <c r="F2" s="49"/>
-      <c r="G2" s="49"/>
-      <c r="H2" s="50"/>
-      <c r="I2" s="57" t="s">
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52"/>
+      <c r="H2" s="53"/>
+      <c r="I2" s="49" t="s">
         <v>31</v>
       </c>
-      <c r="J2" s="58"/>
-      <c r="K2" s="54" t="s">
+      <c r="J2" s="50"/>
+      <c r="K2" s="60" t="s">
         <v>90</v>
       </c>
-      <c r="L2" s="52" t="s">
+      <c r="L2" s="58" t="s">
         <v>21</v>
       </c>
-      <c r="M2" s="54" t="s">
+      <c r="M2" s="60" t="s">
         <v>89</v>
       </c>
-      <c r="N2" s="57" t="s">
+      <c r="N2" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="O2" s="58"/>
-      <c r="P2" s="54" t="s">
+      <c r="O2" s="50"/>
+      <c r="P2" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="Q2" s="59" t="s">
+      <c r="Q2" s="54" t="s">
         <v>24</v>
       </c>
-      <c r="R2" s="60"/>
-      <c r="S2" s="60"/>
-      <c r="T2" s="60"/>
-      <c r="U2" s="60"/>
-      <c r="V2" s="60"/>
-      <c r="W2" s="61"/>
-      <c r="X2" s="48" t="s">
+      <c r="R2" s="55"/>
+      <c r="S2" s="55"/>
+      <c r="T2" s="55"/>
+      <c r="U2" s="55"/>
+      <c r="V2" s="55"/>
+      <c r="W2" s="56"/>
+      <c r="X2" s="51" t="s">
         <v>25</v>
       </c>
-      <c r="Y2" s="49"/>
-      <c r="Z2" s="49"/>
-      <c r="AA2" s="49"/>
-      <c r="AB2" s="50"/>
+      <c r="Y2" s="52"/>
+      <c r="Z2" s="52"/>
+      <c r="AA2" s="52"/>
+      <c r="AB2" s="53"/>
     </row>
     <row r="3" spans="1:28" ht="38.25" x14ac:dyDescent="0.35">
-      <c r="A3" s="50"/>
-      <c r="B3" s="53"/>
-      <c r="C3" s="53"/>
+      <c r="A3" s="53"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="59"/>
       <c r="D3" s="15" t="s">
         <v>26</v>
       </c>
@@ -2789,16 +3241,16 @@
       <c r="J3" s="46" t="s">
         <v>73</v>
       </c>
-      <c r="K3" s="55"/>
-      <c r="L3" s="53"/>
-      <c r="M3" s="55"/>
+      <c r="K3" s="61"/>
+      <c r="L3" s="59"/>
+      <c r="M3" s="61"/>
       <c r="N3" s="45" t="s">
         <v>74</v>
       </c>
       <c r="O3" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="P3" s="55"/>
+      <c r="P3" s="61"/>
       <c r="Q3" s="17" t="s">
         <v>72</v>
       </c>
@@ -2838,11 +3290,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="A1:S1"/>
-    <mergeCell ref="N2:O2"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="Q2:W2"/>
     <mergeCell ref="X2:AB2"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="B2:B3"/>
@@ -2851,9 +3298,148 @@
     <mergeCell ref="M2:M3"/>
     <mergeCell ref="P2:P3"/>
     <mergeCell ref="K2:K3"/>
+    <mergeCell ref="A1:S1"/>
+    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="Q2:W2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBA71AC8-3159-49A5-B6FC-4FA1DF3F7E26}">
+  <sheetPr>
+    <tabColor rgb="FFE8EDFF"/>
+  </sheetPr>
+  <dimension ref="A1:L3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7109375" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="15.7109375" style="1"/>
+    <col min="2" max="6" width="15.7109375" style="2"/>
+    <col min="7" max="7" width="15.7109375" style="12"/>
+    <col min="8" max="8" width="18.140625" style="12" customWidth="1"/>
+    <col min="9" max="16384" width="15.7109375" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" s="23" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="78" t="s">
+        <v>163</v>
+      </c>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
+      <c r="F1" s="78"/>
+      <c r="G1" s="78"/>
+      <c r="H1" s="78"/>
+      <c r="I1" s="78"/>
+      <c r="J1" s="78"/>
+      <c r="K1" s="78"/>
+      <c r="L1" s="78"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A2" s="51" t="s">
+        <v>162</v>
+      </c>
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="53"/>
+      <c r="H2" s="57" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="63.75" x14ac:dyDescent="0.35">
+      <c r="A3" s="15" t="s">
+        <v>155</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>156</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>157</v>
+      </c>
+      <c r="D3" s="15" t="s">
+        <v>158</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>159</v>
+      </c>
+      <c r="F3" s="15" t="s">
+        <v>164</v>
+      </c>
+      <c r="G3" s="16" t="s">
+        <v>160</v>
+      </c>
+      <c r="H3" s="53"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="H2:H3"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H4:H6" xr:uid="{B7229605-3AFC-4A61-911C-7A7A7D3FA5D1}">
+      <formula1>"Oui,Non"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDD13986-9BC7-428C-BEF7-5E284E22308C}">
+  <sheetPr>
+    <tabColor rgb="FFE8EDFF"/>
+  </sheetPr>
+  <dimension ref="A1:N3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="22.28515625" style="11" customWidth="1"/>
+    <col min="2" max="4" width="11.42578125" style="2" customWidth="1"/>
+    <col min="5" max="16384" width="11.42578125" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" s="23" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="78" t="s">
+        <v>144</v>
+      </c>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
+      <c r="F1" s="78"/>
+      <c r="G1" s="78"/>
+      <c r="H1" s="78"/>
+      <c r="I1" s="78"/>
+      <c r="J1" s="78"/>
+      <c r="K1" s="78"/>
+      <c r="L1" s="78"/>
+      <c r="M1" s="78"/>
+      <c r="N1" s="78"/>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A2" s="74" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" ht="55.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="75"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A2:A3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
@@ -2876,29 +3462,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" s="10" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="56" t="s">
+      <c r="A1" s="48" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
-      <c r="K1" s="56"/>
-      <c r="L1" s="56"/>
-      <c r="M1" s="56"/>
-      <c r="N1" s="56"/>
-      <c r="O1" s="56"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
+      <c r="K1" s="48"/>
+      <c r="L1" s="48"/>
+      <c r="M1" s="48"/>
+      <c r="N1" s="48"/>
+      <c r="O1" s="48"/>
     </row>
     <row r="2" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="62" t="s">
         <v>75</v>
       </c>
-      <c r="B2" s="52" t="s">
+      <c r="B2" s="58" t="s">
         <v>76</v>
       </c>
       <c r="C2" s="64" t="s">
@@ -2913,12 +3499,12 @@
     </row>
     <row r="3" spans="1:15" ht="41.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="63"/>
-      <c r="B3" s="53"/>
-      <c r="C3" s="49"/>
-      <c r="D3" s="48"/>
-      <c r="E3" s="49"/>
-      <c r="F3" s="49"/>
-      <c r="G3" s="50"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="52"/>
+      <c r="D3" s="51"/>
+      <c r="E3" s="52"/>
+      <c r="F3" s="52"/>
+      <c r="G3" s="53"/>
     </row>
     <row r="4" spans="1:15" ht="48" thickBot="1" x14ac:dyDescent="0.4">
       <c r="E4" s="25" t="s">
@@ -3044,41 +3630,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" s="10" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="56" t="s">
-        <v>144</v>
-      </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
-      <c r="K1" s="56"/>
-      <c r="L1" s="56"/>
-      <c r="M1" s="56"/>
+      <c r="A1" s="48" t="s">
+        <v>143</v>
+      </c>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
+      <c r="K1" s="48"/>
+      <c r="L1" s="48"/>
+      <c r="M1" s="48"/>
     </row>
     <row r="2" spans="1:13" s="19" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="51" t="s">
+      <c r="A2" s="57" t="s">
+        <v>139</v>
+      </c>
+      <c r="B2" s="58" t="s">
         <v>140</v>
       </c>
-      <c r="B2" s="52" t="s">
+      <c r="C2" s="58" t="s">
         <v>141</v>
       </c>
-      <c r="C2" s="52" t="s">
+      <c r="D2" s="58" t="s">
         <v>142</v>
       </c>
-      <c r="D2" s="52" t="s">
-        <v>143</v>
-      </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A3" s="50"/>
-      <c r="B3" s="53"/>
-      <c r="C3" s="53"/>
-      <c r="D3" s="53"/>
+      <c r="A3" s="53"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -3094,11 +3680,158 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3A89080-2C89-4599-81BF-8F339FE8E625}">
+  <sheetPr>
+    <tabColor rgb="FFFFEDC3"/>
+  </sheetPr>
+  <dimension ref="A1:M14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7109375" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="38.28515625" style="14" customWidth="1"/>
+    <col min="2" max="2" width="23.7109375" style="2" customWidth="1"/>
+    <col min="3" max="3" width="21.85546875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="20.42578125" style="12" customWidth="1"/>
+    <col min="5" max="16384" width="15.7109375" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" s="10" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="48" t="s">
+        <v>228</v>
+      </c>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
+      <c r="K1" s="48"/>
+      <c r="L1" s="48"/>
+      <c r="M1" s="48"/>
+    </row>
+    <row r="2" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="65" t="s">
+        <v>227</v>
+      </c>
+      <c r="B2" s="66"/>
+      <c r="C2" s="66"/>
+      <c r="D2" s="67"/>
+    </row>
+    <row r="3" spans="1:13" ht="41.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="51"/>
+      <c r="B3" s="52"/>
+      <c r="C3" s="52"/>
+      <c r="D3" s="53"/>
+    </row>
+    <row r="4" spans="1:13" ht="79.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B4" s="25" t="s">
+        <v>224</v>
+      </c>
+      <c r="C4" s="26" t="s">
+        <v>225</v>
+      </c>
+      <c r="D4" s="27" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A5" s="28" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="29"/>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A6" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="29"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A7" s="31" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="9"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="29"/>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A8" s="31" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="9"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="29"/>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A9" s="31" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="9"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="29"/>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A10" s="32" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="9"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="29"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A11" s="32" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="9"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="29"/>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A12" s="32" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="9"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="29"/>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A13" s="32" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="9"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="29"/>
+    </row>
+    <row r="14" spans="1:13" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="33" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="34"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:D3"/>
+    <mergeCell ref="A1:M1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C0E4342-D345-4F6D-8348-EF5BA58D69DD}">
   <sheetPr>
     <tabColor rgb="FFB8FEC9"/>
   </sheetPr>
-  <dimension ref="A1:U4"/>
+  <dimension ref="A1:AL4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="15.7109375" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="15.7109375" style="1"/>
@@ -3113,10 +3846,13 @@
     <col min="18" max="19" width="15.7109375" style="1"/>
     <col min="20" max="20" width="15.7109375" style="11"/>
     <col min="21" max="21" width="15.7109375" style="12"/>
-    <col min="22" max="16384" width="15.7109375" style="2"/>
+    <col min="22" max="36" width="15.7109375" style="1"/>
+    <col min="37" max="37" width="15.7109375" style="24"/>
+    <col min="38" max="38" width="15.7109375" style="12"/>
+    <col min="39" max="16384" width="15.7109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" s="20" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:38" s="20" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="72" t="s">
         <v>119</v>
       </c>
@@ -3136,15 +3872,32 @@
       <c r="S1" s="44"/>
       <c r="T1" s="44"/>
       <c r="U1" s="44"/>
-    </row>
-    <row r="2" spans="1:21" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="49" t="s">
+      <c r="V1" s="44"/>
+      <c r="W1" s="44"/>
+      <c r="X1" s="44"/>
+      <c r="Y1" s="44"/>
+      <c r="Z1" s="44"/>
+      <c r="AA1" s="44"/>
+      <c r="AB1" s="44"/>
+      <c r="AC1" s="44"/>
+      <c r="AD1" s="44"/>
+      <c r="AE1" s="44"/>
+      <c r="AF1" s="44"/>
+      <c r="AG1" s="44"/>
+      <c r="AH1" s="44"/>
+      <c r="AI1" s="44"/>
+      <c r="AJ1" s="44"/>
+      <c r="AK1" s="44"/>
+      <c r="AL1" s="44"/>
+    </row>
+    <row r="2" spans="1:38" ht="35.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="52" t="s">
         <v>123</v>
       </c>
-      <c r="B2" s="49"/>
-      <c r="C2" s="50"/>
+      <c r="B2" s="52"/>
+      <c r="C2" s="53"/>
       <c r="D2" s="69" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E2" s="70"/>
       <c r="F2" s="70"/>
@@ -3159,14 +3912,33 @@
       <c r="O2" s="70"/>
       <c r="P2" s="70"/>
       <c r="Q2" s="71"/>
-      <c r="R2" s="49" t="s">
-        <v>124</v>
-      </c>
-      <c r="S2" s="49"/>
-      <c r="T2" s="49"/>
-      <c r="U2" s="50"/>
-    </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="R2" s="52" t="s">
+        <v>192</v>
+      </c>
+      <c r="S2" s="52"/>
+      <c r="T2" s="52"/>
+      <c r="U2" s="53"/>
+      <c r="V2" s="52" t="s">
+        <v>193</v>
+      </c>
+      <c r="W2" s="52"/>
+      <c r="X2" s="52"/>
+      <c r="Y2" s="52"/>
+      <c r="Z2" s="52"/>
+      <c r="AA2" s="52"/>
+      <c r="AB2" s="52"/>
+      <c r="AC2" s="52"/>
+      <c r="AD2" s="52"/>
+      <c r="AE2" s="52"/>
+      <c r="AF2" s="52"/>
+      <c r="AG2" s="52"/>
+      <c r="AH2" s="52"/>
+      <c r="AI2" s="52"/>
+      <c r="AJ2" s="52"/>
+      <c r="AK2" s="52"/>
+      <c r="AL2" s="53"/>
+    </row>
+    <row r="3" spans="1:38" ht="51" x14ac:dyDescent="0.35">
       <c r="A3" s="15" t="s">
         <v>120</v>
       </c>
@@ -3177,7 +3949,7 @@
         <v>122</v>
       </c>
       <c r="D3" s="68" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E3" s="68"/>
       <c r="F3" s="68"/>
@@ -3187,61 +3959,112 @@
       <c r="J3" s="68"/>
       <c r="K3" s="68"/>
       <c r="L3" s="68" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="M3" s="68"/>
       <c r="N3" s="68"/>
       <c r="O3" s="68" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="P3" s="68"/>
       <c r="Q3" s="68"/>
       <c r="R3" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="S3" s="15" t="s">
         <v>125</v>
-      </c>
-      <c r="S3" s="15" t="s">
-        <v>126</v>
       </c>
       <c r="T3" s="16" t="s">
         <v>122</v>
       </c>
       <c r="U3" s="16" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="4" spans="1:21" ht="25.5" x14ac:dyDescent="0.35">
+        <v>126</v>
+      </c>
+      <c r="V3" s="15" t="s">
+        <v>194</v>
+      </c>
+      <c r="W3" s="15" t="s">
+        <v>195</v>
+      </c>
+      <c r="X3" s="15" t="s">
+        <v>196</v>
+      </c>
+      <c r="Y3" s="15" t="s">
+        <v>197</v>
+      </c>
+      <c r="Z3" s="15" t="s">
+        <v>198</v>
+      </c>
+      <c r="AA3" s="15" t="s">
+        <v>199</v>
+      </c>
+      <c r="AB3" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="AC3" s="15" t="s">
+        <v>201</v>
+      </c>
+      <c r="AD3" s="15" t="s">
+        <v>202</v>
+      </c>
+      <c r="AE3" s="15" t="s">
+        <v>203</v>
+      </c>
+      <c r="AF3" s="15" t="s">
+        <v>204</v>
+      </c>
+      <c r="AG3" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="AH3" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="AI3" s="15" t="s">
+        <v>207</v>
+      </c>
+      <c r="AJ3" s="15" t="s">
+        <v>208</v>
+      </c>
+      <c r="AK3" s="79" t="s">
+        <v>209</v>
+      </c>
+      <c r="AL3" s="16" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="4" spans="1:38" ht="25.5" x14ac:dyDescent="0.35">
       <c r="D4" s="16" t="s">
+        <v>130</v>
+      </c>
+      <c r="E4" s="16" t="s">
         <v>131</v>
       </c>
-      <c r="E4" s="16" t="s">
+      <c r="F4" s="16" t="s">
         <v>132</v>
       </c>
-      <c r="F4" s="16" t="s">
+      <c r="G4" s="16" t="s">
+        <v>137</v>
+      </c>
+      <c r="H4" s="16" t="s">
+        <v>138</v>
+      </c>
+      <c r="I4" s="16" t="s">
         <v>133</v>
-      </c>
-      <c r="G4" s="16" t="s">
-        <v>138</v>
-      </c>
-      <c r="H4" s="16" t="s">
-        <v>139</v>
-      </c>
-      <c r="I4" s="16" t="s">
-        <v>134</v>
       </c>
       <c r="J4" s="16" t="s">
         <v>42</v>
       </c>
       <c r="K4" s="16" t="s">
+        <v>134</v>
+      </c>
+      <c r="L4" s="16" t="s">
+        <v>130</v>
+      </c>
+      <c r="M4" s="16" t="s">
+        <v>132</v>
+      </c>
+      <c r="N4" s="16" t="s">
         <v>135</v>
-      </c>
-      <c r="L4" s="16" t="s">
-        <v>131</v>
-      </c>
-      <c r="M4" s="16" t="s">
-        <v>133</v>
-      </c>
-      <c r="N4" s="16" t="s">
-        <v>136</v>
       </c>
       <c r="O4" s="16" t="s">
         <v>120</v>
@@ -3254,7 +4077,8 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
+    <mergeCell ref="V2:AL2"/>
     <mergeCell ref="O3:Q3"/>
     <mergeCell ref="D2:Q2"/>
     <mergeCell ref="A1:M1"/>
@@ -3268,7 +4092,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5692AB71-D55C-4890-A4C4-4497C431AAF2}">
   <sheetPr>
     <tabColor rgb="FFB8FEC9"/>
@@ -3306,21 +4130,21 @@
       <c r="O1" s="72"/>
     </row>
     <row r="2" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="48" t="s">
+      <c r="A2" s="51" t="s">
         <v>44</v>
       </c>
-      <c r="B2" s="49"/>
-      <c r="C2" s="50"/>
-      <c r="D2" s="48" t="s">
+      <c r="B2" s="52"/>
+      <c r="C2" s="53"/>
+      <c r="D2" s="51" t="s">
         <v>45</v>
       </c>
-      <c r="E2" s="49"/>
-      <c r="F2" s="50"/>
-      <c r="G2" s="48" t="s">
+      <c r="E2" s="52"/>
+      <c r="F2" s="53"/>
+      <c r="G2" s="51" t="s">
         <v>46</v>
       </c>
-      <c r="H2" s="49"/>
-      <c r="I2" s="50"/>
+      <c r="H2" s="52"/>
+      <c r="I2" s="53"/>
     </row>
     <row r="3" spans="1:15" ht="25.5" x14ac:dyDescent="0.35">
       <c r="A3" s="15" t="s">
@@ -3363,7 +4187,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB1C31A0-C7DA-43B1-B6AB-AA5BBBECAE63}">
   <sheetPr>
     <tabColor rgb="FFB8FEC9"/>
@@ -3401,20 +4225,20 @@
       <c r="Q1" s="72"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A2" s="48" t="s">
+      <c r="A2" s="51" t="s">
         <v>109</v>
       </c>
-      <c r="B2" s="49"/>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="50"/>
-      <c r="F2" s="48" t="s">
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="53"/>
+      <c r="F2" s="51" t="s">
         <v>110</v>
       </c>
-      <c r="G2" s="49"/>
-      <c r="H2" s="49"/>
-      <c r="I2" s="49"/>
-      <c r="J2" s="50"/>
+      <c r="G2" s="52"/>
+      <c r="H2" s="52"/>
+      <c r="I2" s="52"/>
+      <c r="J2" s="53"/>
     </row>
     <row r="3" spans="1:17" ht="38.25" x14ac:dyDescent="0.35">
       <c r="A3" s="15" t="s">
@@ -3467,7 +4291,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD8FBBB6-BAD2-4D62-996E-E16FA2533A1A}">
   <sheetPr>
     <tabColor rgb="FFB8FEC9"/>
@@ -3501,11 +4325,11 @@
       <c r="O1" s="72"/>
     </row>
     <row r="2" spans="1:15" ht="36" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="48" t="s">
+      <c r="A2" s="51" t="s">
         <v>47</v>
       </c>
-      <c r="B2" s="50"/>
-      <c r="C2" s="52" t="s">
+      <c r="B2" s="53"/>
+      <c r="C2" s="58" t="s">
         <v>50</v>
       </c>
     </row>
@@ -3516,7 +4340,7 @@
       <c r="B3" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="C3" s="53"/>
+      <c r="C3" s="59"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -3527,100 +4351,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{773AF20E-74BF-463C-9F61-BFE009D6FACB}">
-  <sheetPr>
-    <tabColor rgb="FFB8FEC9"/>
-  </sheetPr>
-  <dimension ref="A1:O3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7109375" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="15.7109375" style="11"/>
-    <col min="2" max="2" width="15.7109375" style="1"/>
-    <col min="3" max="7" width="15.7109375" style="2"/>
-    <col min="8" max="8" width="15.7109375" style="14"/>
-    <col min="9" max="9" width="15.7109375" style="2"/>
-    <col min="10" max="10" width="15.7109375" style="12"/>
-    <col min="11" max="16384" width="15.7109375" style="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:15" s="20" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="72" t="s">
-        <v>51</v>
-      </c>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="D1" s="72"/>
-      <c r="E1" s="72"/>
-      <c r="F1" s="72"/>
-      <c r="G1" s="72"/>
-      <c r="H1" s="72"/>
-      <c r="I1" s="72"/>
-      <c r="J1" s="72"/>
-      <c r="K1" s="72"/>
-      <c r="L1" s="72"/>
-      <c r="M1" s="72"/>
-      <c r="N1" s="72"/>
-      <c r="O1" s="72"/>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A2" s="52" t="s">
-        <v>91</v>
-      </c>
-      <c r="B2" s="48" t="s">
-        <v>53</v>
-      </c>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="49"/>
-      <c r="G2" s="50"/>
-      <c r="H2" s="48" t="s">
-        <v>60</v>
-      </c>
-      <c r="I2" s="49"/>
-      <c r="J2" s="50"/>
-    </row>
-    <row r="3" spans="1:15" ht="51" x14ac:dyDescent="0.35">
-      <c r="A3" s="53"/>
-      <c r="B3" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="C3" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="D3" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="E3" s="15" t="s">
-        <v>57</v>
-      </c>
-      <c r="F3" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="G3" s="15" t="s">
-        <v>59</v>
-      </c>
-      <c r="H3" s="17" t="s">
-        <v>63</v>
-      </c>
-      <c r="I3" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="J3" s="16" t="s">
-        <v>61</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="A1:O1"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
améliore le template excel d'export des indicateurs vsme
modifications de style uniquement et de cellules sélectionnées à l'ouverture du fichier/des onglets
</commit_message>
<xml_diff>
--- a/impact/vsme/xlsx/VSME.xlsx
+++ b/impact/vsme/xlsx/VSME.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmonteiro-de-mac-adc\Desktop\ancien bureau\Fichier\CSRD\Tableau ESRS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LDE-CASTELBAJAC-ADC\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2578CB28-8C22-4A67-A7F3-50ADB1D46C11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CD7DF51C-B45F-4FF4-A08E-7C2EC3086646}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="25440" windowHeight="15270" tabRatio="500" firstSheet="2" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="&gt;&gt;&gt; " sheetId="3" r:id="rId1"/>
@@ -923,59 +923,11 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="27">
+  <borders count="13">
     <border>
       <left/>
       <right/>
       <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -1031,132 +983,10 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
       <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
@@ -1171,32 +1001,6 @@
         <color indexed="64"/>
       </right>
       <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
         <color indexed="64"/>
       </top>
       <bottom style="thin">
@@ -1245,35 +1049,53 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1286,145 +1108,13 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="10" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1433,44 +1123,95 @@
     <xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1950,39 +1691,39 @@
     <tabColor rgb="FFFFEDC3"/>
   </sheetPr>
   <dimension ref="C10:K30"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.85546875" style="6" customWidth="1"/>
-    <col min="2" max="2" width="3" style="6" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="6" customWidth="1"/>
-    <col min="4" max="4" width="10.85546875" style="6" customWidth="1"/>
-    <col min="5" max="16384" width="10.85546875" style="6"/>
+    <col min="1" max="1" width="10.81640625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="3" style="3" customWidth="1"/>
+    <col min="3" max="3" width="21.7265625" style="3" customWidth="1"/>
+    <col min="4" max="4" width="10.81640625" style="3" customWidth="1"/>
+    <col min="5" max="16384" width="10.81640625" style="3"/>
   </cols>
   <sheetData>
-    <row r="10" spans="3:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="I10" s="6" t="s">
+    <row r="10" spans="3:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="I10" s="3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="3:9" s="7" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C11" s="47" t="s">
+    <row r="11" spans="3:9" s="4" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C11" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="D11" s="47"/>
-      <c r="E11" s="47"/>
-    </row>
-    <row r="13" spans="3:9" ht="72.75" customHeight="1" x14ac:dyDescent="1.25">
-      <c r="C13" s="8" t="s">
+      <c r="D11" s="34"/>
+      <c r="E11" s="34"/>
+    </row>
+    <row r="13" spans="3:9" ht="72.75" customHeight="1" x14ac:dyDescent="1.95">
+      <c r="C13" s="5" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="25" spans="8:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K25" s="6" t="s">
+    <row r="25" spans="8:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="K25" s="3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="8:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="H30" s="7"/>
+    <row r="30" spans="8:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="H30" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2000,81 +1741,81 @@
     <tabColor rgb="FFB8FEC9"/>
   </sheetPr>
   <dimension ref="A1:O3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7109375" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7265625" defaultRowHeight="17.5" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="15.7109375" style="11"/>
-    <col min="2" max="2" width="15.7109375" style="1"/>
-    <col min="3" max="7" width="15.7109375" style="2"/>
-    <col min="8" max="8" width="15.7109375" style="14"/>
-    <col min="9" max="9" width="15.7109375" style="2"/>
-    <col min="10" max="10" width="15.7109375" style="12"/>
-    <col min="11" max="16384" width="15.7109375" style="2"/>
+    <col min="1" max="1" width="15.7265625" style="7"/>
+    <col min="2" max="2" width="15.7265625" style="1"/>
+    <col min="3" max="7" width="15.7265625" style="2"/>
+    <col min="8" max="8" width="15.7265625" style="10"/>
+    <col min="9" max="9" width="15.7265625" style="2"/>
+    <col min="10" max="10" width="15.7265625" style="8"/>
+    <col min="11" max="16384" width="15.7265625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="20" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="72" t="s">
+    <row r="1" spans="1:15" s="14" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="36" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="D1" s="72"/>
-      <c r="E1" s="72"/>
-      <c r="F1" s="72"/>
-      <c r="G1" s="72"/>
-      <c r="H1" s="72"/>
-      <c r="I1" s="72"/>
-      <c r="J1" s="72"/>
-      <c r="K1" s="72"/>
-      <c r="L1" s="72"/>
-      <c r="M1" s="72"/>
-      <c r="N1" s="72"/>
-      <c r="O1" s="72"/>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A2" s="58" t="s">
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
+      <c r="I1" s="36"/>
+      <c r="J1" s="36"/>
+      <c r="K1" s="36"/>
+      <c r="L1" s="36"/>
+      <c r="M1" s="36"/>
+      <c r="N1" s="36"/>
+      <c r="O1" s="36"/>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.5">
+      <c r="A2" s="42" t="s">
         <v>91</v>
       </c>
-      <c r="B2" s="51" t="s">
+      <c r="B2" s="42" t="s">
         <v>53</v>
       </c>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
-      <c r="E2" s="52"/>
-      <c r="F2" s="52"/>
-      <c r="G2" s="53"/>
-      <c r="H2" s="51" t="s">
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42" t="s">
         <v>60</v>
       </c>
-      <c r="I2" s="52"/>
-      <c r="J2" s="53"/>
-    </row>
-    <row r="3" spans="1:15" ht="51" x14ac:dyDescent="0.35">
-      <c r="A3" s="59"/>
-      <c r="B3" s="15" t="s">
+      <c r="I2" s="42"/>
+      <c r="J2" s="42"/>
+    </row>
+    <row r="3" spans="1:15" ht="50" x14ac:dyDescent="0.5">
+      <c r="A3" s="42"/>
+      <c r="B3" s="50" t="s">
         <v>54</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="50" t="s">
         <v>55</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="50" t="s">
         <v>56</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="E3" s="50" t="s">
         <v>57</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="F3" s="50" t="s">
         <v>58</v>
       </c>
-      <c r="G3" s="15" t="s">
+      <c r="G3" s="50" t="s">
         <v>59</v>
       </c>
-      <c r="H3" s="17" t="s">
+      <c r="H3" s="50" t="s">
         <v>63</v>
       </c>
-      <c r="I3" s="15" t="s">
+      <c r="I3" s="50" t="s">
         <v>62</v>
       </c>
-      <c r="J3" s="16" t="s">
+      <c r="J3" s="50" t="s">
         <v>61</v>
       </c>
     </row>
@@ -2096,293 +1837,294 @@
     <tabColor rgb="FFB8FEC9"/>
   </sheetPr>
   <dimension ref="A1:P21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7109375" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7265625" defaultRowHeight="17.5" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="2" width="15.7109375" style="12"/>
-    <col min="3" max="6" width="15.7109375" style="82"/>
-    <col min="7" max="7" width="15.7109375" style="87"/>
-    <col min="8" max="11" width="15.7109375" style="82"/>
-    <col min="12" max="12" width="15.7109375" style="87"/>
-    <col min="13" max="15" width="15.7109375" style="93"/>
-    <col min="16" max="16" width="15.7109375" style="94"/>
-    <col min="17" max="16384" width="15.7109375" style="2"/>
+    <col min="1" max="2" width="15.7265625" style="8"/>
+    <col min="3" max="6" width="15.7265625" style="26"/>
+    <col min="7" max="7" width="15.7265625" style="28"/>
+    <col min="8" max="8" width="28.90625" style="26" bestFit="1" customWidth="1"/>
+    <col min="9" max="11" width="15.7265625" style="26"/>
+    <col min="12" max="12" width="15.7265625" style="28"/>
+    <col min="13" max="15" width="15.7265625" style="32"/>
+    <col min="16" max="16" width="15.7265625" style="33"/>
+    <col min="17" max="16384" width="15.7265625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="20" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="72" t="s">
+    <row r="1" spans="1:16" s="14" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="36" t="s">
         <v>223</v>
       </c>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="D1" s="72"/>
-      <c r="E1" s="72"/>
-      <c r="F1" s="72"/>
-      <c r="G1" s="72"/>
-      <c r="H1" s="72"/>
-      <c r="I1" s="72"/>
-      <c r="J1" s="72"/>
-      <c r="K1" s="72"/>
-      <c r="L1" s="72"/>
-      <c r="M1" s="72"/>
-      <c r="N1" s="72"/>
-      <c r="O1" s="72"/>
-      <c r="P1" s="88"/>
-    </row>
-    <row r="2" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="58" t="s">
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
+      <c r="I1" s="36"/>
+      <c r="J1" s="36"/>
+      <c r="K1" s="36"/>
+      <c r="L1" s="36"/>
+      <c r="M1" s="36"/>
+      <c r="N1" s="36"/>
+      <c r="O1" s="36"/>
+      <c r="P1" s="29"/>
+    </row>
+    <row r="2" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A2" s="42" t="s">
         <v>212</v>
       </c>
-      <c r="B2" s="58" t="s">
+      <c r="B2" s="42" t="s">
         <v>213</v>
       </c>
-      <c r="C2" s="83" t="s">
+      <c r="C2" s="53" t="s">
         <v>211</v>
       </c>
-      <c r="D2" s="84"/>
-      <c r="E2" s="84"/>
-      <c r="F2" s="84"/>
-      <c r="G2" s="85"/>
-      <c r="H2" s="51" t="s">
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="54"/>
+      <c r="G2" s="54"/>
+      <c r="H2" s="42" t="s">
         <v>193</v>
       </c>
-      <c r="I2" s="52"/>
-      <c r="J2" s="52"/>
-      <c r="K2" s="52"/>
-      <c r="L2" s="53"/>
-      <c r="M2" s="83" t="s">
+      <c r="I2" s="42"/>
+      <c r="J2" s="42"/>
+      <c r="K2" s="42"/>
+      <c r="L2" s="42"/>
+      <c r="M2" s="53" t="s">
         <v>218</v>
       </c>
-      <c r="N2" s="84"/>
-      <c r="O2" s="84"/>
-      <c r="P2" s="85"/>
-    </row>
-    <row r="3" spans="1:16" ht="63.75" x14ac:dyDescent="0.35">
-      <c r="A3" s="59"/>
-      <c r="B3" s="59"/>
-      <c r="C3" s="86"/>
-      <c r="D3" s="18" t="s">
+      <c r="N2" s="54"/>
+      <c r="O2" s="54"/>
+      <c r="P2" s="54"/>
+    </row>
+    <row r="3" spans="1:16" ht="62.5" x14ac:dyDescent="0.5">
+      <c r="A3" s="42"/>
+      <c r="B3" s="42"/>
+      <c r="C3" s="55"/>
+      <c r="D3" s="50" t="s">
         <v>214</v>
       </c>
-      <c r="E3" s="18" t="s">
+      <c r="E3" s="50" t="s">
         <v>215</v>
       </c>
-      <c r="F3" s="18" t="s">
+      <c r="F3" s="50" t="s">
         <v>216</v>
       </c>
-      <c r="G3" s="16" t="s">
+      <c r="G3" s="50" t="s">
         <v>217</v>
       </c>
-      <c r="H3" s="18"/>
-      <c r="I3" s="18" t="s">
+      <c r="H3" s="50"/>
+      <c r="I3" s="50" t="s">
         <v>214</v>
       </c>
-      <c r="J3" s="18" t="s">
+      <c r="J3" s="50" t="s">
         <v>215</v>
       </c>
-      <c r="K3" s="15" t="s">
+      <c r="K3" s="50" t="s">
         <v>216</v>
       </c>
-      <c r="L3" s="16" t="s">
+      <c r="L3" s="50" t="s">
         <v>217</v>
       </c>
-      <c r="M3" s="18" t="s">
+      <c r="M3" s="50" t="s">
         <v>219</v>
       </c>
-      <c r="N3" s="18" t="s">
+      <c r="N3" s="50" t="s">
         <v>220</v>
       </c>
-      <c r="O3" s="18" t="s">
+      <c r="O3" s="50" t="s">
         <v>221</v>
       </c>
-      <c r="P3" s="16" t="s">
+      <c r="P3" s="50" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="25.5" x14ac:dyDescent="0.35">
-      <c r="C4" s="18" t="s">
+    <row r="4" spans="1:16" ht="25" x14ac:dyDescent="0.5">
+      <c r="C4" s="50" t="s">
         <v>124</v>
       </c>
-      <c r="D4" s="86"/>
-      <c r="E4" s="86"/>
-      <c r="F4" s="86"/>
-      <c r="G4" s="16"/>
-      <c r="H4" s="80" t="s">
+      <c r="D4" s="55"/>
+      <c r="E4" s="55"/>
+      <c r="F4" s="55"/>
+      <c r="G4" s="50"/>
+      <c r="H4" s="56" t="s">
         <v>194</v>
       </c>
-      <c r="I4" s="89"/>
-      <c r="J4" s="86"/>
-      <c r="K4" s="86"/>
-      <c r="L4" s="90"/>
-      <c r="M4" s="91"/>
-      <c r="N4" s="91"/>
-      <c r="O4" s="91"/>
-      <c r="P4" s="92"/>
-    </row>
-    <row r="5" spans="1:16" ht="25.5" x14ac:dyDescent="0.35">
-      <c r="C5" s="18" t="s">
+      <c r="I4" s="57"/>
+      <c r="J4" s="55"/>
+      <c r="K4" s="55"/>
+      <c r="L4" s="55"/>
+      <c r="M4" s="30"/>
+      <c r="N4" s="30"/>
+      <c r="O4" s="30"/>
+      <c r="P4" s="31"/>
+    </row>
+    <row r="5" spans="1:16" ht="25" x14ac:dyDescent="0.5">
+      <c r="C5" s="50" t="s">
         <v>125</v>
       </c>
-      <c r="D5" s="86"/>
-      <c r="E5" s="86"/>
-      <c r="F5" s="86"/>
-      <c r="G5" s="16"/>
-      <c r="H5" s="80" t="s">
+      <c r="D5" s="55"/>
+      <c r="E5" s="55"/>
+      <c r="F5" s="55"/>
+      <c r="G5" s="50"/>
+      <c r="H5" s="56" t="s">
         <v>195</v>
       </c>
-      <c r="I5" s="89"/>
-      <c r="J5" s="86"/>
-      <c r="K5" s="86"/>
-      <c r="L5" s="90"/>
-    </row>
-    <row r="6" spans="1:16" ht="51" x14ac:dyDescent="0.35">
-      <c r="C6" s="18" t="s">
+      <c r="I5" s="57"/>
+      <c r="J5" s="55"/>
+      <c r="K5" s="55"/>
+      <c r="L5" s="55"/>
+    </row>
+    <row r="6" spans="1:16" ht="50" x14ac:dyDescent="0.5">
+      <c r="C6" s="50" t="s">
         <v>231</v>
       </c>
-      <c r="D6" s="86"/>
-      <c r="E6" s="86"/>
-      <c r="F6" s="86"/>
-      <c r="G6" s="16"/>
-      <c r="H6" s="80" t="s">
+      <c r="D6" s="55"/>
+      <c r="E6" s="55"/>
+      <c r="F6" s="55"/>
+      <c r="G6" s="50"/>
+      <c r="H6" s="56" t="s">
         <v>196</v>
       </c>
-      <c r="I6" s="86"/>
-      <c r="J6" s="86"/>
-      <c r="K6" s="86"/>
-      <c r="L6" s="90"/>
-    </row>
-    <row r="7" spans="1:16" ht="38.25" x14ac:dyDescent="0.35">
-      <c r="C7" s="18"/>
-      <c r="D7" s="86"/>
-      <c r="E7" s="86"/>
-      <c r="F7" s="86"/>
-      <c r="G7" s="16"/>
-      <c r="H7" s="80" t="s">
+      <c r="I6" s="55"/>
+      <c r="J6" s="55"/>
+      <c r="K6" s="55"/>
+      <c r="L6" s="55"/>
+    </row>
+    <row r="7" spans="1:16" ht="37.5" x14ac:dyDescent="0.5">
+      <c r="C7" s="12"/>
+      <c r="D7" s="27"/>
+      <c r="E7" s="27"/>
+      <c r="F7" s="27"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="56" t="s">
         <v>197</v>
       </c>
-      <c r="I7" s="86"/>
-      <c r="J7" s="86"/>
-      <c r="K7" s="86"/>
-      <c r="L7" s="90"/>
-    </row>
-    <row r="8" spans="1:16" ht="38.25" x14ac:dyDescent="0.35">
-      <c r="H8" s="80" t="s">
+      <c r="I7" s="55"/>
+      <c r="J7" s="55"/>
+      <c r="K7" s="55"/>
+      <c r="L7" s="55"/>
+    </row>
+    <row r="8" spans="1:16" ht="25" x14ac:dyDescent="0.5">
+      <c r="H8" s="56" t="s">
         <v>198</v>
       </c>
-      <c r="I8" s="86"/>
-      <c r="J8" s="86"/>
-      <c r="K8" s="86"/>
-      <c r="L8" s="95"/>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="H9" s="80" t="s">
+      <c r="I8" s="55"/>
+      <c r="J8" s="55"/>
+      <c r="K8" s="55"/>
+      <c r="L8" s="57"/>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.5">
+      <c r="H9" s="56" t="s">
         <v>199</v>
       </c>
-      <c r="I9" s="86"/>
-      <c r="J9" s="86"/>
-      <c r="K9" s="86"/>
-      <c r="L9" s="95"/>
-    </row>
-    <row r="10" spans="1:16" ht="38.25" x14ac:dyDescent="0.35">
-      <c r="H10" s="80" t="s">
+      <c r="I9" s="55"/>
+      <c r="J9" s="55"/>
+      <c r="K9" s="55"/>
+      <c r="L9" s="57"/>
+    </row>
+    <row r="10" spans="1:16" ht="37.5" x14ac:dyDescent="0.5">
+      <c r="H10" s="56" t="s">
         <v>200</v>
       </c>
-      <c r="I10" s="86"/>
-      <c r="J10" s="86"/>
-      <c r="K10" s="86"/>
-      <c r="L10" s="95"/>
-    </row>
-    <row r="11" spans="1:16" ht="25.5" x14ac:dyDescent="0.35">
-      <c r="H11" s="80" t="s">
+      <c r="I10" s="55"/>
+      <c r="J10" s="55"/>
+      <c r="K10" s="55"/>
+      <c r="L10" s="57"/>
+    </row>
+    <row r="11" spans="1:16" ht="25" x14ac:dyDescent="0.5">
+      <c r="H11" s="56" t="s">
         <v>201</v>
       </c>
-      <c r="I11" s="86"/>
-      <c r="J11" s="86"/>
-      <c r="K11" s="86"/>
-      <c r="L11" s="95"/>
-    </row>
-    <row r="12" spans="1:16" ht="25.5" x14ac:dyDescent="0.35">
-      <c r="H12" s="80" t="s">
+      <c r="I11" s="55"/>
+      <c r="J11" s="55"/>
+      <c r="K11" s="55"/>
+      <c r="L11" s="57"/>
+    </row>
+    <row r="12" spans="1:16" ht="25" x14ac:dyDescent="0.5">
+      <c r="H12" s="56" t="s">
         <v>202</v>
       </c>
-      <c r="I12" s="86"/>
-      <c r="J12" s="86"/>
-      <c r="K12" s="86"/>
-      <c r="L12" s="95"/>
-    </row>
-    <row r="13" spans="1:16" ht="25.5" x14ac:dyDescent="0.35">
-      <c r="H13" s="80" t="s">
+      <c r="I12" s="55"/>
+      <c r="J12" s="55"/>
+      <c r="K12" s="55"/>
+      <c r="L12" s="57"/>
+    </row>
+    <row r="13" spans="1:16" ht="25" x14ac:dyDescent="0.5">
+      <c r="H13" s="56" t="s">
         <v>203</v>
       </c>
-      <c r="I13" s="86"/>
-      <c r="J13" s="86"/>
-      <c r="K13" s="86"/>
-      <c r="L13" s="95"/>
-    </row>
-    <row r="14" spans="1:16" ht="25.5" x14ac:dyDescent="0.35">
-      <c r="H14" s="80" t="s">
+      <c r="I13" s="55"/>
+      <c r="J13" s="55"/>
+      <c r="K13" s="55"/>
+      <c r="L13" s="57"/>
+    </row>
+    <row r="14" spans="1:16" ht="25" x14ac:dyDescent="0.5">
+      <c r="H14" s="56" t="s">
         <v>204</v>
       </c>
-      <c r="I14" s="86"/>
-      <c r="J14" s="86"/>
-      <c r="K14" s="86"/>
-      <c r="L14" s="95"/>
-    </row>
-    <row r="15" spans="1:16" ht="38.25" x14ac:dyDescent="0.35">
-      <c r="H15" s="80" t="s">
+      <c r="I14" s="55"/>
+      <c r="J14" s="55"/>
+      <c r="K14" s="55"/>
+      <c r="L14" s="57"/>
+    </row>
+    <row r="15" spans="1:16" ht="37.5" x14ac:dyDescent="0.5">
+      <c r="H15" s="56" t="s">
         <v>205</v>
       </c>
-      <c r="I15" s="86"/>
-      <c r="J15" s="86"/>
-      <c r="K15" s="86"/>
-      <c r="L15" s="95"/>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="H16" s="80" t="s">
+      <c r="I15" s="55"/>
+      <c r="J15" s="55"/>
+      <c r="K15" s="55"/>
+      <c r="L15" s="57"/>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.5">
+      <c r="H16" s="56" t="s">
         <v>206</v>
       </c>
-      <c r="I16" s="86"/>
-      <c r="J16" s="86"/>
-      <c r="K16" s="86"/>
-      <c r="L16" s="95"/>
-    </row>
-    <row r="17" spans="8:12" x14ac:dyDescent="0.35">
-      <c r="H17" s="80" t="s">
+      <c r="I16" s="55"/>
+      <c r="J16" s="55"/>
+      <c r="K16" s="55"/>
+      <c r="L16" s="57"/>
+    </row>
+    <row r="17" spans="8:12" x14ac:dyDescent="0.5">
+      <c r="H17" s="56" t="s">
         <v>207</v>
       </c>
-      <c r="I17" s="86"/>
-      <c r="J17" s="86"/>
-      <c r="K17" s="86"/>
-      <c r="L17" s="95"/>
-    </row>
-    <row r="18" spans="8:12" x14ac:dyDescent="0.35">
-      <c r="H18" s="80" t="s">
+      <c r="I17" s="55"/>
+      <c r="J17" s="55"/>
+      <c r="K17" s="55"/>
+      <c r="L17" s="57"/>
+    </row>
+    <row r="18" spans="8:12" x14ac:dyDescent="0.5">
+      <c r="H18" s="56" t="s">
         <v>208</v>
       </c>
-      <c r="I18" s="86"/>
-      <c r="J18" s="86"/>
-      <c r="K18" s="86"/>
-      <c r="L18" s="95"/>
-    </row>
-    <row r="19" spans="8:12" x14ac:dyDescent="0.35">
-      <c r="H19" s="80" t="s">
+      <c r="I18" s="55"/>
+      <c r="J18" s="55"/>
+      <c r="K18" s="55"/>
+      <c r="L18" s="57"/>
+    </row>
+    <row r="19" spans="8:12" x14ac:dyDescent="0.5">
+      <c r="H19" s="56" t="s">
         <v>229</v>
       </c>
-      <c r="I19" s="89"/>
-      <c r="J19" s="89"/>
-      <c r="K19" s="89"/>
-      <c r="L19" s="90"/>
-    </row>
-    <row r="20" spans="8:12" ht="25.5" x14ac:dyDescent="0.35">
-      <c r="H20" s="80" t="s">
+      <c r="I19" s="57"/>
+      <c r="J19" s="57"/>
+      <c r="K19" s="57"/>
+      <c r="L19" s="55"/>
+    </row>
+    <row r="20" spans="8:12" x14ac:dyDescent="0.5">
+      <c r="H20" s="56" t="s">
         <v>230</v>
       </c>
-      <c r="I20" s="89"/>
-      <c r="J20" s="89"/>
-      <c r="K20" s="89"/>
-      <c r="L20" s="90"/>
-    </row>
-    <row r="21" spans="8:12" x14ac:dyDescent="0.35">
-      <c r="H21" s="81"/>
+      <c r="I20" s="57"/>
+      <c r="J20" s="57"/>
+      <c r="K20" s="57"/>
+      <c r="L20" s="55"/>
+    </row>
+    <row r="21" spans="8:12" x14ac:dyDescent="0.5">
+      <c r="H21" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -2404,77 +2146,77 @@
     <tabColor rgb="FFB8FEC9"/>
   </sheetPr>
   <dimension ref="A1:P3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7109375" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7265625" defaultRowHeight="17.5" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="3" width="15.7109375" style="1"/>
-    <col min="4" max="5" width="15.7109375" style="2"/>
-    <col min="6" max="6" width="15.7109375" style="14"/>
-    <col min="7" max="8" width="15.7109375" style="2"/>
-    <col min="9" max="9" width="15.7109375" style="12"/>
-    <col min="10" max="16384" width="15.7109375" style="2"/>
+    <col min="1" max="3" width="15.7265625" style="1"/>
+    <col min="4" max="5" width="15.7265625" style="2"/>
+    <col min="6" max="6" width="15.7265625" style="10"/>
+    <col min="7" max="8" width="15.7265625" style="2"/>
+    <col min="9" max="9" width="15.7265625" style="8"/>
+    <col min="10" max="16384" width="15.7265625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="20" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="72" t="s">
+    <row r="1" spans="1:16" s="14" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="36" t="s">
         <v>190</v>
       </c>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="D1" s="72"/>
-      <c r="E1" s="72"/>
-      <c r="F1" s="72"/>
-      <c r="G1" s="72"/>
-      <c r="H1" s="72"/>
-      <c r="I1" s="72"/>
-      <c r="J1" s="72"/>
-      <c r="K1" s="72"/>
-      <c r="L1" s="72"/>
-      <c r="M1" s="72"/>
-      <c r="N1" s="72"/>
-      <c r="O1" s="72"/>
-      <c r="P1" s="72"/>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A2" s="51" t="s">
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
+      <c r="I1" s="36"/>
+      <c r="J1" s="36"/>
+      <c r="K1" s="36"/>
+      <c r="L1" s="36"/>
+      <c r="M1" s="36"/>
+      <c r="N1" s="36"/>
+      <c r="O1" s="36"/>
+      <c r="P1" s="36"/>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.5">
+      <c r="A2" s="42" t="s">
         <v>181</v>
       </c>
-      <c r="B2" s="52"/>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
-      <c r="E2" s="53"/>
-      <c r="F2" s="51" t="s">
+      <c r="B2" s="42"/>
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42" t="s">
         <v>186</v>
       </c>
-      <c r="G2" s="52"/>
-      <c r="H2" s="52"/>
-      <c r="I2" s="53"/>
-    </row>
-    <row r="3" spans="1:16" ht="38.25" x14ac:dyDescent="0.35">
-      <c r="A3" s="15" t="s">
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
+      <c r="I2" s="42"/>
+    </row>
+    <row r="3" spans="1:16" ht="37.5" x14ac:dyDescent="0.5">
+      <c r="A3" s="50" t="s">
         <v>191</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="50" t="s">
         <v>182</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="50" t="s">
         <v>183</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="50" t="s">
         <v>184</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="E3" s="50" t="s">
         <v>185</v>
       </c>
-      <c r="F3" s="17" t="s">
+      <c r="F3" s="50" t="s">
         <v>187</v>
       </c>
-      <c r="G3" s="15" t="s">
+      <c r="G3" s="50" t="s">
         <v>188</v>
       </c>
-      <c r="H3" s="15" t="s">
+      <c r="H3" s="50" t="s">
         <v>189</v>
       </c>
-      <c r="I3" s="16" t="s">
+      <c r="I3" s="50" t="s">
         <v>184</v>
       </c>
     </row>
@@ -2506,85 +2248,85 @@
     <tabColor rgb="FFFEE7FC"/>
   </sheetPr>
   <dimension ref="A1:O12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="17.5" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="11.42578125" style="11" customWidth="1"/>
-    <col min="3" max="5" width="11.42578125" style="2" customWidth="1"/>
-    <col min="6" max="6" width="11.42578125" style="2"/>
-    <col min="7" max="7" width="11.42578125" style="14"/>
-    <col min="8" max="8" width="11.42578125" style="2"/>
-    <col min="9" max="9" width="11.42578125" style="13"/>
-    <col min="10" max="16384" width="11.42578125" style="2"/>
+    <col min="1" max="1" width="11.453125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="11.453125" style="7" customWidth="1"/>
+    <col min="3" max="5" width="11.453125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="11.453125" style="2"/>
+    <col min="7" max="7" width="11.453125" style="10"/>
+    <col min="8" max="8" width="11.453125" style="2"/>
+    <col min="9" max="9" width="11.453125" style="9"/>
+    <col min="10" max="16384" width="11.453125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="21" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="73" t="s">
+    <row r="1" spans="1:15" s="15" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="37" t="s">
         <v>79</v>
       </c>
-      <c r="B1" s="73"/>
-      <c r="C1" s="73"/>
-      <c r="D1" s="73"/>
-      <c r="E1" s="73"/>
-      <c r="F1" s="73"/>
-      <c r="G1" s="73"/>
-      <c r="H1" s="73"/>
-      <c r="I1" s="73"/>
-      <c r="J1" s="73"/>
-      <c r="K1" s="73"/>
-      <c r="L1" s="73"/>
-      <c r="M1" s="73"/>
-      <c r="N1" s="73"/>
-      <c r="O1" s="73"/>
-    </row>
-    <row r="2" spans="1:15" ht="39" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="51" t="s">
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="37"/>
+      <c r="H1" s="37"/>
+      <c r="I1" s="37"/>
+      <c r="J1" s="37"/>
+      <c r="K1" s="37"/>
+      <c r="L1" s="37"/>
+      <c r="M1" s="37"/>
+      <c r="N1" s="37"/>
+      <c r="O1" s="37"/>
+    </row>
+    <row r="2" spans="1:15" ht="39" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A2" s="42" t="s">
         <v>80</v>
       </c>
-      <c r="B2" s="53"/>
-      <c r="C2" s="51" t="s">
+      <c r="B2" s="42"/>
+      <c r="C2" s="42" t="s">
         <v>83</v>
       </c>
-      <c r="D2" s="52"/>
-      <c r="E2" s="52"/>
-      <c r="F2" s="53"/>
-      <c r="G2" s="51" t="s">
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42" t="s">
         <v>86</v>
       </c>
-      <c r="H2" s="53"/>
-      <c r="I2" s="58" t="s">
+      <c r="H2" s="42"/>
+      <c r="I2" s="42" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="25.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="15" t="s">
+    <row r="3" spans="1:15" ht="25" x14ac:dyDescent="0.5">
+      <c r="A3" s="50" t="s">
         <v>81</v>
       </c>
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="50" t="s">
         <v>82</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="50" t="s">
         <v>84</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="50" t="s">
         <v>85</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="E3" s="50" t="s">
         <v>103</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="F3" s="50" t="s">
         <v>92</v>
       </c>
-      <c r="G3" s="17" t="s">
+      <c r="G3" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="H3" s="15" t="s">
+      <c r="H3" s="50" t="s">
         <v>87</v>
       </c>
-      <c r="I3" s="59"/>
-    </row>
-    <row r="12" spans="1:15" ht="72.75" x14ac:dyDescent="1.25">
-      <c r="E12" s="22"/>
+      <c r="I3" s="42"/>
+    </row>
+    <row r="12" spans="1:15" ht="74" x14ac:dyDescent="1.95">
+      <c r="E12" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -2605,54 +2347,54 @@
     <tabColor rgb="FFFEE7FC"/>
   </sheetPr>
   <dimension ref="A1:O12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="17.5" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="13.7109375" style="11" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" style="12" customWidth="1"/>
-    <col min="4" max="5" width="11.42578125" style="2" customWidth="1"/>
-    <col min="6" max="16384" width="11.42578125" style="2"/>
+    <col min="1" max="1" width="11.453125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="18.08984375" style="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="36.08984375" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="11.453125" style="2" customWidth="1"/>
+    <col min="6" max="16384" width="11.453125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="21" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="73" t="s">
+    <row r="1" spans="1:15" s="15" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="37" t="s">
         <v>102</v>
       </c>
-      <c r="B1" s="73"/>
-      <c r="C1" s="73"/>
-      <c r="D1" s="73"/>
-      <c r="E1" s="73"/>
-      <c r="F1" s="73"/>
-      <c r="G1" s="73"/>
-      <c r="H1" s="73"/>
-      <c r="I1" s="73"/>
-      <c r="J1" s="73"/>
-      <c r="K1" s="73"/>
-      <c r="L1" s="73"/>
-      <c r="M1" s="73"/>
-      <c r="N1" s="73"/>
-      <c r="O1" s="73"/>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A2" s="51" t="s">
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="37"/>
+      <c r="H1" s="37"/>
+      <c r="I1" s="37"/>
+      <c r="J1" s="37"/>
+      <c r="K1" s="37"/>
+      <c r="L1" s="37"/>
+      <c r="M1" s="37"/>
+      <c r="N1" s="37"/>
+      <c r="O1" s="37"/>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.5">
+      <c r="A2" s="42" t="s">
         <v>64</v>
       </c>
-      <c r="B2" s="53"/>
-      <c r="C2" s="58" t="s">
+      <c r="B2" s="42"/>
+      <c r="C2" s="42" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="51" x14ac:dyDescent="0.35">
-      <c r="A3" s="15" t="s">
+    <row r="3" spans="1:15" ht="37.5" x14ac:dyDescent="0.5">
+      <c r="A3" s="50" t="s">
         <v>65</v>
       </c>
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="50" t="s">
         <v>66</v>
       </c>
-      <c r="C3" s="59"/>
-    </row>
-    <row r="12" spans="1:15" ht="72.75" x14ac:dyDescent="1.25">
-      <c r="E12" s="22"/>
+      <c r="C3" s="42"/>
+    </row>
+    <row r="12" spans="1:15" ht="74" x14ac:dyDescent="1.95">
+      <c r="E12" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2671,109 +2413,109 @@
     <tabColor rgb="FFFEE7FC"/>
   </sheetPr>
   <dimension ref="A1:O7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="17.5" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" style="12" customWidth="1"/>
-    <col min="2" max="3" width="11.42578125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="13.7109375" style="11" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.42578125" style="1"/>
-    <col min="6" max="6" width="13.7109375" style="11" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.7109375" style="2" customWidth="1"/>
-    <col min="8" max="8" width="24.7109375" style="2" customWidth="1"/>
-    <col min="9" max="9" width="26" style="12" customWidth="1"/>
-    <col min="10" max="16384" width="11.42578125" style="2"/>
+    <col min="1" max="1" width="16.453125" style="8" customWidth="1"/>
+    <col min="2" max="3" width="11.453125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="13.7265625" style="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.453125" style="1"/>
+    <col min="6" max="6" width="13.7265625" style="7" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.7265625" style="2" customWidth="1"/>
+    <col min="8" max="8" width="24.7265625" style="2" customWidth="1"/>
+    <col min="9" max="9" width="26" style="8" customWidth="1"/>
+    <col min="10" max="16384" width="11.453125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="21" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="73" t="s">
+    <row r="1" spans="1:15" s="15" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="37" t="s">
         <v>101</v>
       </c>
-      <c r="B1" s="73"/>
-      <c r="C1" s="73"/>
-      <c r="D1" s="73"/>
-      <c r="E1" s="73"/>
-      <c r="F1" s="73"/>
-      <c r="G1" s="73"/>
-      <c r="H1" s="73"/>
-      <c r="I1" s="73"/>
-      <c r="J1" s="73"/>
-      <c r="K1" s="73"/>
-      <c r="L1" s="73"/>
-      <c r="M1" s="73"/>
-      <c r="N1" s="73"/>
-      <c r="O1" s="73"/>
-    </row>
-    <row r="2" spans="1:15" ht="54.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="58" t="s">
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="37"/>
+      <c r="H1" s="37"/>
+      <c r="I1" s="37"/>
+      <c r="J1" s="37"/>
+      <c r="K1" s="37"/>
+      <c r="L1" s="37"/>
+      <c r="M1" s="37"/>
+      <c r="N1" s="37"/>
+      <c r="O1" s="37"/>
+    </row>
+    <row r="2" spans="1:15" ht="54.75" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A2" s="42" t="s">
         <v>93</v>
       </c>
-      <c r="B2" s="51" t="s">
+      <c r="B2" s="42" t="s">
         <v>94</v>
       </c>
-      <c r="C2" s="52"/>
-      <c r="D2" s="53"/>
-      <c r="E2" s="51" t="s">
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42" t="s">
         <v>98</v>
       </c>
-      <c r="F2" s="53"/>
-      <c r="G2" s="51" t="s">
+      <c r="F2" s="42"/>
+      <c r="G2" s="42" t="s">
         <v>105</v>
       </c>
-      <c r="H2" s="52"/>
-      <c r="I2" s="53"/>
-    </row>
-    <row r="3" spans="1:15" ht="97.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="59"/>
-      <c r="B3" s="15" t="s">
+      <c r="H2" s="42"/>
+      <c r="I2" s="42"/>
+    </row>
+    <row r="3" spans="1:15" ht="97.5" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A3" s="42"/>
+      <c r="B3" s="50" t="s">
         <v>95</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="50" t="s">
         <v>96</v>
       </c>
-      <c r="D3" s="16" t="s">
+      <c r="D3" s="50" t="s">
         <v>97</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="E3" s="50" t="s">
         <v>99</v>
       </c>
-      <c r="F3" s="16" t="s">
+      <c r="F3" s="50" t="s">
         <v>98</v>
       </c>
-      <c r="G3" s="35"/>
-      <c r="H3" s="43" t="s">
+      <c r="G3" s="61"/>
+      <c r="H3" s="62" t="s">
         <v>100</v>
       </c>
-      <c r="I3" s="40" t="s">
+      <c r="I3" s="62" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="G4" s="37" t="s">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.5">
+      <c r="G4" s="58" t="s">
         <v>84</v>
       </c>
-      <c r="H4" s="42"/>
-      <c r="I4" s="41"/>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="G5" s="38" t="s">
+      <c r="H4" s="59"/>
+      <c r="I4" s="60"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.5">
+      <c r="G5" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="H5" s="42"/>
-      <c r="I5" s="41"/>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="G6" s="39" t="s">
+      <c r="H5" s="23"/>
+      <c r="I5" s="22"/>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.5">
+      <c r="G6" s="21" t="s">
         <v>106</v>
       </c>
-      <c r="H6" s="42"/>
-      <c r="I6" s="41"/>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="G7" s="36" t="s">
+      <c r="H6" s="23"/>
+      <c r="I6" s="22"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.5">
+      <c r="G7" s="19" t="s">
         <v>107</v>
       </c>
-      <c r="H7" s="42"/>
-      <c r="I7" s="41"/>
+      <c r="H7" s="23"/>
+      <c r="I7" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -2794,59 +2536,59 @@
     <tabColor rgb="FFFEE7FC"/>
   </sheetPr>
   <dimension ref="A1:O3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="17.5" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="2" width="11.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="13.7109375" style="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="13.7109375" style="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="11.42578125" style="2"/>
+    <col min="1" max="2" width="11.453125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="13.7265625" style="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.453125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="13.7265625" style="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="11.453125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="21" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="73" t="s">
+    <row r="1" spans="1:15" s="15" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="37" t="s">
         <v>171</v>
       </c>
-      <c r="B1" s="73"/>
-      <c r="C1" s="73"/>
-      <c r="D1" s="73"/>
-      <c r="E1" s="73"/>
-      <c r="F1" s="73"/>
-      <c r="G1" s="73"/>
-      <c r="H1" s="73"/>
-      <c r="I1" s="73"/>
-      <c r="J1" s="73"/>
-      <c r="K1" s="73"/>
-      <c r="L1" s="73"/>
-      <c r="M1" s="73"/>
-      <c r="N1" s="73"/>
-      <c r="O1" s="73"/>
-    </row>
-    <row r="2" spans="1:15" ht="53.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="51" t="s">
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="37"/>
+      <c r="H1" s="37"/>
+      <c r="I1" s="37"/>
+      <c r="J1" s="37"/>
+      <c r="K1" s="37"/>
+      <c r="L1" s="37"/>
+      <c r="M1" s="37"/>
+      <c r="N1" s="37"/>
+      <c r="O1" s="37"/>
+    </row>
+    <row r="2" spans="1:15" ht="53.25" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A2" s="42" t="s">
         <v>167</v>
       </c>
-      <c r="B2" s="52"/>
-      <c r="C2" s="53"/>
-      <c r="D2" s="51" t="s">
+      <c r="B2" s="42"/>
+      <c r="C2" s="42"/>
+      <c r="D2" s="42" t="s">
         <v>170</v>
       </c>
-      <c r="E2" s="53"/>
-    </row>
-    <row r="3" spans="1:15" ht="114.75" x14ac:dyDescent="0.35">
-      <c r="A3" s="15" t="s">
+      <c r="E2" s="42"/>
+    </row>
+    <row r="3" spans="1:15" ht="112.5" x14ac:dyDescent="0.5">
+      <c r="A3" s="50" t="s">
         <v>165</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="50" t="s">
         <v>166</v>
       </c>
-      <c r="C3" s="16" t="s">
+      <c r="C3" s="50" t="s">
         <v>167</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="50" t="s">
         <v>168</v>
       </c>
-      <c r="E3" s="16" t="s">
+      <c r="E3" s="50" t="s">
         <v>169</v>
       </c>
     </row>
@@ -2875,74 +2617,74 @@
     <tabColor rgb="FFFEE7FC"/>
   </sheetPr>
   <dimension ref="A1:S12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="17.5" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="5" width="11.42578125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="13.7109375" style="11" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.140625" style="12" customWidth="1"/>
-    <col min="8" max="9" width="11.42578125" style="2" customWidth="1"/>
-    <col min="10" max="16384" width="11.42578125" style="2"/>
+    <col min="1" max="5" width="11.453125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="13.7265625" style="7" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.1796875" style="8" customWidth="1"/>
+    <col min="8" max="9" width="11.453125" style="2" customWidth="1"/>
+    <col min="10" max="16384" width="11.453125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="21" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="73" t="s">
+    <row r="1" spans="1:19" s="15" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="37" t="s">
         <v>154</v>
       </c>
-      <c r="B1" s="73"/>
-      <c r="C1" s="73"/>
-      <c r="D1" s="73"/>
-      <c r="E1" s="73"/>
-      <c r="F1" s="73"/>
-      <c r="G1" s="73"/>
-      <c r="H1" s="73"/>
-      <c r="I1" s="73"/>
-      <c r="J1" s="73"/>
-      <c r="K1" s="73"/>
-      <c r="L1" s="73"/>
-      <c r="M1" s="73"/>
-      <c r="N1" s="73"/>
-      <c r="O1" s="73"/>
-      <c r="P1" s="73"/>
-      <c r="Q1" s="73"/>
-      <c r="R1" s="73"/>
-      <c r="S1" s="73"/>
-    </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A2" s="51" t="s">
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="37"/>
+      <c r="H1" s="37"/>
+      <c r="I1" s="37"/>
+      <c r="J1" s="37"/>
+      <c r="K1" s="37"/>
+      <c r="L1" s="37"/>
+      <c r="M1" s="37"/>
+      <c r="N1" s="37"/>
+      <c r="O1" s="37"/>
+      <c r="P1" s="37"/>
+      <c r="Q1" s="37"/>
+      <c r="R1" s="37"/>
+      <c r="S1" s="37"/>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.5">
+      <c r="A2" s="42" t="s">
         <v>146</v>
       </c>
-      <c r="B2" s="52"/>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
-      <c r="E2" s="52"/>
-      <c r="F2" s="53"/>
-      <c r="G2" s="58" t="s">
+      <c r="B2" s="42"/>
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="3" spans="1:19" ht="89.25" x14ac:dyDescent="0.35">
-      <c r="A3" s="15" t="s">
+    <row r="3" spans="1:19" ht="62.5" x14ac:dyDescent="0.5">
+      <c r="A3" s="50" t="s">
         <v>147</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="50" t="s">
         <v>148</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="50" t="s">
         <v>149</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="50" t="s">
         <v>150</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="E3" s="50" t="s">
         <v>151</v>
       </c>
-      <c r="F3" s="16" t="s">
+      <c r="F3" s="50" t="s">
         <v>152</v>
       </c>
-      <c r="G3" s="59"/>
-    </row>
-    <row r="12" spans="1:19" ht="72.75" x14ac:dyDescent="1.25">
-      <c r="I12" s="22"/>
+      <c r="G3" s="42"/>
+    </row>
+    <row r="12" spans="1:19" ht="74" x14ac:dyDescent="1.95">
+      <c r="I12" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2969,74 +2711,75 @@
     <tabColor rgb="FFFEE7FC"/>
   </sheetPr>
   <dimension ref="A1:S12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="17.5" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="5" width="11.42578125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="13.7109375" style="11" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="23.85546875" style="12" customWidth="1"/>
-    <col min="8" max="9" width="11.42578125" style="2" customWidth="1"/>
-    <col min="10" max="16384" width="11.42578125" style="2"/>
+    <col min="1" max="1" width="11.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="5" width="11.453125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="13.7265625" style="7" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.81640625" style="8" customWidth="1"/>
+    <col min="8" max="9" width="11.453125" style="2" customWidth="1"/>
+    <col min="10" max="16384" width="11.453125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="21" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="73" t="s">
+    <row r="1" spans="1:19" s="15" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="37" t="s">
         <v>180</v>
       </c>
-      <c r="B1" s="73"/>
-      <c r="C1" s="73"/>
-      <c r="D1" s="73"/>
-      <c r="E1" s="73"/>
-      <c r="F1" s="73"/>
-      <c r="G1" s="73"/>
-      <c r="H1" s="73"/>
-      <c r="I1" s="73"/>
-      <c r="J1" s="73"/>
-      <c r="K1" s="73"/>
-      <c r="L1" s="73"/>
-      <c r="M1" s="73"/>
-      <c r="N1" s="73"/>
-      <c r="O1" s="73"/>
-      <c r="P1" s="73"/>
-      <c r="Q1" s="73"/>
-      <c r="R1" s="73"/>
-      <c r="S1" s="73"/>
-    </row>
-    <row r="2" spans="1:19" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="51" t="s">
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="37"/>
+      <c r="H1" s="37"/>
+      <c r="I1" s="37"/>
+      <c r="J1" s="37"/>
+      <c r="K1" s="37"/>
+      <c r="L1" s="37"/>
+      <c r="M1" s="37"/>
+      <c r="N1" s="37"/>
+      <c r="O1" s="37"/>
+      <c r="P1" s="37"/>
+      <c r="Q1" s="37"/>
+      <c r="R1" s="37"/>
+      <c r="S1" s="37"/>
+    </row>
+    <row r="2" spans="1:19" ht="33" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A2" s="42" t="s">
         <v>172</v>
       </c>
-      <c r="B2" s="52"/>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
-      <c r="E2" s="52"/>
-      <c r="F2" s="53"/>
-      <c r="G2" s="58" t="s">
+      <c r="B2" s="42"/>
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="3" spans="1:19" ht="127.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="15" t="s">
+    <row r="3" spans="1:19" ht="112.5" x14ac:dyDescent="0.5">
+      <c r="A3" s="50" t="s">
         <v>173</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="50" t="s">
         <v>174</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="50" t="s">
         <v>175</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="50" t="s">
         <v>176</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="E3" s="50" t="s">
         <v>178</v>
       </c>
-      <c r="F3" s="16" t="s">
+      <c r="F3" s="50" t="s">
         <v>177</v>
       </c>
-      <c r="G3" s="59"/>
-    </row>
-    <row r="12" spans="1:19" ht="72.75" x14ac:dyDescent="1.25">
-      <c r="I12" s="22"/>
+      <c r="G3" s="42"/>
+    </row>
+    <row r="12" spans="1:19" ht="74" x14ac:dyDescent="1.95">
+      <c r="I12" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -3063,44 +2806,44 @@
     <tabColor rgb="FFE8EDFF"/>
   </sheetPr>
   <dimension ref="A1:O3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="17.5" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="22.28515625" style="11" customWidth="1"/>
-    <col min="2" max="2" width="26.42578125" style="24" customWidth="1"/>
-    <col min="3" max="5" width="11.42578125" style="2" customWidth="1"/>
-    <col min="6" max="16384" width="11.42578125" style="2"/>
+    <col min="1" max="1" width="22.26953125" style="7" customWidth="1"/>
+    <col min="2" max="2" width="26.453125" style="18" customWidth="1"/>
+    <col min="3" max="5" width="11.453125" style="2" customWidth="1"/>
+    <col min="6" max="16384" width="11.453125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="23" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="78" t="s">
+    <row r="1" spans="1:15" s="17" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="40" t="s">
         <v>68</v>
       </c>
-      <c r="B1" s="78"/>
-      <c r="C1" s="78"/>
-      <c r="D1" s="78"/>
-      <c r="E1" s="78"/>
-      <c r="F1" s="78"/>
-      <c r="G1" s="78"/>
-      <c r="H1" s="78"/>
-      <c r="I1" s="78"/>
-      <c r="J1" s="78"/>
-      <c r="K1" s="78"/>
-      <c r="L1" s="78"/>
-      <c r="M1" s="78"/>
-      <c r="N1" s="78"/>
-      <c r="O1" s="78"/>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A2" s="74" t="s">
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
+      <c r="I1" s="40"/>
+      <c r="J1" s="40"/>
+      <c r="K1" s="40"/>
+      <c r="L1" s="40"/>
+      <c r="M1" s="40"/>
+      <c r="N1" s="40"/>
+      <c r="O1" s="40"/>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.5">
+      <c r="A2" s="41" t="s">
         <v>69</v>
       </c>
-      <c r="B2" s="76" t="s">
+      <c r="B2" s="41" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="55.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="75"/>
-      <c r="B3" s="77"/>
+    <row r="3" spans="1:15" ht="55.5" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A3" s="41"/>
+      <c r="B3" s="41"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -3119,177 +2862,182 @@
     <tabColor rgb="FFFFEDC3"/>
   </sheetPr>
   <dimension ref="A1:AB3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7109375" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7265625" defaultRowHeight="17.5" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="19" style="11" customWidth="1"/>
-    <col min="2" max="2" width="16.85546875" style="12" customWidth="1"/>
-    <col min="3" max="3" width="15.7109375" style="12"/>
-    <col min="4" max="7" width="15.7109375" style="2"/>
-    <col min="8" max="8" width="15.7109375" style="12"/>
-    <col min="9" max="10" width="15.7109375" style="2"/>
-    <col min="11" max="12" width="15.7109375" style="13"/>
-    <col min="13" max="13" width="15.7109375" style="12"/>
-    <col min="14" max="15" width="15.7109375" style="2"/>
-    <col min="16" max="16" width="15.7109375" style="13"/>
-    <col min="17" max="17" width="15.7109375" style="14"/>
-    <col min="18" max="22" width="15.7109375" style="2"/>
-    <col min="23" max="23" width="15.7109375" style="12"/>
-    <col min="24" max="27" width="15.7109375" style="2"/>
-    <col min="28" max="28" width="15.7109375" style="12"/>
-    <col min="29" max="16384" width="15.7109375" style="2"/>
+    <col min="1" max="1" width="19" style="7" customWidth="1"/>
+    <col min="2" max="2" width="16.81640625" style="8" customWidth="1"/>
+    <col min="3" max="3" width="15.7265625" style="8"/>
+    <col min="4" max="7" width="15.7265625" style="2"/>
+    <col min="8" max="8" width="15.7265625" style="8"/>
+    <col min="9" max="10" width="15.7265625" style="2"/>
+    <col min="11" max="12" width="15.7265625" style="9"/>
+    <col min="13" max="13" width="15.7265625" style="8"/>
+    <col min="14" max="15" width="15.7265625" style="2"/>
+    <col min="16" max="16" width="15.7265625" style="9"/>
+    <col min="17" max="17" width="15.7265625" style="10"/>
+    <col min="18" max="22" width="15.7265625" style="2"/>
+    <col min="23" max="23" width="15.7265625" style="8"/>
+    <col min="24" max="27" width="15.7265625" style="2"/>
+    <col min="28" max="28" width="15.7265625" style="8"/>
+    <col min="29" max="16384" width="15.7265625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="10" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="48" t="s">
+    <row r="1" spans="1:28" s="6" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
-      <c r="H1" s="48"/>
-      <c r="I1" s="48"/>
-      <c r="J1" s="48"/>
-      <c r="K1" s="48"/>
-      <c r="L1" s="48"/>
-      <c r="M1" s="48"/>
-      <c r="N1" s="48"/>
-      <c r="O1" s="48"/>
-      <c r="P1" s="48"/>
-      <c r="Q1" s="48"/>
-      <c r="R1" s="48"/>
-      <c r="S1" s="48"/>
-    </row>
-    <row r="2" spans="1:28" s="19" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="57" t="s">
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
+      <c r="J1" s="35"/>
+      <c r="K1" s="35"/>
+      <c r="L1" s="35"/>
+      <c r="M1" s="35"/>
+      <c r="N1" s="35"/>
+      <c r="O1" s="35"/>
+      <c r="P1" s="35"/>
+      <c r="Q1" s="35"/>
+      <c r="R1" s="35"/>
+      <c r="S1" s="35"/>
+    </row>
+    <row r="2" spans="1:28" s="13" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A2" s="42" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="58" t="s">
+      <c r="B2" s="42" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="58" t="s">
+      <c r="C2" s="42" t="s">
         <v>19</v>
       </c>
-      <c r="D2" s="51" t="s">
+      <c r="D2" s="42" t="s">
         <v>20</v>
       </c>
-      <c r="E2" s="52"/>
-      <c r="F2" s="52"/>
-      <c r="G2" s="52"/>
-      <c r="H2" s="53"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
       <c r="I2" s="49" t="s">
         <v>31</v>
       </c>
-      <c r="J2" s="50"/>
-      <c r="K2" s="60" t="s">
+      <c r="J2" s="49"/>
+      <c r="K2" s="49" t="s">
         <v>90</v>
       </c>
-      <c r="L2" s="58" t="s">
+      <c r="L2" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="M2" s="60" t="s">
+      <c r="M2" s="49" t="s">
         <v>89</v>
       </c>
       <c r="N2" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="O2" s="50"/>
-      <c r="P2" s="60" t="s">
+      <c r="O2" s="49"/>
+      <c r="P2" s="49" t="s">
         <v>23</v>
       </c>
-      <c r="Q2" s="54" t="s">
+      <c r="Q2" s="49" t="s">
         <v>24</v>
       </c>
-      <c r="R2" s="55"/>
-      <c r="S2" s="55"/>
-      <c r="T2" s="55"/>
-      <c r="U2" s="55"/>
-      <c r="V2" s="55"/>
-      <c r="W2" s="56"/>
-      <c r="X2" s="51" t="s">
+      <c r="R2" s="49"/>
+      <c r="S2" s="49"/>
+      <c r="T2" s="49"/>
+      <c r="U2" s="49"/>
+      <c r="V2" s="49"/>
+      <c r="W2" s="49"/>
+      <c r="X2" s="42" t="s">
         <v>25</v>
       </c>
-      <c r="Y2" s="52"/>
-      <c r="Z2" s="52"/>
-      <c r="AA2" s="52"/>
-      <c r="AB2" s="53"/>
-    </row>
-    <row r="3" spans="1:28" ht="38.25" x14ac:dyDescent="0.35">
-      <c r="A3" s="53"/>
-      <c r="B3" s="59"/>
-      <c r="C3" s="59"/>
-      <c r="D3" s="15" t="s">
+      <c r="Y2" s="42"/>
+      <c r="Z2" s="42"/>
+      <c r="AA2" s="42"/>
+      <c r="AB2" s="42"/>
+    </row>
+    <row r="3" spans="1:28" ht="37.5" x14ac:dyDescent="0.5">
+      <c r="A3" s="42"/>
+      <c r="B3" s="42"/>
+      <c r="C3" s="42"/>
+      <c r="D3" s="50" t="s">
         <v>26</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="E3" s="50" t="s">
         <v>27</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="F3" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="G3" s="15" t="s">
+      <c r="G3" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="H3" s="16" t="s">
+      <c r="H3" s="50" t="s">
         <v>30</v>
       </c>
-      <c r="I3" s="45" t="s">
+      <c r="I3" s="50" t="s">
         <v>31</v>
       </c>
-      <c r="J3" s="46" t="s">
+      <c r="J3" s="50" t="s">
         <v>73</v>
       </c>
-      <c r="K3" s="61"/>
-      <c r="L3" s="59"/>
-      <c r="M3" s="61"/>
-      <c r="N3" s="45" t="s">
+      <c r="K3" s="49"/>
+      <c r="L3" s="42"/>
+      <c r="M3" s="49"/>
+      <c r="N3" s="50" t="s">
         <v>74</v>
       </c>
-      <c r="O3" s="46" t="s">
+      <c r="O3" s="50" t="s">
         <v>22</v>
       </c>
-      <c r="P3" s="61"/>
-      <c r="Q3" s="17" t="s">
+      <c r="P3" s="49"/>
+      <c r="Q3" s="50" t="s">
         <v>72</v>
       </c>
-      <c r="R3" s="15" t="s">
+      <c r="R3" s="50" t="s">
         <v>32</v>
       </c>
-      <c r="S3" s="15" t="s">
+      <c r="S3" s="50" t="s">
         <v>33</v>
       </c>
-      <c r="T3" s="15" t="s">
+      <c r="T3" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="U3" s="15" t="s">
+      <c r="U3" s="50" t="s">
         <v>34</v>
       </c>
-      <c r="V3" s="15" t="s">
+      <c r="V3" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="W3" s="16" t="s">
+      <c r="W3" s="50" t="s">
         <v>35</v>
       </c>
-      <c r="X3" s="18" t="s">
+      <c r="X3" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="Y3" s="18" t="s">
+      <c r="Y3" s="50" t="s">
         <v>37</v>
       </c>
-      <c r="Z3" s="18" t="s">
+      <c r="Z3" s="50" t="s">
         <v>38</v>
       </c>
-      <c r="AA3" s="18" t="s">
+      <c r="AA3" s="50" t="s">
         <v>39</v>
       </c>
-      <c r="AB3" s="16" t="s">
+      <c r="AB3" s="50" t="s">
         <v>30</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="A1:S1"/>
+    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="Q2:W2"/>
     <mergeCell ref="X2:AB2"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="B2:B3"/>
@@ -3298,11 +3046,6 @@
     <mergeCell ref="M2:M3"/>
     <mergeCell ref="P2:P3"/>
     <mergeCell ref="K2:K3"/>
-    <mergeCell ref="A1:S1"/>
-    <mergeCell ref="N2:O2"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="Q2:W2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -3315,68 +3058,68 @@
     <tabColor rgb="FFE8EDFF"/>
   </sheetPr>
   <dimension ref="A1:L3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7109375" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7265625" defaultRowHeight="17.5" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="15.7109375" style="1"/>
-    <col min="2" max="6" width="15.7109375" style="2"/>
-    <col min="7" max="7" width="15.7109375" style="12"/>
-    <col min="8" max="8" width="18.140625" style="12" customWidth="1"/>
-    <col min="9" max="16384" width="15.7109375" style="2"/>
+    <col min="1" max="1" width="15.7265625" style="1"/>
+    <col min="2" max="6" width="15.7265625" style="2"/>
+    <col min="7" max="7" width="15.7265625" style="8"/>
+    <col min="8" max="8" width="78.81640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="15.7265625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="23" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="78" t="s">
+    <row r="1" spans="1:12" s="17" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="40" t="s">
         <v>163</v>
       </c>
-      <c r="B1" s="78"/>
-      <c r="C1" s="78"/>
-      <c r="D1" s="78"/>
-      <c r="E1" s="78"/>
-      <c r="F1" s="78"/>
-      <c r="G1" s="78"/>
-      <c r="H1" s="78"/>
-      <c r="I1" s="78"/>
-      <c r="J1" s="78"/>
-      <c r="K1" s="78"/>
-      <c r="L1" s="78"/>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A2" s="51" t="s">
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
+      <c r="I1" s="40"/>
+      <c r="J1" s="40"/>
+      <c r="K1" s="40"/>
+      <c r="L1" s="40"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A2" s="42" t="s">
         <v>162</v>
       </c>
-      <c r="B2" s="52"/>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
-      <c r="E2" s="52"/>
-      <c r="F2" s="52"/>
-      <c r="G2" s="53"/>
-      <c r="H2" s="57" t="s">
+      <c r="B2" s="42"/>
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="63.75" x14ac:dyDescent="0.35">
-      <c r="A3" s="15" t="s">
+    <row r="3" spans="1:12" ht="62.5" x14ac:dyDescent="0.5">
+      <c r="A3" s="50" t="s">
         <v>155</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="50" t="s">
         <v>156</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="50" t="s">
         <v>157</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="50" t="s">
         <v>158</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="E3" s="50" t="s">
         <v>159</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="F3" s="50" t="s">
         <v>164</v>
       </c>
-      <c r="G3" s="16" t="s">
+      <c r="G3" s="50" t="s">
         <v>160</v>
       </c>
-      <c r="H3" s="53"/>
+      <c r="H3" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -3400,38 +3143,38 @@
     <tabColor rgb="FFE8EDFF"/>
   </sheetPr>
   <dimension ref="A1:N3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="17.5" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="22.28515625" style="11" customWidth="1"/>
-    <col min="2" max="4" width="11.42578125" style="2" customWidth="1"/>
-    <col min="5" max="16384" width="11.42578125" style="2"/>
+    <col min="1" max="1" width="22.26953125" style="7" customWidth="1"/>
+    <col min="2" max="4" width="11.453125" style="2" customWidth="1"/>
+    <col min="5" max="16384" width="11.453125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="23" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="78" t="s">
+    <row r="1" spans="1:14" s="17" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="40" t="s">
         <v>144</v>
       </c>
-      <c r="B1" s="78"/>
-      <c r="C1" s="78"/>
-      <c r="D1" s="78"/>
-      <c r="E1" s="78"/>
-      <c r="F1" s="78"/>
-      <c r="G1" s="78"/>
-      <c r="H1" s="78"/>
-      <c r="I1" s="78"/>
-      <c r="J1" s="78"/>
-      <c r="K1" s="78"/>
-      <c r="L1" s="78"/>
-      <c r="M1" s="78"/>
-      <c r="N1" s="78"/>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A2" s="74" t="s">
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
+      <c r="I1" s="40"/>
+      <c r="J1" s="40"/>
+      <c r="K1" s="40"/>
+      <c r="L1" s="40"/>
+      <c r="M1" s="40"/>
+      <c r="N1" s="40"/>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.5">
+      <c r="A2" s="38" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="55.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="75"/>
+    <row r="3" spans="1:14" ht="55.5" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A3" s="39"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3449,153 +3192,187 @@
     <tabColor rgb="FFFFEDC3"/>
   </sheetPr>
   <dimension ref="A1:O14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7109375" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7265625" defaultRowHeight="17.5" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="20.28515625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="19.85546875" style="24" customWidth="1"/>
-    <col min="3" max="3" width="19.42578125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="38.28515625" style="14" customWidth="1"/>
-    <col min="5" max="5" width="92.5703125" style="2" customWidth="1"/>
-    <col min="6" max="6" width="15.7109375" style="2"/>
-    <col min="7" max="7" width="20.42578125" style="12" customWidth="1"/>
-    <col min="8" max="16384" width="15.7109375" style="2"/>
+    <col min="1" max="1" width="20.26953125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="19.81640625" style="18" customWidth="1"/>
+    <col min="3" max="3" width="19.453125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="38.26953125" style="10" customWidth="1"/>
+    <col min="5" max="5" width="92.54296875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="15.7265625" style="2"/>
+    <col min="7" max="7" width="20.453125" style="8" customWidth="1"/>
+    <col min="8" max="16384" width="15.7265625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="10" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="48" t="s">
+    <row r="1" spans="1:15" s="6" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
-      <c r="H1" s="48"/>
-      <c r="I1" s="48"/>
-      <c r="J1" s="48"/>
-      <c r="K1" s="48"/>
-      <c r="L1" s="48"/>
-      <c r="M1" s="48"/>
-      <c r="N1" s="48"/>
-      <c r="O1" s="48"/>
-    </row>
-    <row r="2" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="62" t="s">
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
+      <c r="J1" s="35"/>
+      <c r="K1" s="35"/>
+      <c r="L1" s="35"/>
+      <c r="M1" s="35"/>
+      <c r="N1" s="35"/>
+      <c r="O1" s="35"/>
+    </row>
+    <row r="2" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A2" s="41" t="s">
         <v>75</v>
       </c>
-      <c r="B2" s="58" t="s">
+      <c r="B2" s="42" t="s">
         <v>76</v>
       </c>
-      <c r="C2" s="64" t="s">
+      <c r="C2" s="42" t="s">
         <v>77</v>
       </c>
-      <c r="D2" s="65" t="s">
+      <c r="D2" s="42" t="s">
         <v>78</v>
       </c>
-      <c r="E2" s="66"/>
-      <c r="F2" s="66"/>
-      <c r="G2" s="67"/>
-    </row>
-    <row r="3" spans="1:15" ht="41.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="63"/>
-      <c r="B3" s="59"/>
-      <c r="C3" s="52"/>
-      <c r="D3" s="51"/>
-      <c r="E3" s="52"/>
-      <c r="F3" s="52"/>
-      <c r="G3" s="53"/>
-    </row>
-    <row r="4" spans="1:15" ht="48" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="E4" s="25" t="s">
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+    </row>
+    <row r="3" spans="1:15" ht="41.25" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A3" s="41"/>
+      <c r="B3" s="42"/>
+      <c r="C3" s="42"/>
+      <c r="D3" s="42"/>
+      <c r="E3" s="42"/>
+      <c r="F3" s="42"/>
+      <c r="G3" s="42"/>
+    </row>
+    <row r="4" spans="1:15" ht="48" x14ac:dyDescent="0.5">
+      <c r="A4" s="43"/>
+      <c r="B4" s="43"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="44"/>
+      <c r="E4" s="45" t="s">
         <v>2</v>
       </c>
-      <c r="F4" s="26" t="s">
+      <c r="F4" s="45" t="s">
         <v>1</v>
       </c>
-      <c r="G4" s="27" t="s">
+      <c r="G4" s="45" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="D5" s="28" t="s">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.5">
+      <c r="A5" s="43"/>
+      <c r="B5" s="43"/>
+      <c r="C5" s="44"/>
+      <c r="D5" s="46" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="29"/>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="D6" s="30" t="s">
+      <c r="E5" s="43"/>
+      <c r="F5" s="43"/>
+      <c r="G5" s="43"/>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.5">
+      <c r="A6" s="43"/>
+      <c r="B6" s="43"/>
+      <c r="C6" s="44"/>
+      <c r="D6" s="46" t="s">
         <v>5</v>
       </c>
-      <c r="E6" s="4"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="29"/>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="D7" s="31" t="s">
+      <c r="E6" s="43"/>
+      <c r="F6" s="43"/>
+      <c r="G6" s="43"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.5">
+      <c r="A7" s="43"/>
+      <c r="B7" s="43"/>
+      <c r="C7" s="44"/>
+      <c r="D7" s="46" t="s">
         <v>6</v>
       </c>
-      <c r="E7" s="9"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="29"/>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="D8" s="31" t="s">
+      <c r="E7" s="43"/>
+      <c r="F7" s="43"/>
+      <c r="G7" s="43"/>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.5">
+      <c r="A8" s="43"/>
+      <c r="B8" s="43"/>
+      <c r="C8" s="44"/>
+      <c r="D8" s="46" t="s">
         <v>7</v>
       </c>
-      <c r="E8" s="9"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="29"/>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="D9" s="31" t="s">
+      <c r="E8" s="43"/>
+      <c r="F8" s="43"/>
+      <c r="G8" s="43"/>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.5">
+      <c r="A9" s="43"/>
+      <c r="B9" s="43"/>
+      <c r="C9" s="44"/>
+      <c r="D9" s="46" t="s">
         <v>8</v>
       </c>
-      <c r="E9" s="9"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="29"/>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="D10" s="32" t="s">
+      <c r="E9" s="43"/>
+      <c r="F9" s="43"/>
+      <c r="G9" s="43"/>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.5">
+      <c r="A10" s="43"/>
+      <c r="B10" s="43"/>
+      <c r="C10" s="44"/>
+      <c r="D10" s="47" t="s">
         <v>9</v>
       </c>
-      <c r="E10" s="9"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="29"/>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="D11" s="32" t="s">
+      <c r="E10" s="43"/>
+      <c r="F10" s="43"/>
+      <c r="G10" s="43"/>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.5">
+      <c r="A11" s="43"/>
+      <c r="B11" s="43"/>
+      <c r="C11" s="44"/>
+      <c r="D11" s="47" t="s">
         <v>10</v>
       </c>
-      <c r="E11" s="9"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="29"/>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="D12" s="32" t="s">
+      <c r="E11" s="43"/>
+      <c r="F11" s="43"/>
+      <c r="G11" s="43"/>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.5">
+      <c r="A12" s="43"/>
+      <c r="B12" s="43"/>
+      <c r="C12" s="44"/>
+      <c r="D12" s="47" t="s">
         <v>11</v>
       </c>
-      <c r="E12" s="9"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="29"/>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="D13" s="32" t="s">
+      <c r="E12" s="43"/>
+      <c r="F12" s="43"/>
+      <c r="G12" s="43"/>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.5">
+      <c r="A13" s="43"/>
+      <c r="B13" s="43"/>
+      <c r="C13" s="44"/>
+      <c r="D13" s="47" t="s">
         <v>12</v>
       </c>
-      <c r="E13" s="9"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="29"/>
-    </row>
-    <row r="14" spans="1:15" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="D14" s="33" t="s">
+      <c r="E13" s="43"/>
+      <c r="F13" s="43"/>
+      <c r="G13" s="43"/>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.5">
+      <c r="A14" s="43"/>
+      <c r="B14" s="43"/>
+      <c r="C14" s="44"/>
+      <c r="D14" s="48" t="s">
         <v>13</v>
       </c>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="34"/>
+      <c r="E14" s="43"/>
+      <c r="F14" s="43"/>
+      <c r="G14" s="43"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -3621,50 +3398,50 @@
     <tabColor rgb="FFFFEDC3"/>
   </sheetPr>
   <dimension ref="A1:M3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7109375" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7265625" defaultRowHeight="17.5" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="19" style="11" customWidth="1"/>
-    <col min="2" max="3" width="16.85546875" style="12" customWidth="1"/>
-    <col min="4" max="4" width="15.7109375" style="12"/>
-    <col min="5" max="16384" width="15.7109375" style="2"/>
+    <col min="1" max="1" width="19" style="7" customWidth="1"/>
+    <col min="2" max="3" width="16.81640625" style="8" customWidth="1"/>
+    <col min="4" max="4" width="15.7265625" style="8"/>
+    <col min="5" max="16384" width="15.7265625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="10" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="48" t="s">
+    <row r="1" spans="1:13" s="6" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="35" t="s">
         <v>143</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
-      <c r="H1" s="48"/>
-      <c r="I1" s="48"/>
-      <c r="J1" s="48"/>
-      <c r="K1" s="48"/>
-      <c r="L1" s="48"/>
-      <c r="M1" s="48"/>
-    </row>
-    <row r="2" spans="1:13" s="19" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="57" t="s">
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
+      <c r="J1" s="35"/>
+      <c r="K1" s="35"/>
+      <c r="L1" s="35"/>
+      <c r="M1" s="35"/>
+    </row>
+    <row r="2" spans="1:13" s="13" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A2" s="42" t="s">
         <v>139</v>
       </c>
-      <c r="B2" s="58" t="s">
+      <c r="B2" s="42" t="s">
         <v>140</v>
       </c>
-      <c r="C2" s="58" t="s">
+      <c r="C2" s="42" t="s">
         <v>141</v>
       </c>
-      <c r="D2" s="58" t="s">
+      <c r="D2" s="42" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A3" s="53"/>
-      <c r="B3" s="59"/>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.5">
+      <c r="A3" s="42"/>
+      <c r="B3" s="42"/>
+      <c r="C3" s="42"/>
+      <c r="D3" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -3685,136 +3462,137 @@
     <tabColor rgb="FFFFEDC3"/>
   </sheetPr>
   <dimension ref="A1:M14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7109375" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7265625" defaultRowHeight="17.5" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="38.28515625" style="14" customWidth="1"/>
-    <col min="2" max="2" width="23.7109375" style="2" customWidth="1"/>
-    <col min="3" max="3" width="21.85546875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="20.42578125" style="12" customWidth="1"/>
-    <col min="5" max="16384" width="15.7109375" style="2"/>
+    <col min="1" max="1" width="38.26953125" style="10" customWidth="1"/>
+    <col min="2" max="2" width="23.7265625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="21.81640625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="20.453125" style="8" customWidth="1"/>
+    <col min="5" max="16384" width="15.7265625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="10" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="48" t="s">
+    <row r="1" spans="1:13" s="6" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="35" t="s">
         <v>228</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
-      <c r="H1" s="48"/>
-      <c r="I1" s="48"/>
-      <c r="J1" s="48"/>
-      <c r="K1" s="48"/>
-      <c r="L1" s="48"/>
-      <c r="M1" s="48"/>
-    </row>
-    <row r="2" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="65" t="s">
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
+      <c r="J1" s="35"/>
+      <c r="K1" s="35"/>
+      <c r="L1" s="35"/>
+      <c r="M1" s="35"/>
+    </row>
+    <row r="2" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A2" s="42" t="s">
         <v>227</v>
       </c>
-      <c r="B2" s="66"/>
-      <c r="C2" s="66"/>
-      <c r="D2" s="67"/>
-    </row>
-    <row r="3" spans="1:13" ht="41.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="51"/>
-      <c r="B3" s="52"/>
-      <c r="C3" s="52"/>
-      <c r="D3" s="53"/>
-    </row>
-    <row r="4" spans="1:13" ht="79.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B4" s="25" t="s">
+      <c r="B2" s="42"/>
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+    </row>
+    <row r="3" spans="1:13" ht="41.25" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A3" s="42"/>
+      <c r="B3" s="42"/>
+      <c r="C3" s="42"/>
+      <c r="D3" s="42"/>
+    </row>
+    <row r="4" spans="1:13" ht="80" x14ac:dyDescent="0.5">
+      <c r="A4" s="44"/>
+      <c r="B4" s="45" t="s">
         <v>224</v>
       </c>
-      <c r="C4" s="26" t="s">
+      <c r="C4" s="45" t="s">
         <v>225</v>
       </c>
-      <c r="D4" s="27" t="s">
+      <c r="D4" s="45" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A5" s="28" t="s">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.5">
+      <c r="A5" s="46" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="29"/>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A6" s="30" t="s">
+      <c r="B5" s="43"/>
+      <c r="C5" s="43"/>
+      <c r="D5" s="43"/>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.5">
+      <c r="A6" s="46" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="4"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="29"/>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A7" s="31" t="s">
+      <c r="B6" s="43"/>
+      <c r="C6" s="43"/>
+      <c r="D6" s="43"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.5">
+      <c r="A7" s="46" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="9"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="29"/>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A8" s="31" t="s">
+      <c r="B7" s="43"/>
+      <c r="C7" s="43"/>
+      <c r="D7" s="43"/>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.5">
+      <c r="A8" s="46" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="9"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="29"/>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A9" s="31" t="s">
+      <c r="B8" s="43"/>
+      <c r="C8" s="43"/>
+      <c r="D8" s="43"/>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.5">
+      <c r="A9" s="46" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="9"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="29"/>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A10" s="32" t="s">
+      <c r="B9" s="43"/>
+      <c r="C9" s="43"/>
+      <c r="D9" s="43"/>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.5">
+      <c r="A10" s="47" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="9"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="29"/>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A11" s="32" t="s">
+      <c r="B10" s="43"/>
+      <c r="C10" s="43"/>
+      <c r="D10" s="43"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.5">
+      <c r="A11" s="47" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="9"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="29"/>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A12" s="32" t="s">
+      <c r="B11" s="43"/>
+      <c r="C11" s="43"/>
+      <c r="D11" s="43"/>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.5">
+      <c r="A12" s="47" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="9"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="29"/>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A13" s="32" t="s">
+      <c r="B12" s="43"/>
+      <c r="C12" s="43"/>
+      <c r="D12" s="43"/>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.5">
+      <c r="A13" s="47" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="9"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="29"/>
-    </row>
-    <row r="14" spans="1:13" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="33" t="s">
+      <c r="B13" s="43"/>
+      <c r="C13" s="43"/>
+      <c r="D13" s="43"/>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.5">
+      <c r="A14" s="48" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="34"/>
+      <c r="B14" s="43"/>
+      <c r="C14" s="43"/>
+      <c r="D14" s="43"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3832,247 +3610,247 @@
     <tabColor rgb="FFB8FEC9"/>
   </sheetPr>
   <dimension ref="A1:AL4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7109375" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7265625" defaultRowHeight="17.5" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="2" width="15.7109375" style="1"/>
-    <col min="3" max="3" width="15.7109375" style="12"/>
-    <col min="4" max="10" width="15.7109375" style="2"/>
-    <col min="11" max="11" width="15.7109375" style="12"/>
-    <col min="12" max="12" width="15.7109375" style="2" customWidth="1"/>
-    <col min="13" max="13" width="15.7109375" style="2"/>
-    <col min="14" max="14" width="15.7109375" style="12"/>
-    <col min="15" max="16" width="15.7109375" style="2"/>
-    <col min="17" max="17" width="15.7109375" style="12"/>
-    <col min="18" max="19" width="15.7109375" style="1"/>
-    <col min="20" max="20" width="15.7109375" style="11"/>
-    <col min="21" max="21" width="15.7109375" style="12"/>
-    <col min="22" max="36" width="15.7109375" style="1"/>
-    <col min="37" max="37" width="15.7109375" style="24"/>
-    <col min="38" max="38" width="15.7109375" style="12"/>
-    <col min="39" max="16384" width="15.7109375" style="2"/>
+    <col min="1" max="2" width="15.7265625" style="1"/>
+    <col min="3" max="3" width="15.7265625" style="8"/>
+    <col min="4" max="10" width="15.7265625" style="2"/>
+    <col min="11" max="11" width="15.7265625" style="8"/>
+    <col min="12" max="12" width="15.7265625" style="2" customWidth="1"/>
+    <col min="13" max="13" width="15.7265625" style="2"/>
+    <col min="14" max="14" width="15.7265625" style="8"/>
+    <col min="15" max="16" width="15.7265625" style="2"/>
+    <col min="17" max="17" width="15.7265625" style="8"/>
+    <col min="18" max="19" width="15.7265625" style="1"/>
+    <col min="20" max="20" width="15.7265625" style="7"/>
+    <col min="21" max="21" width="15.7265625" style="8"/>
+    <col min="22" max="36" width="15.7265625" style="1"/>
+    <col min="37" max="37" width="15.7265625" style="18"/>
+    <col min="38" max="38" width="15.7265625" style="8"/>
+    <col min="39" max="16384" width="15.7265625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:38" s="20" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="72" t="s">
+    <row r="1" spans="1:38" s="14" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="36" t="s">
         <v>119</v>
       </c>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="D1" s="72"/>
-      <c r="E1" s="72"/>
-      <c r="F1" s="72"/>
-      <c r="G1" s="72"/>
-      <c r="H1" s="72"/>
-      <c r="I1" s="72"/>
-      <c r="J1" s="72"/>
-      <c r="K1" s="72"/>
-      <c r="L1" s="72"/>
-      <c r="M1" s="72"/>
-      <c r="R1" s="44"/>
-      <c r="S1" s="44"/>
-      <c r="T1" s="44"/>
-      <c r="U1" s="44"/>
-      <c r="V1" s="44"/>
-      <c r="W1" s="44"/>
-      <c r="X1" s="44"/>
-      <c r="Y1" s="44"/>
-      <c r="Z1" s="44"/>
-      <c r="AA1" s="44"/>
-      <c r="AB1" s="44"/>
-      <c r="AC1" s="44"/>
-      <c r="AD1" s="44"/>
-      <c r="AE1" s="44"/>
-      <c r="AF1" s="44"/>
-      <c r="AG1" s="44"/>
-      <c r="AH1" s="44"/>
-      <c r="AI1" s="44"/>
-      <c r="AJ1" s="44"/>
-      <c r="AK1" s="44"/>
-      <c r="AL1" s="44"/>
-    </row>
-    <row r="2" spans="1:38" ht="35.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="52" t="s">
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
+      <c r="I1" s="36"/>
+      <c r="J1" s="36"/>
+      <c r="K1" s="36"/>
+      <c r="L1" s="36"/>
+      <c r="M1" s="36"/>
+      <c r="R1" s="24"/>
+      <c r="S1" s="24"/>
+      <c r="T1" s="24"/>
+      <c r="U1" s="24"/>
+      <c r="V1" s="24"/>
+      <c r="W1" s="24"/>
+      <c r="X1" s="24"/>
+      <c r="Y1" s="24"/>
+      <c r="Z1" s="24"/>
+      <c r="AA1" s="24"/>
+      <c r="AB1" s="24"/>
+      <c r="AC1" s="24"/>
+      <c r="AD1" s="24"/>
+      <c r="AE1" s="24"/>
+      <c r="AF1" s="24"/>
+      <c r="AG1" s="24"/>
+      <c r="AH1" s="24"/>
+      <c r="AI1" s="24"/>
+      <c r="AJ1" s="24"/>
+      <c r="AK1" s="24"/>
+      <c r="AL1" s="24"/>
+    </row>
+    <row r="2" spans="1:38" ht="35.25" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A2" s="42" t="s">
         <v>123</v>
       </c>
-      <c r="B2" s="52"/>
-      <c r="C2" s="53"/>
-      <c r="D2" s="69" t="s">
+      <c r="B2" s="42"/>
+      <c r="C2" s="42"/>
+      <c r="D2" s="51" t="s">
         <v>136</v>
       </c>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
-      <c r="I2" s="70"/>
-      <c r="J2" s="70"/>
-      <c r="K2" s="70"/>
-      <c r="L2" s="70"/>
-      <c r="M2" s="70"/>
-      <c r="N2" s="70"/>
-      <c r="O2" s="70"/>
-      <c r="P2" s="70"/>
-      <c r="Q2" s="71"/>
-      <c r="R2" s="52" t="s">
+      <c r="E2" s="51"/>
+      <c r="F2" s="51"/>
+      <c r="G2" s="51"/>
+      <c r="H2" s="51"/>
+      <c r="I2" s="51"/>
+      <c r="J2" s="51"/>
+      <c r="K2" s="51"/>
+      <c r="L2" s="51"/>
+      <c r="M2" s="51"/>
+      <c r="N2" s="51"/>
+      <c r="O2" s="51"/>
+      <c r="P2" s="51"/>
+      <c r="Q2" s="51"/>
+      <c r="R2" s="42" t="s">
         <v>192</v>
       </c>
-      <c r="S2" s="52"/>
-      <c r="T2" s="52"/>
-      <c r="U2" s="53"/>
-      <c r="V2" s="52" t="s">
+      <c r="S2" s="42"/>
+      <c r="T2" s="42"/>
+      <c r="U2" s="42"/>
+      <c r="V2" s="42" t="s">
         <v>193</v>
       </c>
-      <c r="W2" s="52"/>
-      <c r="X2" s="52"/>
-      <c r="Y2" s="52"/>
-      <c r="Z2" s="52"/>
-      <c r="AA2" s="52"/>
-      <c r="AB2" s="52"/>
-      <c r="AC2" s="52"/>
-      <c r="AD2" s="52"/>
-      <c r="AE2" s="52"/>
-      <c r="AF2" s="52"/>
-      <c r="AG2" s="52"/>
-      <c r="AH2" s="52"/>
-      <c r="AI2" s="52"/>
-      <c r="AJ2" s="52"/>
-      <c r="AK2" s="52"/>
-      <c r="AL2" s="53"/>
-    </row>
-    <row r="3" spans="1:38" ht="51" x14ac:dyDescent="0.35">
-      <c r="A3" s="15" t="s">
+      <c r="W2" s="42"/>
+      <c r="X2" s="42"/>
+      <c r="Y2" s="42"/>
+      <c r="Z2" s="42"/>
+      <c r="AA2" s="42"/>
+      <c r="AB2" s="42"/>
+      <c r="AC2" s="42"/>
+      <c r="AD2" s="42"/>
+      <c r="AE2" s="42"/>
+      <c r="AF2" s="42"/>
+      <c r="AG2" s="42"/>
+      <c r="AH2" s="42"/>
+      <c r="AI2" s="42"/>
+      <c r="AJ2" s="42"/>
+      <c r="AK2" s="42"/>
+      <c r="AL2" s="42"/>
+    </row>
+    <row r="3" spans="1:38" ht="50" x14ac:dyDescent="0.5">
+      <c r="A3" s="50" t="s">
         <v>120</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="50" t="s">
         <v>121</v>
       </c>
-      <c r="C3" s="16" t="s">
+      <c r="C3" s="50" t="s">
         <v>122</v>
       </c>
-      <c r="D3" s="68" t="s">
+      <c r="D3" s="52" t="s">
         <v>127</v>
       </c>
-      <c r="E3" s="68"/>
-      <c r="F3" s="68"/>
-      <c r="G3" s="68"/>
-      <c r="H3" s="68"/>
-      <c r="I3" s="68"/>
-      <c r="J3" s="68"/>
-      <c r="K3" s="68"/>
-      <c r="L3" s="68" t="s">
+      <c r="E3" s="52"/>
+      <c r="F3" s="52"/>
+      <c r="G3" s="52"/>
+      <c r="H3" s="52"/>
+      <c r="I3" s="52"/>
+      <c r="J3" s="52"/>
+      <c r="K3" s="52"/>
+      <c r="L3" s="52" t="s">
         <v>128</v>
       </c>
-      <c r="M3" s="68"/>
-      <c r="N3" s="68"/>
-      <c r="O3" s="68" t="s">
+      <c r="M3" s="52"/>
+      <c r="N3" s="52"/>
+      <c r="O3" s="52" t="s">
         <v>129</v>
       </c>
-      <c r="P3" s="68"/>
-      <c r="Q3" s="68"/>
-      <c r="R3" s="15" t="s">
+      <c r="P3" s="52"/>
+      <c r="Q3" s="52"/>
+      <c r="R3" s="50" t="s">
         <v>124</v>
       </c>
-      <c r="S3" s="15" t="s">
+      <c r="S3" s="50" t="s">
         <v>125</v>
       </c>
-      <c r="T3" s="16" t="s">
+      <c r="T3" s="50" t="s">
         <v>122</v>
       </c>
-      <c r="U3" s="16" t="s">
+      <c r="U3" s="50" t="s">
         <v>126</v>
       </c>
-      <c r="V3" s="15" t="s">
+      <c r="V3" s="50" t="s">
         <v>194</v>
       </c>
-      <c r="W3" s="15" t="s">
+      <c r="W3" s="50" t="s">
         <v>195</v>
       </c>
-      <c r="X3" s="15" t="s">
+      <c r="X3" s="50" t="s">
         <v>196</v>
       </c>
-      <c r="Y3" s="15" t="s">
+      <c r="Y3" s="50" t="s">
         <v>197</v>
       </c>
-      <c r="Z3" s="15" t="s">
+      <c r="Z3" s="50" t="s">
         <v>198</v>
       </c>
-      <c r="AA3" s="15" t="s">
+      <c r="AA3" s="50" t="s">
         <v>199</v>
       </c>
-      <c r="AB3" s="15" t="s">
+      <c r="AB3" s="50" t="s">
         <v>200</v>
       </c>
-      <c r="AC3" s="15" t="s">
+      <c r="AC3" s="50" t="s">
         <v>201</v>
       </c>
-      <c r="AD3" s="15" t="s">
+      <c r="AD3" s="50" t="s">
         <v>202</v>
       </c>
-      <c r="AE3" s="15" t="s">
+      <c r="AE3" s="50" t="s">
         <v>203</v>
       </c>
-      <c r="AF3" s="15" t="s">
+      <c r="AF3" s="50" t="s">
         <v>204</v>
       </c>
-      <c r="AG3" s="15" t="s">
+      <c r="AG3" s="50" t="s">
         <v>205</v>
       </c>
-      <c r="AH3" s="15" t="s">
+      <c r="AH3" s="50" t="s">
         <v>206</v>
       </c>
-      <c r="AI3" s="15" t="s">
+      <c r="AI3" s="50" t="s">
         <v>207</v>
       </c>
-      <c r="AJ3" s="15" t="s">
+      <c r="AJ3" s="50" t="s">
         <v>208</v>
       </c>
-      <c r="AK3" s="79" t="s">
+      <c r="AK3" s="50" t="s">
         <v>209</v>
       </c>
-      <c r="AL3" s="16" t="s">
+      <c r="AL3" s="50" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="4" spans="1:38" ht="25.5" x14ac:dyDescent="0.35">
-      <c r="D4" s="16" t="s">
+    <row r="4" spans="1:38" ht="25" x14ac:dyDescent="0.5">
+      <c r="D4" s="50" t="s">
         <v>130</v>
       </c>
-      <c r="E4" s="16" t="s">
+      <c r="E4" s="50" t="s">
         <v>131</v>
       </c>
-      <c r="F4" s="16" t="s">
+      <c r="F4" s="50" t="s">
         <v>132</v>
       </c>
-      <c r="G4" s="16" t="s">
+      <c r="G4" s="50" t="s">
         <v>137</v>
       </c>
-      <c r="H4" s="16" t="s">
+      <c r="H4" s="50" t="s">
         <v>138</v>
       </c>
-      <c r="I4" s="16" t="s">
+      <c r="I4" s="50" t="s">
         <v>133</v>
       </c>
-      <c r="J4" s="16" t="s">
+      <c r="J4" s="50" t="s">
         <v>42</v>
       </c>
-      <c r="K4" s="16" t="s">
+      <c r="K4" s="50" t="s">
         <v>134</v>
       </c>
-      <c r="L4" s="16" t="s">
+      <c r="L4" s="50" t="s">
         <v>130</v>
       </c>
-      <c r="M4" s="16" t="s">
+      <c r="M4" s="50" t="s">
         <v>132</v>
       </c>
-      <c r="N4" s="16" t="s">
+      <c r="N4" s="50" t="s">
         <v>135</v>
       </c>
-      <c r="O4" s="16" t="s">
+      <c r="O4" s="50" t="s">
         <v>120</v>
       </c>
-      <c r="P4" s="16" t="s">
+      <c r="P4" s="50" t="s">
         <v>121</v>
       </c>
-      <c r="Q4" s="16" t="s">
+      <c r="Q4" s="50" t="s">
         <v>122</v>
       </c>
     </row>
@@ -4098,80 +3876,80 @@
     <tabColor rgb="FFB8FEC9"/>
   </sheetPr>
   <dimension ref="A1:O3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="17.5" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="2" width="11.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" style="12" customWidth="1"/>
-    <col min="4" max="5" width="11.42578125" style="2" customWidth="1"/>
-    <col min="6" max="6" width="11.42578125" style="12"/>
-    <col min="7" max="7" width="11.42578125" style="14"/>
-    <col min="8" max="8" width="11.42578125" style="2"/>
-    <col min="9" max="9" width="11.42578125" style="12"/>
-    <col min="10" max="16384" width="11.42578125" style="2"/>
+    <col min="1" max="2" width="11.453125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="11.453125" style="8" customWidth="1"/>
+    <col min="4" max="5" width="11.453125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="11.453125" style="8"/>
+    <col min="7" max="7" width="11.453125" style="10"/>
+    <col min="8" max="8" width="11.453125" style="2"/>
+    <col min="9" max="9" width="11.453125" style="8"/>
+    <col min="10" max="16384" width="11.453125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="20" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="72" t="s">
+    <row r="1" spans="1:15" s="14" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="D1" s="72"/>
-      <c r="E1" s="72"/>
-      <c r="F1" s="72"/>
-      <c r="G1" s="72"/>
-      <c r="H1" s="72"/>
-      <c r="I1" s="72"/>
-      <c r="J1" s="72"/>
-      <c r="K1" s="72"/>
-      <c r="L1" s="72"/>
-      <c r="M1" s="72"/>
-      <c r="N1" s="72"/>
-      <c r="O1" s="72"/>
-    </row>
-    <row r="2" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="51" t="s">
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
+      <c r="I1" s="36"/>
+      <c r="J1" s="36"/>
+      <c r="K1" s="36"/>
+      <c r="L1" s="36"/>
+      <c r="M1" s="36"/>
+      <c r="N1" s="36"/>
+      <c r="O1" s="36"/>
+    </row>
+    <row r="2" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A2" s="42" t="s">
         <v>44</v>
       </c>
-      <c r="B2" s="52"/>
-      <c r="C2" s="53"/>
-      <c r="D2" s="51" t="s">
+      <c r="B2" s="42"/>
+      <c r="C2" s="42"/>
+      <c r="D2" s="42" t="s">
         <v>45</v>
       </c>
-      <c r="E2" s="52"/>
-      <c r="F2" s="53"/>
-      <c r="G2" s="51" t="s">
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42" t="s">
         <v>46</v>
       </c>
-      <c r="H2" s="52"/>
-      <c r="I2" s="53"/>
-    </row>
-    <row r="3" spans="1:15" ht="25.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="15" t="s">
+      <c r="H2" s="42"/>
+      <c r="I2" s="42"/>
+    </row>
+    <row r="3" spans="1:15" ht="25" x14ac:dyDescent="0.5">
+      <c r="A3" s="50" t="s">
         <v>41</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="50" t="s">
         <v>42</v>
       </c>
-      <c r="C3" s="16" t="s">
+      <c r="C3" s="50" t="s">
         <v>43</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="50" t="s">
         <v>41</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="E3" s="50" t="s">
         <v>42</v>
       </c>
-      <c r="F3" s="16" t="s">
+      <c r="F3" s="50" t="s">
         <v>43</v>
       </c>
-      <c r="G3" s="17" t="s">
+      <c r="G3" s="50" t="s">
         <v>41</v>
       </c>
-      <c r="H3" s="15" t="s">
+      <c r="H3" s="50" t="s">
         <v>42</v>
       </c>
-      <c r="I3" s="16" t="s">
+      <c r="I3" s="50" t="s">
         <v>43</v>
       </c>
     </row>
@@ -4193,82 +3971,82 @@
     <tabColor rgb="FFB8FEC9"/>
   </sheetPr>
   <dimension ref="A1:Q3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7109375" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7265625" defaultRowHeight="17.5" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="2" width="15.7109375" style="1"/>
-    <col min="3" max="5" width="15.7109375" style="2"/>
-    <col min="6" max="6" width="15.7109375" style="14"/>
-    <col min="7" max="9" width="15.7109375" style="2"/>
-    <col min="10" max="10" width="15.7109375" style="12"/>
-    <col min="11" max="16384" width="15.7109375" style="2"/>
+    <col min="1" max="2" width="15.7265625" style="1"/>
+    <col min="3" max="5" width="15.7265625" style="2"/>
+    <col min="6" max="6" width="15.7265625" style="10"/>
+    <col min="7" max="9" width="15.7265625" style="2"/>
+    <col min="10" max="10" width="15.7265625" style="8"/>
+    <col min="11" max="16384" width="15.7265625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="20" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="72" t="s">
+    <row r="1" spans="1:17" s="14" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="36" t="s">
         <v>108</v>
       </c>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="D1" s="72"/>
-      <c r="E1" s="72"/>
-      <c r="F1" s="72"/>
-      <c r="G1" s="72"/>
-      <c r="H1" s="72"/>
-      <c r="I1" s="72"/>
-      <c r="J1" s="72"/>
-      <c r="K1" s="72"/>
-      <c r="L1" s="72"/>
-      <c r="M1" s="72"/>
-      <c r="N1" s="72"/>
-      <c r="O1" s="72"/>
-      <c r="P1" s="72"/>
-      <c r="Q1" s="72"/>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A2" s="51" t="s">
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
+      <c r="I1" s="36"/>
+      <c r="J1" s="36"/>
+      <c r="K1" s="36"/>
+      <c r="L1" s="36"/>
+      <c r="M1" s="36"/>
+      <c r="N1" s="36"/>
+      <c r="O1" s="36"/>
+      <c r="P1" s="36"/>
+      <c r="Q1" s="36"/>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.5">
+      <c r="A2" s="42" t="s">
         <v>109</v>
       </c>
-      <c r="B2" s="52"/>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
-      <c r="E2" s="53"/>
-      <c r="F2" s="51" t="s">
+      <c r="B2" s="42"/>
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42" t="s">
         <v>110</v>
       </c>
-      <c r="G2" s="52"/>
-      <c r="H2" s="52"/>
-      <c r="I2" s="52"/>
-      <c r="J2" s="53"/>
-    </row>
-    <row r="3" spans="1:17" ht="38.25" x14ac:dyDescent="0.35">
-      <c r="A3" s="15" t="s">
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
+      <c r="I2" s="42"/>
+      <c r="J2" s="42"/>
+    </row>
+    <row r="3" spans="1:17" ht="37.5" x14ac:dyDescent="0.5">
+      <c r="A3" s="50" t="s">
         <v>42</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="50" t="s">
         <v>115</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="50" t="s">
         <v>116</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="50" t="s">
         <v>117</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="E3" s="50" t="s">
         <v>118</v>
       </c>
-      <c r="F3" s="17" t="s">
+      <c r="F3" s="50" t="s">
         <v>42</v>
       </c>
-      <c r="G3" s="15" t="s">
+      <c r="G3" s="50" t="s">
         <v>111</v>
       </c>
-      <c r="H3" s="15" t="s">
+      <c r="H3" s="50" t="s">
         <v>112</v>
       </c>
-      <c r="I3" s="15" t="s">
+      <c r="I3" s="50" t="s">
         <v>113</v>
       </c>
-      <c r="J3" s="16" t="s">
+      <c r="J3" s="50" t="s">
         <v>114</v>
       </c>
     </row>
@@ -4297,50 +4075,50 @@
     <tabColor rgb="FFB8FEC9"/>
   </sheetPr>
   <dimension ref="A1:O3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7109375" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7265625" defaultRowHeight="17.5" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="15.7109375" style="1"/>
-    <col min="2" max="2" width="15.7109375" style="11"/>
-    <col min="3" max="3" width="17.85546875" style="12" customWidth="1"/>
-    <col min="4" max="16384" width="15.7109375" style="2"/>
+    <col min="1" max="1" width="15.7265625" style="1"/>
+    <col min="2" max="2" width="15.7265625" style="7"/>
+    <col min="3" max="3" width="17.81640625" style="8" customWidth="1"/>
+    <col min="4" max="16384" width="15.7265625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="20" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="72" t="s">
+    <row r="1" spans="1:15" s="14" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="36" t="s">
         <v>52</v>
       </c>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="D1" s="72"/>
-      <c r="E1" s="72"/>
-      <c r="F1" s="72"/>
-      <c r="G1" s="72"/>
-      <c r="H1" s="72"/>
-      <c r="I1" s="72"/>
-      <c r="J1" s="72"/>
-      <c r="K1" s="72"/>
-      <c r="L1" s="72"/>
-      <c r="M1" s="72"/>
-      <c r="N1" s="72"/>
-      <c r="O1" s="72"/>
-    </row>
-    <row r="2" spans="1:15" ht="36" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="51" t="s">
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
+      <c r="I1" s="36"/>
+      <c r="J1" s="36"/>
+      <c r="K1" s="36"/>
+      <c r="L1" s="36"/>
+      <c r="M1" s="36"/>
+      <c r="N1" s="36"/>
+      <c r="O1" s="36"/>
+    </row>
+    <row r="2" spans="1:15" ht="36" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A2" s="42" t="s">
         <v>47</v>
       </c>
-      <c r="B2" s="53"/>
-      <c r="C2" s="58" t="s">
+      <c r="B2" s="42"/>
+      <c r="C2" s="42" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="89.25" x14ac:dyDescent="0.35">
-      <c r="A3" s="15" t="s">
+    <row r="3" spans="1:15" ht="75" x14ac:dyDescent="0.5">
+      <c r="A3" s="50" t="s">
         <v>48</v>
       </c>
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="50" t="s">
         <v>49</v>
       </c>
-      <c r="C3" s="59"/>
+      <c r="C3" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
fix: correction d'une coquille dans une cellule
</commit_message>
<xml_diff>
--- a/impact/vsme/xlsx/VSME.xlsx
+++ b/impact/vsme/xlsx/VSME.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LDE-CASTELBAJAC-ADC\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CD7DF51C-B45F-4FF4-A08E-7C2EC3086646}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E4A0CEF-146C-44EE-BB08-2CFD9A22D9B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28980" yWindow="1545" windowWidth="21600" windowHeight="11175" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="&gt;&gt;&gt; " sheetId="3" r:id="rId1"/>
@@ -587,12 +587,6 @@
     <t>L’entreprise a-t-elle confirmé des incidents graves au sein de son personnel liés à la discrimination ?</t>
   </si>
   <si>
-    <t xml:space="preserve">Description des actions mises en oeuvre pour gérer les indidents confirmés </t>
-  </si>
-  <si>
-    <t>Autres thèmes concernant des indidents graves confirmés relatifs aux droits de l’homme</t>
-  </si>
-  <si>
     <t>Incidents graves en matière de droits de l’homme dans la chaîne de valeur et auprès des parties prenantes externes</t>
   </si>
   <si>
@@ -750,6 +744,12 @@
   </si>
   <si>
     <t xml:space="preserve">Total </t>
+  </si>
+  <si>
+    <t>Autres thèmes concernant des incidents graves confirmés relatifs aux droits de l’homme</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Description des actions mises en oeuvre pour gérer les incidents confirmés </t>
   </si>
 </sst>
 </file>
@@ -1144,33 +1144,6 @@
     <xf numFmtId="0" fontId="3" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1179,23 +1152,8 @@
     <xf numFmtId="0" fontId="8" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="9" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1211,6 +1169,48 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1706,11 +1706,11 @@
       </c>
     </row>
     <row r="11" spans="3:9" s="4" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C11" s="34" t="s">
+      <c r="C11" s="49" t="s">
         <v>14</v>
       </c>
-      <c r="D11" s="34"/>
-      <c r="E11" s="34"/>
+      <c r="D11" s="49"/>
+      <c r="E11" s="49"/>
     </row>
     <row r="13" spans="3:9" ht="72.75" customHeight="1" x14ac:dyDescent="1.95">
       <c r="C13" s="5" t="s">
@@ -1753,69 +1753,69 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" s="14" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="56" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
-      <c r="J1" s="36"/>
-      <c r="K1" s="36"/>
-      <c r="L1" s="36"/>
-      <c r="M1" s="36"/>
-      <c r="N1" s="36"/>
-      <c r="O1" s="36"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
+      <c r="K1" s="56"/>
+      <c r="L1" s="56"/>
+      <c r="M1" s="56"/>
+      <c r="N1" s="56"/>
+      <c r="O1" s="56"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.5">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="52" t="s">
         <v>91</v>
       </c>
-      <c r="B2" s="42" t="s">
+      <c r="B2" s="52" t="s">
         <v>53</v>
       </c>
-      <c r="C2" s="42"/>
-      <c r="D2" s="42"/>
-      <c r="E2" s="42"/>
-      <c r="F2" s="42"/>
-      <c r="G2" s="42"/>
-      <c r="H2" s="42" t="s">
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52"/>
+      <c r="H2" s="52" t="s">
         <v>60</v>
       </c>
-      <c r="I2" s="42"/>
-      <c r="J2" s="42"/>
+      <c r="I2" s="52"/>
+      <c r="J2" s="52"/>
     </row>
     <row r="3" spans="1:15" ht="50" x14ac:dyDescent="0.5">
-      <c r="A3" s="42"/>
-      <c r="B3" s="50" t="s">
+      <c r="A3" s="52"/>
+      <c r="B3" s="40" t="s">
         <v>54</v>
       </c>
-      <c r="C3" s="50" t="s">
+      <c r="C3" s="40" t="s">
         <v>55</v>
       </c>
-      <c r="D3" s="50" t="s">
+      <c r="D3" s="40" t="s">
         <v>56</v>
       </c>
-      <c r="E3" s="50" t="s">
+      <c r="E3" s="40" t="s">
         <v>57</v>
       </c>
-      <c r="F3" s="50" t="s">
+      <c r="F3" s="40" t="s">
         <v>58</v>
       </c>
-      <c r="G3" s="50" t="s">
+      <c r="G3" s="40" t="s">
         <v>59</v>
       </c>
-      <c r="H3" s="50" t="s">
+      <c r="H3" s="40" t="s">
         <v>63</v>
       </c>
-      <c r="I3" s="50" t="s">
+      <c r="I3" s="40" t="s">
         <v>62</v>
       </c>
-      <c r="J3" s="50" t="s">
+      <c r="J3" s="40" t="s">
         <v>61</v>
       </c>
     </row>
@@ -1851,277 +1851,277 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" s="14" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="36" t="s">
-        <v>223</v>
-      </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
-      <c r="J1" s="36"/>
-      <c r="K1" s="36"/>
-      <c r="L1" s="36"/>
-      <c r="M1" s="36"/>
-      <c r="N1" s="36"/>
-      <c r="O1" s="36"/>
+      <c r="A1" s="56" t="s">
+        <v>221</v>
+      </c>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
+      <c r="K1" s="56"/>
+      <c r="L1" s="56"/>
+      <c r="M1" s="56"/>
+      <c r="N1" s="56"/>
+      <c r="O1" s="56"/>
       <c r="P1" s="29"/>
     </row>
     <row r="2" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="52" t="s">
+        <v>210</v>
+      </c>
+      <c r="B2" s="52" t="s">
+        <v>211</v>
+      </c>
+      <c r="C2" s="57" t="s">
+        <v>209</v>
+      </c>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="58"/>
+      <c r="H2" s="52" t="s">
+        <v>191</v>
+      </c>
+      <c r="I2" s="52"/>
+      <c r="J2" s="52"/>
+      <c r="K2" s="52"/>
+      <c r="L2" s="52"/>
+      <c r="M2" s="57" t="s">
+        <v>216</v>
+      </c>
+      <c r="N2" s="58"/>
+      <c r="O2" s="58"/>
+      <c r="P2" s="58"/>
+    </row>
+    <row r="3" spans="1:16" ht="62.5" x14ac:dyDescent="0.5">
+      <c r="A3" s="52"/>
+      <c r="B3" s="52"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="40" t="s">
         <v>212</v>
       </c>
-      <c r="B2" s="42" t="s">
+      <c r="E3" s="40" t="s">
         <v>213</v>
       </c>
-      <c r="C2" s="53" t="s">
-        <v>211</v>
-      </c>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="54"/>
-      <c r="H2" s="42" t="s">
-        <v>193</v>
-      </c>
-      <c r="I2" s="42"/>
-      <c r="J2" s="42"/>
-      <c r="K2" s="42"/>
-      <c r="L2" s="42"/>
-      <c r="M2" s="53" t="s">
+      <c r="F3" s="40" t="s">
+        <v>214</v>
+      </c>
+      <c r="G3" s="40" t="s">
+        <v>215</v>
+      </c>
+      <c r="H3" s="40"/>
+      <c r="I3" s="40" t="s">
+        <v>212</v>
+      </c>
+      <c r="J3" s="40" t="s">
+        <v>213</v>
+      </c>
+      <c r="K3" s="40" t="s">
+        <v>214</v>
+      </c>
+      <c r="L3" s="40" t="s">
+        <v>215</v>
+      </c>
+      <c r="M3" s="40" t="s">
+        <v>217</v>
+      </c>
+      <c r="N3" s="40" t="s">
         <v>218</v>
       </c>
-      <c r="N2" s="54"/>
-      <c r="O2" s="54"/>
-      <c r="P2" s="54"/>
-    </row>
-    <row r="3" spans="1:16" ht="62.5" x14ac:dyDescent="0.5">
-      <c r="A3" s="42"/>
-      <c r="B3" s="42"/>
-      <c r="C3" s="55"/>
-      <c r="D3" s="50" t="s">
-        <v>214</v>
-      </c>
-      <c r="E3" s="50" t="s">
-        <v>215</v>
-      </c>
-      <c r="F3" s="50" t="s">
-        <v>216</v>
-      </c>
-      <c r="G3" s="50" t="s">
-        <v>217</v>
-      </c>
-      <c r="H3" s="50"/>
-      <c r="I3" s="50" t="s">
-        <v>214</v>
-      </c>
-      <c r="J3" s="50" t="s">
-        <v>215</v>
-      </c>
-      <c r="K3" s="50" t="s">
-        <v>216</v>
-      </c>
-      <c r="L3" s="50" t="s">
-        <v>217</v>
-      </c>
-      <c r="M3" s="50" t="s">
+      <c r="O3" s="40" t="s">
         <v>219</v>
       </c>
-      <c r="N3" s="50" t="s">
+      <c r="P3" s="40" t="s">
         <v>220</v>
       </c>
-      <c r="O3" s="50" t="s">
-        <v>221</v>
-      </c>
-      <c r="P3" s="50" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" ht="25" x14ac:dyDescent="0.5">
-      <c r="C4" s="50" t="s">
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.5">
+      <c r="C4" s="40" t="s">
         <v>124</v>
       </c>
-      <c r="D4" s="55"/>
-      <c r="E4" s="55"/>
-      <c r="F4" s="55"/>
-      <c r="G4" s="50"/>
-      <c r="H4" s="56" t="s">
-        <v>194</v>
-      </c>
-      <c r="I4" s="57"/>
-      <c r="J4" s="55"/>
-      <c r="K4" s="55"/>
-      <c r="L4" s="55"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="41"/>
+      <c r="F4" s="41"/>
+      <c r="G4" s="40"/>
+      <c r="H4" s="42" t="s">
+        <v>192</v>
+      </c>
+      <c r="I4" s="43"/>
+      <c r="J4" s="41"/>
+      <c r="K4" s="41"/>
+      <c r="L4" s="41"/>
       <c r="M4" s="30"/>
       <c r="N4" s="30"/>
       <c r="O4" s="30"/>
       <c r="P4" s="31"/>
     </row>
-    <row r="5" spans="1:16" ht="25" x14ac:dyDescent="0.5">
-      <c r="C5" s="50" t="s">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.5">
+      <c r="C5" s="40" t="s">
         <v>125</v>
       </c>
-      <c r="D5" s="55"/>
-      <c r="E5" s="55"/>
-      <c r="F5" s="55"/>
-      <c r="G5" s="50"/>
-      <c r="H5" s="56" t="s">
-        <v>195</v>
-      </c>
-      <c r="I5" s="57"/>
-      <c r="J5" s="55"/>
-      <c r="K5" s="55"/>
-      <c r="L5" s="55"/>
-    </row>
-    <row r="6" spans="1:16" ht="50" x14ac:dyDescent="0.5">
-      <c r="C6" s="50" t="s">
-        <v>231</v>
-      </c>
-      <c r="D6" s="55"/>
-      <c r="E6" s="55"/>
-      <c r="F6" s="55"/>
-      <c r="G6" s="50"/>
-      <c r="H6" s="56" t="s">
-        <v>196</v>
-      </c>
-      <c r="I6" s="55"/>
-      <c r="J6" s="55"/>
-      <c r="K6" s="55"/>
-      <c r="L6" s="55"/>
-    </row>
-    <row r="7" spans="1:16" ht="37.5" x14ac:dyDescent="0.5">
+      <c r="D5" s="41"/>
+      <c r="E5" s="41"/>
+      <c r="F5" s="41"/>
+      <c r="G5" s="40"/>
+      <c r="H5" s="42" t="s">
+        <v>193</v>
+      </c>
+      <c r="I5" s="43"/>
+      <c r="J5" s="41"/>
+      <c r="K5" s="41"/>
+      <c r="L5" s="41"/>
+    </row>
+    <row r="6" spans="1:16" ht="25" x14ac:dyDescent="0.5">
+      <c r="C6" s="40" t="s">
+        <v>229</v>
+      </c>
+      <c r="D6" s="41"/>
+      <c r="E6" s="41"/>
+      <c r="F6" s="41"/>
+      <c r="G6" s="40"/>
+      <c r="H6" s="42" t="s">
+        <v>194</v>
+      </c>
+      <c r="I6" s="41"/>
+      <c r="J6" s="41"/>
+      <c r="K6" s="41"/>
+      <c r="L6" s="41"/>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.5">
       <c r="C7" s="12"/>
       <c r="D7" s="27"/>
       <c r="E7" s="27"/>
       <c r="F7" s="27"/>
       <c r="G7" s="11"/>
-      <c r="H7" s="56" t="s">
+      <c r="H7" s="42" t="s">
+        <v>195</v>
+      </c>
+      <c r="I7" s="41"/>
+      <c r="J7" s="41"/>
+      <c r="K7" s="41"/>
+      <c r="L7" s="41"/>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.5">
+      <c r="H8" s="42" t="s">
+        <v>196</v>
+      </c>
+      <c r="I8" s="41"/>
+      <c r="J8" s="41"/>
+      <c r="K8" s="41"/>
+      <c r="L8" s="43"/>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.5">
+      <c r="H9" s="42" t="s">
         <v>197</v>
       </c>
-      <c r="I7" s="55"/>
-      <c r="J7" s="55"/>
-      <c r="K7" s="55"/>
-      <c r="L7" s="55"/>
-    </row>
-    <row r="8" spans="1:16" ht="25" x14ac:dyDescent="0.5">
-      <c r="H8" s="56" t="s">
+      <c r="I9" s="41"/>
+      <c r="J9" s="41"/>
+      <c r="K9" s="41"/>
+      <c r="L9" s="43"/>
+    </row>
+    <row r="10" spans="1:16" ht="25" x14ac:dyDescent="0.5">
+      <c r="H10" s="42" t="s">
         <v>198</v>
       </c>
-      <c r="I8" s="55"/>
-      <c r="J8" s="55"/>
-      <c r="K8" s="55"/>
-      <c r="L8" s="57"/>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.5">
-      <c r="H9" s="56" t="s">
+      <c r="I10" s="41"/>
+      <c r="J10" s="41"/>
+      <c r="K10" s="41"/>
+      <c r="L10" s="43"/>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.5">
+      <c r="H11" s="42" t="s">
         <v>199</v>
       </c>
-      <c r="I9" s="55"/>
-      <c r="J9" s="55"/>
-      <c r="K9" s="55"/>
-      <c r="L9" s="57"/>
-    </row>
-    <row r="10" spans="1:16" ht="37.5" x14ac:dyDescent="0.5">
-      <c r="H10" s="56" t="s">
+      <c r="I11" s="41"/>
+      <c r="J11" s="41"/>
+      <c r="K11" s="41"/>
+      <c r="L11" s="43"/>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.5">
+      <c r="H12" s="42" t="s">
         <v>200</v>
       </c>
-      <c r="I10" s="55"/>
-      <c r="J10" s="55"/>
-      <c r="K10" s="55"/>
-      <c r="L10" s="57"/>
-    </row>
-    <row r="11" spans="1:16" ht="25" x14ac:dyDescent="0.5">
-      <c r="H11" s="56" t="s">
+      <c r="I12" s="41"/>
+      <c r="J12" s="41"/>
+      <c r="K12" s="41"/>
+      <c r="L12" s="43"/>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.5">
+      <c r="H13" s="42" t="s">
         <v>201</v>
       </c>
-      <c r="I11" s="55"/>
-      <c r="J11" s="55"/>
-      <c r="K11" s="55"/>
-      <c r="L11" s="57"/>
-    </row>
-    <row r="12" spans="1:16" ht="25" x14ac:dyDescent="0.5">
-      <c r="H12" s="56" t="s">
+      <c r="I13" s="41"/>
+      <c r="J13" s="41"/>
+      <c r="K13" s="41"/>
+      <c r="L13" s="43"/>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.5">
+      <c r="H14" s="42" t="s">
         <v>202</v>
       </c>
-      <c r="I12" s="55"/>
-      <c r="J12" s="55"/>
-      <c r="K12" s="55"/>
-      <c r="L12" s="57"/>
-    </row>
-    <row r="13" spans="1:16" ht="25" x14ac:dyDescent="0.5">
-      <c r="H13" s="56" t="s">
+      <c r="I14" s="41"/>
+      <c r="J14" s="41"/>
+      <c r="K14" s="41"/>
+      <c r="L14" s="43"/>
+    </row>
+    <row r="15" spans="1:16" ht="25" x14ac:dyDescent="0.5">
+      <c r="H15" s="42" t="s">
         <v>203</v>
       </c>
-      <c r="I13" s="55"/>
-      <c r="J13" s="55"/>
-      <c r="K13" s="55"/>
-      <c r="L13" s="57"/>
-    </row>
-    <row r="14" spans="1:16" ht="25" x14ac:dyDescent="0.5">
-      <c r="H14" s="56" t="s">
+      <c r="I15" s="41"/>
+      <c r="J15" s="41"/>
+      <c r="K15" s="41"/>
+      <c r="L15" s="43"/>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.5">
+      <c r="H16" s="42" t="s">
         <v>204</v>
       </c>
-      <c r="I14" s="55"/>
-      <c r="J14" s="55"/>
-      <c r="K14" s="55"/>
-      <c r="L14" s="57"/>
-    </row>
-    <row r="15" spans="1:16" ht="37.5" x14ac:dyDescent="0.5">
-      <c r="H15" s="56" t="s">
+      <c r="I16" s="41"/>
+      <c r="J16" s="41"/>
+      <c r="K16" s="41"/>
+      <c r="L16" s="43"/>
+    </row>
+    <row r="17" spans="8:12" x14ac:dyDescent="0.5">
+      <c r="H17" s="42" t="s">
         <v>205</v>
       </c>
-      <c r="I15" s="55"/>
-      <c r="J15" s="55"/>
-      <c r="K15" s="55"/>
-      <c r="L15" s="57"/>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.5">
-      <c r="H16" s="56" t="s">
+      <c r="I17" s="41"/>
+      <c r="J17" s="41"/>
+      <c r="K17" s="41"/>
+      <c r="L17" s="43"/>
+    </row>
+    <row r="18" spans="8:12" x14ac:dyDescent="0.5">
+      <c r="H18" s="42" t="s">
         <v>206</v>
       </c>
-      <c r="I16" s="55"/>
-      <c r="J16" s="55"/>
-      <c r="K16" s="55"/>
-      <c r="L16" s="57"/>
-    </row>
-    <row r="17" spans="8:12" x14ac:dyDescent="0.5">
-      <c r="H17" s="56" t="s">
-        <v>207</v>
-      </c>
-      <c r="I17" s="55"/>
-      <c r="J17" s="55"/>
-      <c r="K17" s="55"/>
-      <c r="L17" s="57"/>
-    </row>
-    <row r="18" spans="8:12" x14ac:dyDescent="0.5">
-      <c r="H18" s="56" t="s">
-        <v>208</v>
-      </c>
-      <c r="I18" s="55"/>
-      <c r="J18" s="55"/>
-      <c r="K18" s="55"/>
-      <c r="L18" s="57"/>
+      <c r="I18" s="41"/>
+      <c r="J18" s="41"/>
+      <c r="K18" s="41"/>
+      <c r="L18" s="43"/>
     </row>
     <row r="19" spans="8:12" x14ac:dyDescent="0.5">
-      <c r="H19" s="56" t="s">
-        <v>229</v>
-      </c>
-      <c r="I19" s="57"/>
-      <c r="J19" s="57"/>
-      <c r="K19" s="57"/>
-      <c r="L19" s="55"/>
+      <c r="H19" s="42" t="s">
+        <v>227</v>
+      </c>
+      <c r="I19" s="43"/>
+      <c r="J19" s="43"/>
+      <c r="K19" s="43"/>
+      <c r="L19" s="41"/>
     </row>
     <row r="20" spans="8:12" x14ac:dyDescent="0.5">
-      <c r="H20" s="56" t="s">
-        <v>230</v>
-      </c>
-      <c r="I20" s="57"/>
-      <c r="J20" s="57"/>
-      <c r="K20" s="57"/>
-      <c r="L20" s="55"/>
+      <c r="H20" s="42" t="s">
+        <v>228</v>
+      </c>
+      <c r="I20" s="43"/>
+      <c r="J20" s="43"/>
+      <c r="K20" s="43"/>
+      <c r="L20" s="41"/>
     </row>
     <row r="21" spans="8:12" x14ac:dyDescent="0.5">
       <c r="H21" s="25"/>
@@ -2157,67 +2157,67 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" s="14" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="36" t="s">
-        <v>190</v>
-      </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
-      <c r="J1" s="36"/>
-      <c r="K1" s="36"/>
-      <c r="L1" s="36"/>
-      <c r="M1" s="36"/>
-      <c r="N1" s="36"/>
-      <c r="O1" s="36"/>
-      <c r="P1" s="36"/>
+      <c r="A1" s="56" t="s">
+        <v>188</v>
+      </c>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
+      <c r="K1" s="56"/>
+      <c r="L1" s="56"/>
+      <c r="M1" s="56"/>
+      <c r="N1" s="56"/>
+      <c r="O1" s="56"/>
+      <c r="P1" s="56"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.5">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="52" t="s">
+        <v>179</v>
+      </c>
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52" t="s">
+        <v>184</v>
+      </c>
+      <c r="G2" s="52"/>
+      <c r="H2" s="52"/>
+      <c r="I2" s="52"/>
+    </row>
+    <row r="3" spans="1:16" ht="37.5" x14ac:dyDescent="0.5">
+      <c r="A3" s="40" t="s">
+        <v>189</v>
+      </c>
+      <c r="B3" s="40" t="s">
+        <v>180</v>
+      </c>
+      <c r="C3" s="40" t="s">
         <v>181</v>
       </c>
-      <c r="B2" s="42"/>
-      <c r="C2" s="42"/>
-      <c r="D2" s="42"/>
-      <c r="E2" s="42"/>
-      <c r="F2" s="42" t="s">
+      <c r="D3" s="40" t="s">
+        <v>182</v>
+      </c>
+      <c r="E3" s="40" t="s">
+        <v>183</v>
+      </c>
+      <c r="F3" s="40" t="s">
+        <v>185</v>
+      </c>
+      <c r="G3" s="40" t="s">
         <v>186</v>
       </c>
-      <c r="G2" s="42"/>
-      <c r="H2" s="42"/>
-      <c r="I2" s="42"/>
-    </row>
-    <row r="3" spans="1:16" ht="37.5" x14ac:dyDescent="0.5">
-      <c r="A3" s="50" t="s">
-        <v>191</v>
-      </c>
-      <c r="B3" s="50" t="s">
+      <c r="H3" s="40" t="s">
+        <v>187</v>
+      </c>
+      <c r="I3" s="40" t="s">
         <v>182</v>
-      </c>
-      <c r="C3" s="50" t="s">
-        <v>183</v>
-      </c>
-      <c r="D3" s="50" t="s">
-        <v>184</v>
-      </c>
-      <c r="E3" s="50" t="s">
-        <v>185</v>
-      </c>
-      <c r="F3" s="50" t="s">
-        <v>187</v>
-      </c>
-      <c r="G3" s="50" t="s">
-        <v>188</v>
-      </c>
-      <c r="H3" s="50" t="s">
-        <v>189</v>
-      </c>
-      <c r="I3" s="50" t="s">
-        <v>184</v>
       </c>
     </row>
   </sheetData>
@@ -2261,69 +2261,69 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" s="15" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="59" t="s">
         <v>79</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
-      <c r="H1" s="37"/>
-      <c r="I1" s="37"/>
-      <c r="J1" s="37"/>
-      <c r="K1" s="37"/>
-      <c r="L1" s="37"/>
-      <c r="M1" s="37"/>
-      <c r="N1" s="37"/>
-      <c r="O1" s="37"/>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="59"/>
+      <c r="I1" s="59"/>
+      <c r="J1" s="59"/>
+      <c r="K1" s="59"/>
+      <c r="L1" s="59"/>
+      <c r="M1" s="59"/>
+      <c r="N1" s="59"/>
+      <c r="O1" s="59"/>
     </row>
     <row r="2" spans="1:15" ht="39" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="52" t="s">
         <v>80</v>
       </c>
-      <c r="B2" s="42"/>
-      <c r="C2" s="42" t="s">
+      <c r="B2" s="52"/>
+      <c r="C2" s="52" t="s">
         <v>83</v>
       </c>
-      <c r="D2" s="42"/>
-      <c r="E2" s="42"/>
-      <c r="F2" s="42"/>
-      <c r="G2" s="42" t="s">
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52" t="s">
         <v>86</v>
       </c>
-      <c r="H2" s="42"/>
-      <c r="I2" s="42" t="s">
+      <c r="H2" s="52"/>
+      <c r="I2" s="52" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="3" spans="1:15" ht="25" x14ac:dyDescent="0.5">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="40" t="s">
         <v>81</v>
       </c>
-      <c r="B3" s="50" t="s">
+      <c r="B3" s="40" t="s">
         <v>82</v>
       </c>
-      <c r="C3" s="50" t="s">
+      <c r="C3" s="40" t="s">
         <v>84</v>
       </c>
-      <c r="D3" s="50" t="s">
+      <c r="D3" s="40" t="s">
         <v>85</v>
       </c>
-      <c r="E3" s="50" t="s">
+      <c r="E3" s="40" t="s">
         <v>103</v>
       </c>
-      <c r="F3" s="50" t="s">
+      <c r="F3" s="40" t="s">
         <v>92</v>
       </c>
-      <c r="G3" s="50" t="s">
+      <c r="G3" s="40" t="s">
         <v>28</v>
       </c>
-      <c r="H3" s="50" t="s">
+      <c r="H3" s="40" t="s">
         <v>87</v>
       </c>
-      <c r="I3" s="42"/>
+      <c r="I3" s="52"/>
     </row>
     <row r="12" spans="1:15" ht="74" x14ac:dyDescent="1.95">
       <c r="E12" s="16"/>
@@ -2357,41 +2357,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" s="15" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="59" t="s">
         <v>102</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
-      <c r="H1" s="37"/>
-      <c r="I1" s="37"/>
-      <c r="J1" s="37"/>
-      <c r="K1" s="37"/>
-      <c r="L1" s="37"/>
-      <c r="M1" s="37"/>
-      <c r="N1" s="37"/>
-      <c r="O1" s="37"/>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="59"/>
+      <c r="I1" s="59"/>
+      <c r="J1" s="59"/>
+      <c r="K1" s="59"/>
+      <c r="L1" s="59"/>
+      <c r="M1" s="59"/>
+      <c r="N1" s="59"/>
+      <c r="O1" s="59"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.5">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="52" t="s">
         <v>64</v>
       </c>
-      <c r="B2" s="42"/>
-      <c r="C2" s="42" t="s">
+      <c r="B2" s="52"/>
+      <c r="C2" s="52" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:15" ht="37.5" x14ac:dyDescent="0.5">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="40" t="s">
         <v>65</v>
       </c>
-      <c r="B3" s="50" t="s">
+      <c r="B3" s="40" t="s">
         <v>66</v>
       </c>
-      <c r="C3" s="42"/>
+      <c r="C3" s="52"/>
     </row>
     <row r="12" spans="1:15" ht="74" x14ac:dyDescent="1.95">
       <c r="E12" s="16"/>
@@ -2427,74 +2427,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" s="15" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="59" t="s">
         <v>101</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
-      <c r="H1" s="37"/>
-      <c r="I1" s="37"/>
-      <c r="J1" s="37"/>
-      <c r="K1" s="37"/>
-      <c r="L1" s="37"/>
-      <c r="M1" s="37"/>
-      <c r="N1" s="37"/>
-      <c r="O1" s="37"/>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="59"/>
+      <c r="I1" s="59"/>
+      <c r="J1" s="59"/>
+      <c r="K1" s="59"/>
+      <c r="L1" s="59"/>
+      <c r="M1" s="59"/>
+      <c r="N1" s="59"/>
+      <c r="O1" s="59"/>
     </row>
     <row r="2" spans="1:15" ht="54.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="52" t="s">
         <v>93</v>
       </c>
-      <c r="B2" s="42" t="s">
+      <c r="B2" s="52" t="s">
         <v>94</v>
       </c>
-      <c r="C2" s="42"/>
-      <c r="D2" s="42"/>
-      <c r="E2" s="42" t="s">
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52" t="s">
         <v>98</v>
       </c>
-      <c r="F2" s="42"/>
-      <c r="G2" s="42" t="s">
+      <c r="F2" s="52"/>
+      <c r="G2" s="52" t="s">
         <v>105</v>
       </c>
-      <c r="H2" s="42"/>
-      <c r="I2" s="42"/>
+      <c r="H2" s="52"/>
+      <c r="I2" s="52"/>
     </row>
     <row r="3" spans="1:15" ht="97.5" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A3" s="42"/>
-      <c r="B3" s="50" t="s">
+      <c r="A3" s="52"/>
+      <c r="B3" s="40" t="s">
         <v>95</v>
       </c>
-      <c r="C3" s="50" t="s">
+      <c r="C3" s="40" t="s">
         <v>96</v>
       </c>
-      <c r="D3" s="50" t="s">
+      <c r="D3" s="40" t="s">
         <v>97</v>
       </c>
-      <c r="E3" s="50" t="s">
+      <c r="E3" s="40" t="s">
         <v>99</v>
       </c>
-      <c r="F3" s="50" t="s">
+      <c r="F3" s="40" t="s">
         <v>98</v>
       </c>
-      <c r="G3" s="61"/>
-      <c r="H3" s="62" t="s">
+      <c r="G3" s="47"/>
+      <c r="H3" s="48" t="s">
         <v>100</v>
       </c>
-      <c r="I3" s="62" t="s">
+      <c r="I3" s="48" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.5">
-      <c r="G4" s="58" t="s">
+      <c r="G4" s="44" t="s">
         <v>84</v>
       </c>
-      <c r="H4" s="59"/>
-      <c r="I4" s="60"/>
+      <c r="H4" s="45"/>
+      <c r="I4" s="46"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.5">
       <c r="G5" s="20" t="s">
@@ -2546,49 +2546,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" s="15" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="59" t="s">
         <v>171</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
-      <c r="H1" s="37"/>
-      <c r="I1" s="37"/>
-      <c r="J1" s="37"/>
-      <c r="K1" s="37"/>
-      <c r="L1" s="37"/>
-      <c r="M1" s="37"/>
-      <c r="N1" s="37"/>
-      <c r="O1" s="37"/>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="59"/>
+      <c r="I1" s="59"/>
+      <c r="J1" s="59"/>
+      <c r="K1" s="59"/>
+      <c r="L1" s="59"/>
+      <c r="M1" s="59"/>
+      <c r="N1" s="59"/>
+      <c r="O1" s="59"/>
     </row>
     <row r="2" spans="1:15" ht="53.25" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="52" t="s">
         <v>167</v>
       </c>
-      <c r="B2" s="42"/>
-      <c r="C2" s="42"/>
-      <c r="D2" s="42" t="s">
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52" t="s">
         <v>170</v>
       </c>
-      <c r="E2" s="42"/>
+      <c r="E2" s="52"/>
     </row>
     <row r="3" spans="1:15" ht="112.5" x14ac:dyDescent="0.5">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="40" t="s">
         <v>165</v>
       </c>
-      <c r="B3" s="50" t="s">
+      <c r="B3" s="40" t="s">
         <v>166</v>
       </c>
-      <c r="C3" s="50" t="s">
+      <c r="C3" s="40" t="s">
         <v>167</v>
       </c>
-      <c r="D3" s="50" t="s">
+      <c r="D3" s="40" t="s">
         <v>168</v>
       </c>
-      <c r="E3" s="50" t="s">
+      <c r="E3" s="40" t="s">
         <v>169</v>
       </c>
     </row>
@@ -2627,61 +2627,61 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" s="15" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="59" t="s">
         <v>154</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
-      <c r="H1" s="37"/>
-      <c r="I1" s="37"/>
-      <c r="J1" s="37"/>
-      <c r="K1" s="37"/>
-      <c r="L1" s="37"/>
-      <c r="M1" s="37"/>
-      <c r="N1" s="37"/>
-      <c r="O1" s="37"/>
-      <c r="P1" s="37"/>
-      <c r="Q1" s="37"/>
-      <c r="R1" s="37"/>
-      <c r="S1" s="37"/>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="59"/>
+      <c r="I1" s="59"/>
+      <c r="J1" s="59"/>
+      <c r="K1" s="59"/>
+      <c r="L1" s="59"/>
+      <c r="M1" s="59"/>
+      <c r="N1" s="59"/>
+      <c r="O1" s="59"/>
+      <c r="P1" s="59"/>
+      <c r="Q1" s="59"/>
+      <c r="R1" s="59"/>
+      <c r="S1" s="59"/>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.5">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="52" t="s">
         <v>146</v>
       </c>
-      <c r="B2" s="42"/>
-      <c r="C2" s="42"/>
-      <c r="D2" s="42"/>
-      <c r="E2" s="42"/>
-      <c r="F2" s="42"/>
-      <c r="G2" s="42" t="s">
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="3" spans="1:19" ht="62.5" x14ac:dyDescent="0.5">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="40" t="s">
         <v>147</v>
       </c>
-      <c r="B3" s="50" t="s">
+      <c r="B3" s="40" t="s">
         <v>148</v>
       </c>
-      <c r="C3" s="50" t="s">
+      <c r="C3" s="40" t="s">
         <v>149</v>
       </c>
-      <c r="D3" s="50" t="s">
+      <c r="D3" s="40" t="s">
         <v>150</v>
       </c>
-      <c r="E3" s="50" t="s">
+      <c r="E3" s="40" t="s">
         <v>151</v>
       </c>
-      <c r="F3" s="50" t="s">
+      <c r="F3" s="40" t="s">
         <v>152</v>
       </c>
-      <c r="G3" s="42"/>
+      <c r="G3" s="52"/>
     </row>
     <row r="12" spans="1:19" ht="74" x14ac:dyDescent="1.95">
       <c r="I12" s="16"/>
@@ -2713,70 +2713,73 @@
   <dimension ref="A1:S12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="17.5" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="11.36328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="5" width="11.453125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="13.7265625" style="7" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.08984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.7265625" style="7" customWidth="1"/>
     <col min="7" max="7" width="23.81640625" style="8" customWidth="1"/>
     <col min="8" max="9" width="11.453125" style="2" customWidth="1"/>
     <col min="10" max="16384" width="11.453125" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" s="15" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="37" t="s">
-        <v>180</v>
-      </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
-      <c r="H1" s="37"/>
-      <c r="I1" s="37"/>
-      <c r="J1" s="37"/>
-      <c r="K1" s="37"/>
-      <c r="L1" s="37"/>
-      <c r="M1" s="37"/>
-      <c r="N1" s="37"/>
-      <c r="O1" s="37"/>
-      <c r="P1" s="37"/>
-      <c r="Q1" s="37"/>
-      <c r="R1" s="37"/>
-      <c r="S1" s="37"/>
+      <c r="A1" s="59" t="s">
+        <v>178</v>
+      </c>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="59"/>
+      <c r="I1" s="59"/>
+      <c r="J1" s="59"/>
+      <c r="K1" s="59"/>
+      <c r="L1" s="59"/>
+      <c r="M1" s="59"/>
+      <c r="N1" s="59"/>
+      <c r="O1" s="59"/>
+      <c r="P1" s="59"/>
+      <c r="Q1" s="59"/>
+      <c r="R1" s="59"/>
+      <c r="S1" s="59"/>
     </row>
     <row r="2" spans="1:19" ht="33" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="52" t="s">
         <v>172</v>
       </c>
-      <c r="B2" s="42"/>
-      <c r="C2" s="42"/>
-      <c r="D2" s="42"/>
-      <c r="E2" s="42"/>
-      <c r="F2" s="42"/>
-      <c r="G2" s="42" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="3" spans="1:19" ht="112.5" x14ac:dyDescent="0.5">
-      <c r="A3" s="50" t="s">
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" ht="100" x14ac:dyDescent="0.5">
+      <c r="A3" s="40" t="s">
         <v>173</v>
       </c>
-      <c r="B3" s="50" t="s">
+      <c r="B3" s="40" t="s">
         <v>174</v>
       </c>
-      <c r="C3" s="50" t="s">
+      <c r="C3" s="40" t="s">
         <v>175</v>
       </c>
-      <c r="D3" s="50" t="s">
+      <c r="D3" s="40" t="s">
         <v>176</v>
       </c>
-      <c r="E3" s="50" t="s">
-        <v>178</v>
-      </c>
-      <c r="F3" s="50" t="s">
-        <v>177</v>
-      </c>
-      <c r="G3" s="42"/>
+      <c r="E3" s="40" t="s">
+        <v>230</v>
+      </c>
+      <c r="F3" s="40" t="s">
+        <v>231</v>
+      </c>
+      <c r="G3" s="52"/>
     </row>
     <row r="12" spans="1:19" ht="74" x14ac:dyDescent="1.95">
       <c r="I12" s="16"/>
@@ -2815,35 +2818,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" s="17" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="60" t="s">
         <v>68</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
-      <c r="I1" s="40"/>
-      <c r="J1" s="40"/>
-      <c r="K1" s="40"/>
-      <c r="L1" s="40"/>
-      <c r="M1" s="40"/>
-      <c r="N1" s="40"/>
-      <c r="O1" s="40"/>
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+      <c r="H1" s="60"/>
+      <c r="I1" s="60"/>
+      <c r="J1" s="60"/>
+      <c r="K1" s="60"/>
+      <c r="L1" s="60"/>
+      <c r="M1" s="60"/>
+      <c r="N1" s="60"/>
+      <c r="O1" s="60"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.5">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="53" t="s">
         <v>69</v>
       </c>
-      <c r="B2" s="41" t="s">
+      <c r="B2" s="53" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:15" ht="55.5" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A3" s="41"/>
-      <c r="B3" s="41"/>
+      <c r="A3" s="53"/>
+      <c r="B3" s="53"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2883,161 +2886,156 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" s="6" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="50" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
-      <c r="K1" s="35"/>
-      <c r="L1" s="35"/>
-      <c r="M1" s="35"/>
-      <c r="N1" s="35"/>
-      <c r="O1" s="35"/>
-      <c r="P1" s="35"/>
-      <c r="Q1" s="35"/>
-      <c r="R1" s="35"/>
-      <c r="S1" s="35"/>
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
+      <c r="D1" s="50"/>
+      <c r="E1" s="50"/>
+      <c r="F1" s="50"/>
+      <c r="G1" s="50"/>
+      <c r="H1" s="50"/>
+      <c r="I1" s="50"/>
+      <c r="J1" s="50"/>
+      <c r="K1" s="50"/>
+      <c r="L1" s="50"/>
+      <c r="M1" s="50"/>
+      <c r="N1" s="50"/>
+      <c r="O1" s="50"/>
+      <c r="P1" s="50"/>
+      <c r="Q1" s="50"/>
+      <c r="R1" s="50"/>
+      <c r="S1" s="50"/>
     </row>
     <row r="2" spans="1:28" s="13" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="52" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="42" t="s">
+      <c r="B2" s="52" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="42" t="s">
+      <c r="C2" s="52" t="s">
         <v>19</v>
       </c>
-      <c r="D2" s="42" t="s">
+      <c r="D2" s="52" t="s">
         <v>20</v>
       </c>
-      <c r="E2" s="42"/>
-      <c r="F2" s="42"/>
-      <c r="G2" s="42"/>
-      <c r="H2" s="42"/>
-      <c r="I2" s="49" t="s">
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52"/>
+      <c r="H2" s="52"/>
+      <c r="I2" s="51" t="s">
         <v>31</v>
       </c>
-      <c r="J2" s="49"/>
-      <c r="K2" s="49" t="s">
+      <c r="J2" s="51"/>
+      <c r="K2" s="51" t="s">
         <v>90</v>
       </c>
-      <c r="L2" s="42" t="s">
+      <c r="L2" s="52" t="s">
         <v>21</v>
       </c>
-      <c r="M2" s="49" t="s">
+      <c r="M2" s="51" t="s">
         <v>89</v>
       </c>
-      <c r="N2" s="49" t="s">
+      <c r="N2" s="51" t="s">
         <v>22</v>
       </c>
-      <c r="O2" s="49"/>
-      <c r="P2" s="49" t="s">
+      <c r="O2" s="51"/>
+      <c r="P2" s="51" t="s">
         <v>23</v>
       </c>
-      <c r="Q2" s="49" t="s">
+      <c r="Q2" s="51" t="s">
         <v>24</v>
       </c>
-      <c r="R2" s="49"/>
-      <c r="S2" s="49"/>
-      <c r="T2" s="49"/>
-      <c r="U2" s="49"/>
-      <c r="V2" s="49"/>
-      <c r="W2" s="49"/>
-      <c r="X2" s="42" t="s">
+      <c r="R2" s="51"/>
+      <c r="S2" s="51"/>
+      <c r="T2" s="51"/>
+      <c r="U2" s="51"/>
+      <c r="V2" s="51"/>
+      <c r="W2" s="51"/>
+      <c r="X2" s="52" t="s">
         <v>25</v>
       </c>
-      <c r="Y2" s="42"/>
-      <c r="Z2" s="42"/>
-      <c r="AA2" s="42"/>
-      <c r="AB2" s="42"/>
+      <c r="Y2" s="52"/>
+      <c r="Z2" s="52"/>
+      <c r="AA2" s="52"/>
+      <c r="AB2" s="52"/>
     </row>
     <row r="3" spans="1:28" ht="37.5" x14ac:dyDescent="0.5">
-      <c r="A3" s="42"/>
-      <c r="B3" s="42"/>
-      <c r="C3" s="42"/>
-      <c r="D3" s="50" t="s">
+      <c r="A3" s="52"/>
+      <c r="B3" s="52"/>
+      <c r="C3" s="52"/>
+      <c r="D3" s="40" t="s">
         <v>26</v>
       </c>
-      <c r="E3" s="50" t="s">
+      <c r="E3" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="F3" s="50" t="s">
+      <c r="F3" s="40" t="s">
         <v>28</v>
       </c>
-      <c r="G3" s="50" t="s">
+      <c r="G3" s="40" t="s">
         <v>29</v>
       </c>
-      <c r="H3" s="50" t="s">
+      <c r="H3" s="40" t="s">
         <v>30</v>
       </c>
-      <c r="I3" s="50" t="s">
+      <c r="I3" s="40" t="s">
         <v>31</v>
       </c>
-      <c r="J3" s="50" t="s">
+      <c r="J3" s="40" t="s">
         <v>73</v>
       </c>
-      <c r="K3" s="49"/>
-      <c r="L3" s="42"/>
-      <c r="M3" s="49"/>
-      <c r="N3" s="50" t="s">
+      <c r="K3" s="51"/>
+      <c r="L3" s="52"/>
+      <c r="M3" s="51"/>
+      <c r="N3" s="40" t="s">
         <v>74</v>
       </c>
-      <c r="O3" s="50" t="s">
+      <c r="O3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="P3" s="49"/>
-      <c r="Q3" s="50" t="s">
+      <c r="P3" s="51"/>
+      <c r="Q3" s="40" t="s">
         <v>72</v>
       </c>
-      <c r="R3" s="50" t="s">
+      <c r="R3" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="S3" s="50" t="s">
+      <c r="S3" s="40" t="s">
         <v>33</v>
       </c>
-      <c r="T3" s="50" t="s">
+      <c r="T3" s="40" t="s">
         <v>29</v>
       </c>
-      <c r="U3" s="50" t="s">
+      <c r="U3" s="40" t="s">
         <v>34</v>
       </c>
-      <c r="V3" s="50" t="s">
+      <c r="V3" s="40" t="s">
         <v>28</v>
       </c>
-      <c r="W3" s="50" t="s">
+      <c r="W3" s="40" t="s">
         <v>35</v>
       </c>
-      <c r="X3" s="50" t="s">
+      <c r="X3" s="40" t="s">
         <v>36</v>
       </c>
-      <c r="Y3" s="50" t="s">
+      <c r="Y3" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="Z3" s="50" t="s">
+      <c r="Z3" s="40" t="s">
         <v>38</v>
       </c>
-      <c r="AA3" s="50" t="s">
+      <c r="AA3" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="AB3" s="50" t="s">
+      <c r="AB3" s="40" t="s">
         <v>30</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="A1:S1"/>
-    <mergeCell ref="N2:O2"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="Q2:W2"/>
     <mergeCell ref="X2:AB2"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="B2:B3"/>
@@ -3046,6 +3044,11 @@
     <mergeCell ref="M2:M3"/>
     <mergeCell ref="P2:P3"/>
     <mergeCell ref="K2:K3"/>
+    <mergeCell ref="A1:S1"/>
+    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="Q2:W2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -3060,66 +3063,67 @@
   <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="15.7265625" defaultRowHeight="17.5" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="15.7265625" style="1"/>
-    <col min="2" max="6" width="15.7265625" style="2"/>
-    <col min="7" max="7" width="15.7265625" style="8"/>
+    <col min="1" max="1" width="15.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="5" width="15.36328125" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.26953125" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.6328125" style="8" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="78.81640625" style="8" bestFit="1" customWidth="1"/>
     <col min="9" max="16384" width="15.7265625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" s="17" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="60" t="s">
         <v>163</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
-      <c r="I1" s="40"/>
-      <c r="J1" s="40"/>
-      <c r="K1" s="40"/>
-      <c r="L1" s="40"/>
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+      <c r="H1" s="60"/>
+      <c r="I1" s="60"/>
+      <c r="J1" s="60"/>
+      <c r="K1" s="60"/>
+      <c r="L1" s="60"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.5">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="52" t="s">
         <v>162</v>
       </c>
-      <c r="B2" s="42"/>
-      <c r="C2" s="42"/>
-      <c r="D2" s="42"/>
-      <c r="E2" s="42"/>
-      <c r="F2" s="42"/>
-      <c r="G2" s="42"/>
-      <c r="H2" s="42" t="s">
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52"/>
+      <c r="H2" s="52" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="62.5" x14ac:dyDescent="0.5">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="40" t="s">
         <v>155</v>
       </c>
-      <c r="B3" s="50" t="s">
+      <c r="B3" s="40" t="s">
         <v>156</v>
       </c>
-      <c r="C3" s="50" t="s">
+      <c r="C3" s="40" t="s">
         <v>157</v>
       </c>
-      <c r="D3" s="50" t="s">
+      <c r="D3" s="40" t="s">
         <v>158</v>
       </c>
-      <c r="E3" s="50" t="s">
+      <c r="E3" s="40" t="s">
         <v>159</v>
       </c>
-      <c r="F3" s="50" t="s">
+      <c r="F3" s="40" t="s">
         <v>164</v>
       </c>
-      <c r="G3" s="50" t="s">
+      <c r="G3" s="40" t="s">
         <v>160</v>
       </c>
-      <c r="H3" s="42"/>
+      <c r="H3" s="52"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -3151,30 +3155,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" s="17" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="60" t="s">
         <v>144</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
-      <c r="I1" s="40"/>
-      <c r="J1" s="40"/>
-      <c r="K1" s="40"/>
-      <c r="L1" s="40"/>
-      <c r="M1" s="40"/>
-      <c r="N1" s="40"/>
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+      <c r="H1" s="60"/>
+      <c r="I1" s="60"/>
+      <c r="J1" s="60"/>
+      <c r="K1" s="60"/>
+      <c r="L1" s="60"/>
+      <c r="M1" s="60"/>
+      <c r="N1" s="60"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.5">
-      <c r="A2" s="38" t="s">
+      <c r="A2" s="61" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="3" spans="1:14" ht="55.5" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A3" s="39"/>
+      <c r="A3" s="62"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3205,174 +3209,174 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" s="6" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="50" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
-      <c r="K1" s="35"/>
-      <c r="L1" s="35"/>
-      <c r="M1" s="35"/>
-      <c r="N1" s="35"/>
-      <c r="O1" s="35"/>
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
+      <c r="D1" s="50"/>
+      <c r="E1" s="50"/>
+      <c r="F1" s="50"/>
+      <c r="G1" s="50"/>
+      <c r="H1" s="50"/>
+      <c r="I1" s="50"/>
+      <c r="J1" s="50"/>
+      <c r="K1" s="50"/>
+      <c r="L1" s="50"/>
+      <c r="M1" s="50"/>
+      <c r="N1" s="50"/>
+      <c r="O1" s="50"/>
     </row>
     <row r="2" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="53" t="s">
         <v>75</v>
       </c>
-      <c r="B2" s="42" t="s">
+      <c r="B2" s="52" t="s">
         <v>76</v>
       </c>
-      <c r="C2" s="42" t="s">
+      <c r="C2" s="52" t="s">
         <v>77</v>
       </c>
-      <c r="D2" s="42" t="s">
+      <c r="D2" s="52" t="s">
         <v>78</v>
       </c>
-      <c r="E2" s="42"/>
-      <c r="F2" s="42"/>
-      <c r="G2" s="42"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52"/>
     </row>
     <row r="3" spans="1:15" ht="41.25" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A3" s="41"/>
-      <c r="B3" s="42"/>
-      <c r="C3" s="42"/>
-      <c r="D3" s="42"/>
-      <c r="E3" s="42"/>
-      <c r="F3" s="42"/>
-      <c r="G3" s="42"/>
+      <c r="A3" s="53"/>
+      <c r="B3" s="52"/>
+      <c r="C3" s="52"/>
+      <c r="D3" s="52"/>
+      <c r="E3" s="52"/>
+      <c r="F3" s="52"/>
+      <c r="G3" s="52"/>
     </row>
     <row r="4" spans="1:15" ht="48" x14ac:dyDescent="0.5">
-      <c r="A4" s="43"/>
-      <c r="B4" s="43"/>
-      <c r="C4" s="44"/>
-      <c r="D4" s="44"/>
-      <c r="E4" s="45" t="s">
+      <c r="A4" s="34"/>
+      <c r="B4" s="34"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="F4" s="45" t="s">
+      <c r="F4" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="G4" s="45" t="s">
+      <c r="G4" s="36" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.5">
-      <c r="A5" s="43"/>
-      <c r="B5" s="43"/>
-      <c r="C5" s="44"/>
-      <c r="D5" s="46" t="s">
+      <c r="A5" s="34"/>
+      <c r="B5" s="34"/>
+      <c r="C5" s="35"/>
+      <c r="D5" s="37" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="43"/>
-      <c r="F5" s="43"/>
-      <c r="G5" s="43"/>
+      <c r="E5" s="34"/>
+      <c r="F5" s="34"/>
+      <c r="G5" s="34"/>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.5">
-      <c r="A6" s="43"/>
-      <c r="B6" s="43"/>
-      <c r="C6" s="44"/>
-      <c r="D6" s="46" t="s">
+      <c r="A6" s="34"/>
+      <c r="B6" s="34"/>
+      <c r="C6" s="35"/>
+      <c r="D6" s="37" t="s">
         <v>5</v>
       </c>
-      <c r="E6" s="43"/>
-      <c r="F6" s="43"/>
-      <c r="G6" s="43"/>
+      <c r="E6" s="34"/>
+      <c r="F6" s="34"/>
+      <c r="G6" s="34"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.5">
-      <c r="A7" s="43"/>
-      <c r="B7" s="43"/>
-      <c r="C7" s="44"/>
-      <c r="D7" s="46" t="s">
+      <c r="A7" s="34"/>
+      <c r="B7" s="34"/>
+      <c r="C7" s="35"/>
+      <c r="D7" s="37" t="s">
         <v>6</v>
       </c>
-      <c r="E7" s="43"/>
-      <c r="F7" s="43"/>
-      <c r="G7" s="43"/>
+      <c r="E7" s="34"/>
+      <c r="F7" s="34"/>
+      <c r="G7" s="34"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.5">
-      <c r="A8" s="43"/>
-      <c r="B8" s="43"/>
-      <c r="C8" s="44"/>
-      <c r="D8" s="46" t="s">
+      <c r="A8" s="34"/>
+      <c r="B8" s="34"/>
+      <c r="C8" s="35"/>
+      <c r="D8" s="37" t="s">
         <v>7</v>
       </c>
-      <c r="E8" s="43"/>
-      <c r="F8" s="43"/>
-      <c r="G8" s="43"/>
+      <c r="E8" s="34"/>
+      <c r="F8" s="34"/>
+      <c r="G8" s="34"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.5">
-      <c r="A9" s="43"/>
-      <c r="B9" s="43"/>
-      <c r="C9" s="44"/>
-      <c r="D9" s="46" t="s">
+      <c r="A9" s="34"/>
+      <c r="B9" s="34"/>
+      <c r="C9" s="35"/>
+      <c r="D9" s="37" t="s">
         <v>8</v>
       </c>
-      <c r="E9" s="43"/>
-      <c r="F9" s="43"/>
-      <c r="G9" s="43"/>
+      <c r="E9" s="34"/>
+      <c r="F9" s="34"/>
+      <c r="G9" s="34"/>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.5">
-      <c r="A10" s="43"/>
-      <c r="B10" s="43"/>
-      <c r="C10" s="44"/>
-      <c r="D10" s="47" t="s">
+      <c r="A10" s="34"/>
+      <c r="B10" s="34"/>
+      <c r="C10" s="35"/>
+      <c r="D10" s="38" t="s">
         <v>9</v>
       </c>
-      <c r="E10" s="43"/>
-      <c r="F10" s="43"/>
-      <c r="G10" s="43"/>
+      <c r="E10" s="34"/>
+      <c r="F10" s="34"/>
+      <c r="G10" s="34"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.5">
-      <c r="A11" s="43"/>
-      <c r="B11" s="43"/>
-      <c r="C11" s="44"/>
-      <c r="D11" s="47" t="s">
+      <c r="A11" s="34"/>
+      <c r="B11" s="34"/>
+      <c r="C11" s="35"/>
+      <c r="D11" s="38" t="s">
         <v>10</v>
       </c>
-      <c r="E11" s="43"/>
-      <c r="F11" s="43"/>
-      <c r="G11" s="43"/>
+      <c r="E11" s="34"/>
+      <c r="F11" s="34"/>
+      <c r="G11" s="34"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.5">
-      <c r="A12" s="43"/>
-      <c r="B12" s="43"/>
-      <c r="C12" s="44"/>
-      <c r="D12" s="47" t="s">
+      <c r="A12" s="34"/>
+      <c r="B12" s="34"/>
+      <c r="C12" s="35"/>
+      <c r="D12" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="E12" s="43"/>
-      <c r="F12" s="43"/>
-      <c r="G12" s="43"/>
+      <c r="E12" s="34"/>
+      <c r="F12" s="34"/>
+      <c r="G12" s="34"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.5">
-      <c r="A13" s="43"/>
-      <c r="B13" s="43"/>
-      <c r="C13" s="44"/>
-      <c r="D13" s="47" t="s">
+      <c r="A13" s="34"/>
+      <c r="B13" s="34"/>
+      <c r="C13" s="35"/>
+      <c r="D13" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="E13" s="43"/>
-      <c r="F13" s="43"/>
-      <c r="G13" s="43"/>
+      <c r="E13" s="34"/>
+      <c r="F13" s="34"/>
+      <c r="G13" s="34"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.5">
-      <c r="A14" s="43"/>
-      <c r="B14" s="43"/>
-      <c r="C14" s="44"/>
-      <c r="D14" s="48" t="s">
+      <c r="A14" s="34"/>
+      <c r="B14" s="34"/>
+      <c r="C14" s="35"/>
+      <c r="D14" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="E14" s="43"/>
-      <c r="F14" s="43"/>
-      <c r="G14" s="43"/>
+      <c r="E14" s="34"/>
+      <c r="F14" s="34"/>
+      <c r="G14" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -3407,41 +3411,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" s="6" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="50" t="s">
         <v>143</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
-      <c r="K1" s="35"/>
-      <c r="L1" s="35"/>
-      <c r="M1" s="35"/>
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
+      <c r="D1" s="50"/>
+      <c r="E1" s="50"/>
+      <c r="F1" s="50"/>
+      <c r="G1" s="50"/>
+      <c r="H1" s="50"/>
+      <c r="I1" s="50"/>
+      <c r="J1" s="50"/>
+      <c r="K1" s="50"/>
+      <c r="L1" s="50"/>
+      <c r="M1" s="50"/>
     </row>
     <row r="2" spans="1:13" s="13" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="52" t="s">
         <v>139</v>
       </c>
-      <c r="B2" s="42" t="s">
+      <c r="B2" s="52" t="s">
         <v>140</v>
       </c>
-      <c r="C2" s="42" t="s">
+      <c r="C2" s="52" t="s">
         <v>141</v>
       </c>
-      <c r="D2" s="42" t="s">
+      <c r="D2" s="52" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.5">
-      <c r="A3" s="42"/>
-      <c r="B3" s="42"/>
-      <c r="C3" s="42"/>
-      <c r="D3" s="42"/>
+      <c r="A3" s="52"/>
+      <c r="B3" s="52"/>
+      <c r="C3" s="52"/>
+      <c r="D3" s="52"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -3472,127 +3476,127 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" s="6" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="35" t="s">
-        <v>228</v>
-      </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
-      <c r="K1" s="35"/>
-      <c r="L1" s="35"/>
-      <c r="M1" s="35"/>
+      <c r="A1" s="50" t="s">
+        <v>226</v>
+      </c>
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
+      <c r="D1" s="50"/>
+      <c r="E1" s="50"/>
+      <c r="F1" s="50"/>
+      <c r="G1" s="50"/>
+      <c r="H1" s="50"/>
+      <c r="I1" s="50"/>
+      <c r="J1" s="50"/>
+      <c r="K1" s="50"/>
+      <c r="L1" s="50"/>
+      <c r="M1" s="50"/>
     </row>
     <row r="2" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A2" s="42" t="s">
-        <v>227</v>
-      </c>
-      <c r="B2" s="42"/>
-      <c r="C2" s="42"/>
-      <c r="D2" s="42"/>
+      <c r="A2" s="52" t="s">
+        <v>225</v>
+      </c>
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
     </row>
     <row r="3" spans="1:13" ht="41.25" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A3" s="42"/>
-      <c r="B3" s="42"/>
-      <c r="C3" s="42"/>
-      <c r="D3" s="42"/>
+      <c r="A3" s="52"/>
+      <c r="B3" s="52"/>
+      <c r="C3" s="52"/>
+      <c r="D3" s="52"/>
     </row>
     <row r="4" spans="1:13" ht="80" x14ac:dyDescent="0.5">
-      <c r="A4" s="44"/>
-      <c r="B4" s="45" t="s">
+      <c r="A4" s="35"/>
+      <c r="B4" s="36" t="s">
+        <v>222</v>
+      </c>
+      <c r="C4" s="36" t="s">
+        <v>223</v>
+      </c>
+      <c r="D4" s="36" t="s">
         <v>224</v>
       </c>
-      <c r="C4" s="45" t="s">
-        <v>225</v>
-      </c>
-      <c r="D4" s="45" t="s">
-        <v>226</v>
-      </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.5">
-      <c r="A5" s="46" t="s">
+      <c r="A5" s="37" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="43"/>
-      <c r="C5" s="43"/>
-      <c r="D5" s="43"/>
+      <c r="B5" s="34"/>
+      <c r="C5" s="34"/>
+      <c r="D5" s="34"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.5">
-      <c r="A6" s="46" t="s">
+      <c r="A6" s="37" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="43"/>
-      <c r="C6" s="43"/>
-      <c r="D6" s="43"/>
+      <c r="B6" s="34"/>
+      <c r="C6" s="34"/>
+      <c r="D6" s="34"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.5">
-      <c r="A7" s="46" t="s">
+      <c r="A7" s="37" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="43"/>
-      <c r="C7" s="43"/>
-      <c r="D7" s="43"/>
+      <c r="B7" s="34"/>
+      <c r="C7" s="34"/>
+      <c r="D7" s="34"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.5">
-      <c r="A8" s="46" t="s">
+      <c r="A8" s="37" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="43"/>
-      <c r="C8" s="43"/>
-      <c r="D8" s="43"/>
+      <c r="B8" s="34"/>
+      <c r="C8" s="34"/>
+      <c r="D8" s="34"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.5">
-      <c r="A9" s="46" t="s">
+      <c r="A9" s="37" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="43"/>
-      <c r="C9" s="43"/>
-      <c r="D9" s="43"/>
+      <c r="B9" s="34"/>
+      <c r="C9" s="34"/>
+      <c r="D9" s="34"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.5">
-      <c r="A10" s="47" t="s">
+      <c r="A10" s="38" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="43"/>
-      <c r="C10" s="43"/>
-      <c r="D10" s="43"/>
+      <c r="B10" s="34"/>
+      <c r="C10" s="34"/>
+      <c r="D10" s="34"/>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.5">
-      <c r="A11" s="47" t="s">
+      <c r="A11" s="38" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="43"/>
-      <c r="C11" s="43"/>
-      <c r="D11" s="43"/>
+      <c r="B11" s="34"/>
+      <c r="C11" s="34"/>
+      <c r="D11" s="34"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.5">
-      <c r="A12" s="47" t="s">
+      <c r="A12" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="43"/>
-      <c r="C12" s="43"/>
-      <c r="D12" s="43"/>
+      <c r="B12" s="34"/>
+      <c r="C12" s="34"/>
+      <c r="D12" s="34"/>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.5">
-      <c r="A13" s="47" t="s">
+      <c r="A13" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="43"/>
-      <c r="C13" s="43"/>
-      <c r="D13" s="43"/>
+      <c r="B13" s="34"/>
+      <c r="C13" s="34"/>
+      <c r="D13" s="34"/>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.5">
-      <c r="A14" s="48" t="s">
+      <c r="A14" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="43"/>
-      <c r="C14" s="43"/>
-      <c r="D14" s="43"/>
+      <c r="B14" s="34"/>
+      <c r="C14" s="34"/>
+      <c r="D14" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3631,21 +3635,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" s="14" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="56" t="s">
         <v>119</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
-      <c r="J1" s="36"/>
-      <c r="K1" s="36"/>
-      <c r="L1" s="36"/>
-      <c r="M1" s="36"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
+      <c r="K1" s="56"/>
+      <c r="L1" s="56"/>
+      <c r="M1" s="56"/>
       <c r="R1" s="24"/>
       <c r="S1" s="24"/>
       <c r="T1" s="24"/>
@@ -3669,188 +3673,188 @@
       <c r="AL1" s="24"/>
     </row>
     <row r="2" spans="1:38" ht="35.25" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="52" t="s">
         <v>123</v>
       </c>
-      <c r="B2" s="42"/>
-      <c r="C2" s="42"/>
-      <c r="D2" s="51" t="s">
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="55" t="s">
         <v>136</v>
       </c>
-      <c r="E2" s="51"/>
-      <c r="F2" s="51"/>
-      <c r="G2" s="51"/>
-      <c r="H2" s="51"/>
-      <c r="I2" s="51"/>
-      <c r="J2" s="51"/>
-      <c r="K2" s="51"/>
-      <c r="L2" s="51"/>
-      <c r="M2" s="51"/>
-      <c r="N2" s="51"/>
-      <c r="O2" s="51"/>
-      <c r="P2" s="51"/>
-      <c r="Q2" s="51"/>
-      <c r="R2" s="42" t="s">
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
+      <c r="H2" s="55"/>
+      <c r="I2" s="55"/>
+      <c r="J2" s="55"/>
+      <c r="K2" s="55"/>
+      <c r="L2" s="55"/>
+      <c r="M2" s="55"/>
+      <c r="N2" s="55"/>
+      <c r="O2" s="55"/>
+      <c r="P2" s="55"/>
+      <c r="Q2" s="55"/>
+      <c r="R2" s="52" t="s">
+        <v>190</v>
+      </c>
+      <c r="S2" s="52"/>
+      <c r="T2" s="52"/>
+      <c r="U2" s="52"/>
+      <c r="V2" s="52" t="s">
+        <v>191</v>
+      </c>
+      <c r="W2" s="52"/>
+      <c r="X2" s="52"/>
+      <c r="Y2" s="52"/>
+      <c r="Z2" s="52"/>
+      <c r="AA2" s="52"/>
+      <c r="AB2" s="52"/>
+      <c r="AC2" s="52"/>
+      <c r="AD2" s="52"/>
+      <c r="AE2" s="52"/>
+      <c r="AF2" s="52"/>
+      <c r="AG2" s="52"/>
+      <c r="AH2" s="52"/>
+      <c r="AI2" s="52"/>
+      <c r="AJ2" s="52"/>
+      <c r="AK2" s="52"/>
+      <c r="AL2" s="52"/>
+    </row>
+    <row r="3" spans="1:38" ht="50" x14ac:dyDescent="0.5">
+      <c r="A3" s="40" t="s">
+        <v>120</v>
+      </c>
+      <c r="B3" s="40" t="s">
+        <v>121</v>
+      </c>
+      <c r="C3" s="40" t="s">
+        <v>122</v>
+      </c>
+      <c r="D3" s="54" t="s">
+        <v>127</v>
+      </c>
+      <c r="E3" s="54"/>
+      <c r="F3" s="54"/>
+      <c r="G3" s="54"/>
+      <c r="H3" s="54"/>
+      <c r="I3" s="54"/>
+      <c r="J3" s="54"/>
+      <c r="K3" s="54"/>
+      <c r="L3" s="54" t="s">
+        <v>128</v>
+      </c>
+      <c r="M3" s="54"/>
+      <c r="N3" s="54"/>
+      <c r="O3" s="54" t="s">
+        <v>129</v>
+      </c>
+      <c r="P3" s="54"/>
+      <c r="Q3" s="54"/>
+      <c r="R3" s="40" t="s">
+        <v>124</v>
+      </c>
+      <c r="S3" s="40" t="s">
+        <v>125</v>
+      </c>
+      <c r="T3" s="40" t="s">
+        <v>122</v>
+      </c>
+      <c r="U3" s="40" t="s">
+        <v>126</v>
+      </c>
+      <c r="V3" s="40" t="s">
         <v>192</v>
       </c>
-      <c r="S2" s="42"/>
-      <c r="T2" s="42"/>
-      <c r="U2" s="42"/>
-      <c r="V2" s="42" t="s">
+      <c r="W3" s="40" t="s">
         <v>193</v>
       </c>
-      <c r="W2" s="42"/>
-      <c r="X2" s="42"/>
-      <c r="Y2" s="42"/>
-      <c r="Z2" s="42"/>
-      <c r="AA2" s="42"/>
-      <c r="AB2" s="42"/>
-      <c r="AC2" s="42"/>
-      <c r="AD2" s="42"/>
-      <c r="AE2" s="42"/>
-      <c r="AF2" s="42"/>
-      <c r="AG2" s="42"/>
-      <c r="AH2" s="42"/>
-      <c r="AI2" s="42"/>
-      <c r="AJ2" s="42"/>
-      <c r="AK2" s="42"/>
-      <c r="AL2" s="42"/>
-    </row>
-    <row r="3" spans="1:38" ht="50" x14ac:dyDescent="0.5">
-      <c r="A3" s="50" t="s">
+      <c r="X3" s="40" t="s">
+        <v>194</v>
+      </c>
+      <c r="Y3" s="40" t="s">
+        <v>195</v>
+      </c>
+      <c r="Z3" s="40" t="s">
+        <v>196</v>
+      </c>
+      <c r="AA3" s="40" t="s">
+        <v>197</v>
+      </c>
+      <c r="AB3" s="40" t="s">
+        <v>198</v>
+      </c>
+      <c r="AC3" s="40" t="s">
+        <v>199</v>
+      </c>
+      <c r="AD3" s="40" t="s">
+        <v>200</v>
+      </c>
+      <c r="AE3" s="40" t="s">
+        <v>201</v>
+      </c>
+      <c r="AF3" s="40" t="s">
+        <v>202</v>
+      </c>
+      <c r="AG3" s="40" t="s">
+        <v>203</v>
+      </c>
+      <c r="AH3" s="40" t="s">
+        <v>204</v>
+      </c>
+      <c r="AI3" s="40" t="s">
+        <v>205</v>
+      </c>
+      <c r="AJ3" s="40" t="s">
+        <v>206</v>
+      </c>
+      <c r="AK3" s="40" t="s">
+        <v>207</v>
+      </c>
+      <c r="AL3" s="40" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="4" spans="1:38" ht="25" x14ac:dyDescent="0.5">
+      <c r="D4" s="40" t="s">
+        <v>130</v>
+      </c>
+      <c r="E4" s="40" t="s">
+        <v>131</v>
+      </c>
+      <c r="F4" s="40" t="s">
+        <v>132</v>
+      </c>
+      <c r="G4" s="40" t="s">
+        <v>137</v>
+      </c>
+      <c r="H4" s="40" t="s">
+        <v>138</v>
+      </c>
+      <c r="I4" s="40" t="s">
+        <v>133</v>
+      </c>
+      <c r="J4" s="40" t="s">
+        <v>42</v>
+      </c>
+      <c r="K4" s="40" t="s">
+        <v>134</v>
+      </c>
+      <c r="L4" s="40" t="s">
+        <v>130</v>
+      </c>
+      <c r="M4" s="40" t="s">
+        <v>132</v>
+      </c>
+      <c r="N4" s="40" t="s">
+        <v>135</v>
+      </c>
+      <c r="O4" s="40" t="s">
         <v>120</v>
       </c>
-      <c r="B3" s="50" t="s">
+      <c r="P4" s="40" t="s">
         <v>121</v>
       </c>
-      <c r="C3" s="50" t="s">
-        <v>122</v>
-      </c>
-      <c r="D3" s="52" t="s">
-        <v>127</v>
-      </c>
-      <c r="E3" s="52"/>
-      <c r="F3" s="52"/>
-      <c r="G3" s="52"/>
-      <c r="H3" s="52"/>
-      <c r="I3" s="52"/>
-      <c r="J3" s="52"/>
-      <c r="K3" s="52"/>
-      <c r="L3" s="52" t="s">
-        <v>128</v>
-      </c>
-      <c r="M3" s="52"/>
-      <c r="N3" s="52"/>
-      <c r="O3" s="52" t="s">
-        <v>129</v>
-      </c>
-      <c r="P3" s="52"/>
-      <c r="Q3" s="52"/>
-      <c r="R3" s="50" t="s">
-        <v>124</v>
-      </c>
-      <c r="S3" s="50" t="s">
-        <v>125</v>
-      </c>
-      <c r="T3" s="50" t="s">
-        <v>122</v>
-      </c>
-      <c r="U3" s="50" t="s">
-        <v>126</v>
-      </c>
-      <c r="V3" s="50" t="s">
-        <v>194</v>
-      </c>
-      <c r="W3" s="50" t="s">
-        <v>195</v>
-      </c>
-      <c r="X3" s="50" t="s">
-        <v>196</v>
-      </c>
-      <c r="Y3" s="50" t="s">
-        <v>197</v>
-      </c>
-      <c r="Z3" s="50" t="s">
-        <v>198</v>
-      </c>
-      <c r="AA3" s="50" t="s">
-        <v>199</v>
-      </c>
-      <c r="AB3" s="50" t="s">
-        <v>200</v>
-      </c>
-      <c r="AC3" s="50" t="s">
-        <v>201</v>
-      </c>
-      <c r="AD3" s="50" t="s">
-        <v>202</v>
-      </c>
-      <c r="AE3" s="50" t="s">
-        <v>203</v>
-      </c>
-      <c r="AF3" s="50" t="s">
-        <v>204</v>
-      </c>
-      <c r="AG3" s="50" t="s">
-        <v>205</v>
-      </c>
-      <c r="AH3" s="50" t="s">
-        <v>206</v>
-      </c>
-      <c r="AI3" s="50" t="s">
-        <v>207</v>
-      </c>
-      <c r="AJ3" s="50" t="s">
-        <v>208</v>
-      </c>
-      <c r="AK3" s="50" t="s">
-        <v>209</v>
-      </c>
-      <c r="AL3" s="50" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="4" spans="1:38" ht="25" x14ac:dyDescent="0.5">
-      <c r="D4" s="50" t="s">
-        <v>130</v>
-      </c>
-      <c r="E4" s="50" t="s">
-        <v>131</v>
-      </c>
-      <c r="F4" s="50" t="s">
-        <v>132</v>
-      </c>
-      <c r="G4" s="50" t="s">
-        <v>137</v>
-      </c>
-      <c r="H4" s="50" t="s">
-        <v>138</v>
-      </c>
-      <c r="I4" s="50" t="s">
-        <v>133</v>
-      </c>
-      <c r="J4" s="50" t="s">
-        <v>42</v>
-      </c>
-      <c r="K4" s="50" t="s">
-        <v>134</v>
-      </c>
-      <c r="L4" s="50" t="s">
-        <v>130</v>
-      </c>
-      <c r="M4" s="50" t="s">
-        <v>132</v>
-      </c>
-      <c r="N4" s="50" t="s">
-        <v>135</v>
-      </c>
-      <c r="O4" s="50" t="s">
-        <v>120</v>
-      </c>
-      <c r="P4" s="50" t="s">
-        <v>121</v>
-      </c>
-      <c r="Q4" s="50" t="s">
+      <c r="Q4" s="40" t="s">
         <v>122</v>
       </c>
     </row>
@@ -3889,67 +3893,67 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" s="14" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="56" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
-      <c r="J1" s="36"/>
-      <c r="K1" s="36"/>
-      <c r="L1" s="36"/>
-      <c r="M1" s="36"/>
-      <c r="N1" s="36"/>
-      <c r="O1" s="36"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
+      <c r="K1" s="56"/>
+      <c r="L1" s="56"/>
+      <c r="M1" s="56"/>
+      <c r="N1" s="56"/>
+      <c r="O1" s="56"/>
     </row>
     <row r="2" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="52" t="s">
         <v>44</v>
       </c>
-      <c r="B2" s="42"/>
-      <c r="C2" s="42"/>
-      <c r="D2" s="42" t="s">
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52" t="s">
         <v>45</v>
       </c>
-      <c r="E2" s="42"/>
-      <c r="F2" s="42"/>
-      <c r="G2" s="42" t="s">
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52" t="s">
         <v>46</v>
       </c>
-      <c r="H2" s="42"/>
-      <c r="I2" s="42"/>
+      <c r="H2" s="52"/>
+      <c r="I2" s="52"/>
     </row>
     <row r="3" spans="1:15" ht="25" x14ac:dyDescent="0.5">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="B3" s="50" t="s">
+      <c r="B3" s="40" t="s">
         <v>42</v>
       </c>
-      <c r="C3" s="50" t="s">
+      <c r="C3" s="40" t="s">
         <v>43</v>
       </c>
-      <c r="D3" s="50" t="s">
+      <c r="D3" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="E3" s="50" t="s">
+      <c r="E3" s="40" t="s">
         <v>42</v>
       </c>
-      <c r="F3" s="50" t="s">
+      <c r="F3" s="40" t="s">
         <v>43</v>
       </c>
-      <c r="G3" s="50" t="s">
+      <c r="G3" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="H3" s="50" t="s">
+      <c r="H3" s="40" t="s">
         <v>42</v>
       </c>
-      <c r="I3" s="50" t="s">
+      <c r="I3" s="40" t="s">
         <v>43</v>
       </c>
     </row>
@@ -3982,71 +3986,71 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" s="14" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="56" t="s">
         <v>108</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
-      <c r="J1" s="36"/>
-      <c r="K1" s="36"/>
-      <c r="L1" s="36"/>
-      <c r="M1" s="36"/>
-      <c r="N1" s="36"/>
-      <c r="O1" s="36"/>
-      <c r="P1" s="36"/>
-      <c r="Q1" s="36"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
+      <c r="K1" s="56"/>
+      <c r="L1" s="56"/>
+      <c r="M1" s="56"/>
+      <c r="N1" s="56"/>
+      <c r="O1" s="56"/>
+      <c r="P1" s="56"/>
+      <c r="Q1" s="56"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.5">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="52" t="s">
         <v>109</v>
       </c>
-      <c r="B2" s="42"/>
-      <c r="C2" s="42"/>
-      <c r="D2" s="42"/>
-      <c r="E2" s="42"/>
-      <c r="F2" s="42" t="s">
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52" t="s">
         <v>110</v>
       </c>
-      <c r="G2" s="42"/>
-      <c r="H2" s="42"/>
-      <c r="I2" s="42"/>
-      <c r="J2" s="42"/>
+      <c r="G2" s="52"/>
+      <c r="H2" s="52"/>
+      <c r="I2" s="52"/>
+      <c r="J2" s="52"/>
     </row>
     <row r="3" spans="1:17" ht="37.5" x14ac:dyDescent="0.5">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="40" t="s">
         <v>42</v>
       </c>
-      <c r="B3" s="50" t="s">
+      <c r="B3" s="40" t="s">
         <v>115</v>
       </c>
-      <c r="C3" s="50" t="s">
+      <c r="C3" s="40" t="s">
         <v>116</v>
       </c>
-      <c r="D3" s="50" t="s">
+      <c r="D3" s="40" t="s">
         <v>117</v>
       </c>
-      <c r="E3" s="50" t="s">
+      <c r="E3" s="40" t="s">
         <v>118</v>
       </c>
-      <c r="F3" s="50" t="s">
+      <c r="F3" s="40" t="s">
         <v>42</v>
       </c>
-      <c r="G3" s="50" t="s">
+      <c r="G3" s="40" t="s">
         <v>111</v>
       </c>
-      <c r="H3" s="50" t="s">
+      <c r="H3" s="40" t="s">
         <v>112</v>
       </c>
-      <c r="I3" s="50" t="s">
+      <c r="I3" s="40" t="s">
         <v>113</v>
       </c>
-      <c r="J3" s="50" t="s">
+      <c r="J3" s="40" t="s">
         <v>114</v>
       </c>
     </row>
@@ -4084,41 +4088,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" s="14" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="56" t="s">
         <v>52</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
-      <c r="J1" s="36"/>
-      <c r="K1" s="36"/>
-      <c r="L1" s="36"/>
-      <c r="M1" s="36"/>
-      <c r="N1" s="36"/>
-      <c r="O1" s="36"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
+      <c r="K1" s="56"/>
+      <c r="L1" s="56"/>
+      <c r="M1" s="56"/>
+      <c r="N1" s="56"/>
+      <c r="O1" s="56"/>
     </row>
     <row r="2" spans="1:15" ht="36" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="52" t="s">
         <v>47</v>
       </c>
-      <c r="B2" s="42"/>
-      <c r="C2" s="42" t="s">
+      <c r="B2" s="52"/>
+      <c r="C2" s="52" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:15" ht="75" x14ac:dyDescent="0.5">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="B3" s="50" t="s">
+      <c r="B3" s="40" t="s">
         <v>49</v>
       </c>
-      <c r="C3" s="42"/>
+      <c r="C3" s="52"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>